<commit_message>
Bot tu dong cap nhat ngay 2026-06-03
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,111 +425,111 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>product_link</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>brand_name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>price_old</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>price_new</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>price_change</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>price_change_percent</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>sold_count_old</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sold_count_new</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sold_count_increase</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>revenue_increase</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>rating_old</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>rating_new</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rating_change</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>review_count_old</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>review_count_new</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>review_count_increase</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>date_compared</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -525,73 +537,73 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>279287522</v>
+        <v>274937386</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bộ áo điều hòa KITO NEWPRO KT10 thế hệ mới nhất 2026 quạt 24V siêu bên ,chống chai ,chống phồng</t>
+          <t>Bộ bơi nữ big size cao cấp, mẫu 2 mảnh áo cộc tay có khóa kéo trước, quần boxer trẻ trung, chất thun bơi lạnh Lycra co giãn đa chiều, dày dặn mịn mát, chống thấm nước nhanh khô | KT110</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-ao-dieu-hoa-kito-newpro-kt10-the-he-moi-nhat-2026-quat-24v-sieu-ben-chong-chai-chong-phong-p279287522-p279287522.html</t>
+          <t>https://tiki.vn/bo-boi-nu-big-size-cao-cap-mau-2-manh-ao-coc-tay-co-khoa-keo-truoc-quan-boxer-tre-trung-chat-thun-boi-lanh-lycra-co-gian-da-chieu-day-dan-min-mat-chong-tham-nuoc-nhanh-kho-kt110-p274937386-p274937386.html</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Kito</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>963000</v>
+        <v>480000</v>
       </c>
       <c r="G2" t="n">
-        <v>1070000</v>
+        <v>480000</v>
       </c>
       <c r="H2" t="n">
-        <v>107000</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>11.11</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>1440000</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -602,21 +614,21 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>278498646</v>
+        <v>104791604</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Quần short Nam tập Gym thể thao, mặc nhà, đi chơi - T0588</t>
+          <t>Quần lót nữ thái lan 828 – Chất thun lạnh - giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-short-nam-tap-gym-the-thao-mac-nha-di-choi-t0588-p278498646-p278498646.html</t>
+          <t>https://tiki.vn/quan-lot-nu-thai-lan-828-chat-thun-lanh-giao-mau-ngau-nhien-p104791604-p104791604.html</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -625,53 +637,130 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>110000</v>
+        <v>44000</v>
       </c>
       <c r="G3" t="n">
-        <v>110000</v>
+        <v>36080</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-7920</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>-18</v>
       </c>
       <c r="J3" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="L3" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-11000000</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>244298960</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Quần Mặc Váy Su Thông Hơi Trơn 6530 | Mát Mẻ, Không Lộ, Chống Hớ Hiệu Quả</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/quan-vay-dai-thong-hoi-6530-p244298960-p244298960.html</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Thời trang nam</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>42000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>34860</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-7140</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-17</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>UPDATED</t>
         </is>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-06-20
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,17 +543,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8407712</t>
+          <t>26666649</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Giày Sandal Nam BIGGBEN Da Bò Thật SD68</t>
+          <t>Dép Nam BIGGBEN Da Bò Thật Cao Cấp DN196</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-sandal-nam-biggben-da-bo-that-sd68-p8407712.html?spid=8407714</t>
+          <t>https://tiki.vn/dep-nam-biggben-da-bo-that-cao-cap-dn196-p26666649.html?spid=26666651</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -570,10 +570,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>419000</v>
+        <v>379000</v>
       </c>
       <c r="H2" t="n">
-        <v>419000</v>
+        <v>379000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,35 +582,35 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="L2" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M2" t="n">
-        <v>43995000</v>
+        <v>41690000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="P2" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="S2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -627,37 +627,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>38160273</t>
+          <t>66803444</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Giày Boot Nam BIGGBEN Da Bò Thật Cao Cấp BT2</t>
+          <t>Áo Cardigan Nữ Họa Tiết Xinh Thời Trang Korea ALN037 MayHomes Mẫu Mới Mùa Xuân</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-boot-nam-biggben-da-bo-that-cao-cap-bt2-p38160273.html?spid=38160275</t>
+          <t>https://tiki.vn/ao-cardigan-nu-hoa-tiet-xinh-thoi-trang-korea-aln037-mayhomes-mau-moi-mua-xuan-p66803444.html?spid=66803452</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>MAYHOMES</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>2000000</v>
+        <v>149000</v>
       </c>
       <c r="H3" t="n">
-        <v>2000000</v>
+        <v>149000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,35 +666,35 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>10</v>
+        <v>172</v>
       </c>
       <c r="L3" t="n">
-        <v>10</v>
+        <v>172</v>
       </c>
       <c r="M3" t="n">
-        <v>20000000</v>
+        <v>25628000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="P3" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,37 +711,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>183685137</t>
+          <t>273388482</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thắt Lưng Dây Nịt Nam Vải Dù US ARMY, Phong Cách Sang Trọng Cổ Điển Mặt Khóa Hợp Kim Thép Chống Ghỉ Cao Cấp -HÀNG CHÍNH HÃNG</t>
+          <t>Combo 7 quần lót cotton nữ nhiều màu du lịch dùng 1 lần</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-day-nit-nam-vai-du-us-army-phong-cach-sang-trong-co-dien-mat-khoa-hop-kim-thep-chong-ghi-cao-cap-hang-chinh-hang-p183685137.html?spid=183685139</t>
+          <t>https://tiki.vn/combo-7-quan-lot-cotton-nu-nhieu-mau-du-lich-dung-1-lan-p273388482.html?spid=273388612</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>US ARMY</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>79000</v>
+        <v>169000</v>
       </c>
       <c r="H4" t="n">
-        <v>79000</v>
+        <v>169000</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -750,35 +750,35 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>209</v>
+        <v>33</v>
       </c>
       <c r="L4" t="n">
-        <v>209</v>
+        <v>33</v>
       </c>
       <c r="M4" t="n">
-        <v>16511000</v>
+        <v>5577000</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="P4" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="S4" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -795,538 +795,538 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20535045</t>
+          <t>190792898</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Thắt lưng nam da bò AT Leather - P142</t>
+          <t>Giày sandal nam da bò thật BIGGBEN cao cấp SD123</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-nam-da-bo-at-leather-p142-p20535045.html?spid=20535047</t>
+          <t>https://tiki.vn/giay-sandal-nam-da-bo-that-biggben-cao-cap-sd123-p190792898.html?spid=190792908</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ANH THO LEATHER</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>295000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>295000</v>
+        <v>399000</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>399000</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>173</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>181</v>
+        <v>12</v>
       </c>
       <c r="L5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M5" t="n">
-        <v>2360000</v>
+        <v>4788000</v>
       </c>
       <c r="N5" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Bán thêm +8 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>52189164</t>
+          <t>275431635</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Combo 3 quần lót nam sợi cotton Organic mềm mịn thoáng mát co giãn 4 chiều MRM Manlywear (TẶNG Đôi Tất Nam Cao Cấp màu ngẫu nhiên)</t>
+          <t>Dép quai kẹp Bitis nam (38-43)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-3-qua-n-lo-t-nam-so-i-cotton-organic-me-m-mi-n-thoa-ng-ma-t-co-gia-n-4-chie-u-mrm-manlywear-tang-doi-tat-nam-cao-cap-mau-ngau-nhien-p52189164.html?spid=52189172</t>
+          <t>https://tiki.vn/dep-quai-kep-bitis-nam-38-43-p275431635.html?spid=275431639</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>255000</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>255000</v>
+        <v>75000</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>75000</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>3420</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3424</v>
+        <v>22</v>
       </c>
       <c r="L6" t="n">
+        <v>22</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>4</v>
       </c>
-      <c r="M6" t="n">
-        <v>1020000</v>
-      </c>
-      <c r="N6" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="O6" t="n">
-        <v>4.6</v>
-      </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q6" t="n">
-        <v>967</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>967</v>
+        <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Bán thêm +4 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>104791604</t>
+          <t>16651795</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Quần lót nữ thái lan 828 – Chất thun lạnh - giao màu ngẫu nhiên</t>
+          <t>️[5 Quần] ComBo 5 Quần Lót Nam THUN LẠNH Lưng Bự Hàng Việt Nam Cao Cấp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nu-thai-lan-828-chat-thun-lanh-giao-mau-ngau-nhien-p104791604.html?spid=270215619</t>
+          <t>https://tiki.vn/5-quan-combo-5-quan-lot-nam-thun-lanh-lung-bu-hang-viet-nam-cao-cap-p16651795.html?spid=51148098</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MENLIVE</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>35640</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>44000</v>
+        <v>155800</v>
       </c>
       <c r="H7" t="n">
-        <v>8360</v>
+        <v>155800</v>
       </c>
       <c r="I7" t="n">
-        <v>23.46</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="L7" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="M7" t="n">
-        <v>748000</v>
+        <v>1402200</v>
       </c>
       <c r="N7" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
         <v>2</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Giá tăng 8,360đ (+23.5%) | Bán thêm +17 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>49733157</t>
+          <t>275431720</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Quần bơi nam giới dáng vừa, độ dài trên gối, chất thun bơi lạnh dày đẹp, co giãn 4 chiều ôm đùi gọn gàng dễ chịu, thoáng mát nhanh khô | BN005</t>
+          <t>Dép quai kẹp Bitis nam (38-43)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-boi-nam-dang-lung-mau-moi-2020-vai-boi-day-dan-dep-co-gian-4-chieu-bn005-p49733157.html?spid=49733163</t>
+          <t>https://tiki.vn/dep-quai-kep-bitis-nam-38-43-p275431720.html?spid=275431728</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>115000</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>115000</v>
+        <v>75000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>75000</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>101</v>
+        <v>8</v>
       </c>
       <c r="L8" t="n">
+        <v>8</v>
+      </c>
+      <c r="M8" t="n">
+        <v>600000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>5</v>
       </c>
-      <c r="M8" t="n">
-        <v>575000</v>
-      </c>
-      <c r="N8" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="O8" t="n">
-        <v>4.6</v>
-      </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q8" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +5 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>276303219</t>
+          <t>34159013</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bộ Váy Thể Thao Nữ Gồm Áo Thun Và Váy 2 Lớp Sành Điệu</t>
+          <t>Combo 5 Đôi Tất Cổ Ngắn Cùng Màu Cotton Thương Hiệu MRM Manlywear</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-vay-the-thao-nu-gom-ao-thun-va-vay-2-lop-sanh-dieu-p276303219.html?spid=276306416</t>
+          <t>https://tiki.vn/combo-5-doi-tat-nam-vo-nam-co-ngan-cao-cap-mrm-fashion-cung-mau-p34159013.html?spid=34159015</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MRM Manlywear</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>129000</v>
       </c>
       <c r="G9" t="n">
-        <v>239000</v>
+        <v>129000</v>
       </c>
       <c r="H9" t="n">
-        <v>239000</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>5467</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>5470</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>239000</v>
+        <v>387000</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>1101</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>1101</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +3 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>107802069</t>
+          <t>212048690</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
+          <t>NHIỀU MẪU Ghim cài áo đính đá xích cao cấp - ghim cài vest cưới Tien Nguyen</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
+          <t>https://tiki.vn/nhieu-mau-ghim-cai-ao-dinh-da-xich-cao-cap-ghim-cai-vest-cuoi-tien-nguyen-p212048690.html?spid=212048699</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>32000</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>32000</v>
+        <v>159000</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>159000</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1022</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1028</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>192000</v>
+        <v>159000</v>
       </c>
       <c r="N10" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q10" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Bán thêm +6 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>67538621</t>
+          <t>107802069</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
+          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538631</t>
+          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>May 10</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>135000</v>
+        <v>32000</v>
       </c>
       <c r="G11" t="n">
-        <v>135000</v>
+        <v>32000</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1335,38 +1335,38 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>16591</v>
+        <v>1028</v>
       </c>
       <c r="K11" t="n">
-        <v>16592</v>
+        <v>1029</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>135000</v>
+        <v>32000</v>
       </c>
       <c r="N11" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="O11" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>4842</v>
+        <v>68</v>
       </c>
       <c r="R11" t="n">
-        <v>4842</v>
+        <v>68</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1383,74 +1383,74 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>31649352</t>
+          <t>276945307</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2 cặp miếng lót mũi giày nam cao su non đệm êm ngón chân - buybox - BBPK50</t>
+          <t>Áo lót nữ Angelavic 529 – Bra thun lạnh tăm, mút liền, cài sau, không gọng, nâng đỡ thoải mái</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/2-cap-mieng-lot-mui-giay-nam-cao-su-non-dem-em-ngon-chan-buybox-bbpk50-p31649352.html?spid=85084352</t>
+          <t>https://tiki.vn/ao-lot-nu-ao-bra-thun-lanh-tam-mut-lien-cai-sau-529-p276945307.html?spid=276945325</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>buybox</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>34000</v>
+        <v>84700</v>
       </c>
       <c r="G12" t="n">
-        <v>34000</v>
+        <v>110000</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>25300</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>29.87</v>
       </c>
       <c r="J12" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>102000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,29 +1460,29 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Bán thêm +3 sản phẩm</t>
+          <t>Giá tăng 25,300đ (+29.9%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>272890964</t>
+          <t>277877891</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hộp 40 Viên Pin Nhí AAA (3A) Maxell Super 1.5V - Sử dụng cho remote TV, remote máy lạnh,...</t>
+          <t>Móc Nối Tăng Size Áo Ngực 3 Móc 59S – Phụ Kiện Nới Rộng Bra Linh Hoạt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-40-vien-pin-nhi-aaa-3a-maxell-super-1-5v-su-dung-cho-remote-tv-remote-may-lanh-p272890964.html?spid=279273132</t>
+          <t>https://tiki.vn/moc-noi-tang-size-ao-nguc-3-moc-59s-phu-kien-noi-rong-bra-linh-hoat-p277877891.html?spid=277877897</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1491,50 +1491,50 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>98000</v>
+        <v>15400</v>
       </c>
       <c r="G13" t="n">
-        <v>98000</v>
+        <v>20000</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>4600</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>29.87</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K13" t="n">
+        <v>23</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="n">
+      <c r="R13" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="n">
-        <v>98000</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,29 +1544,29 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá tăng 4,600đ (+29.9%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>207271635</t>
+          <t>193886649</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mũ lưỡi trai nam đẹp chất liệu vải dù thoáng mát dễ thấm hút mồ hôi kiểu dáng đẹp phù hợp cả nam và nữ</t>
+          <t>Áo sơ mi nữ form rộng kiểu tay lỡ cổ tròn NeSa Shop, chất liệu Đũi tơ thấm hút mồ hôi, áo sơ mi nữ nhiều màu, SMH.034</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mu-luoi-trai-nam-dep-chat-lieu-vai-du-thoang-mat-de-tham-hut-mo-hoi-kieu-dang-dep-phu-hop-ca-nam-va-nu-p207271635.html?spid=207271648</t>
+          <t>https://tiki.vn/ao-so-mi-nu-form-rong-kieu-tay-lo-co-tron-nesa-shop-chat-lieu-dui-to-tham-hut-mo-hoi-ao-so-mi-nu-nhieu-mau-smh-34-p193886649.html?spid=193886658</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1575,94 +1575,94 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>189000</v>
       </c>
       <c r="G14" t="n">
-        <v>24900</v>
+        <v>189000</v>
       </c>
       <c r="H14" t="n">
-        <v>24900</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>74700</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="O14" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q14" t="n">
         <v>5</v>
       </c>
-      <c r="P14" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="S14" t="n">
         <v>1</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Rating 4.2→4.3 (+0.10) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>163806087</t>
+          <t>277544802</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da</t>
+          <t>Áo Chống Nắng Nam ,Chất Vải Thun Lạnh, Chống Tia UV, Thoáng Mát, Thấm Hút Mồ Hôi</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-p163806087.html?spid=253461440</t>
+          <t>https://tiki.vn/ao-chong-nang-nam-chat-vai-thun-lanh-chong-tia-uv-thoang-mat-tham-hut-mo-hoi-p277544802.html?spid=277544808</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>Kun93</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>59000</v>
+        <v>185000</v>
       </c>
       <c r="G15" t="n">
-        <v>59000</v>
+        <v>185000</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -1671,16 +1671,16 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="K15" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>59000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>5</v>
@@ -1692,17 +1692,17 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1712,29 +1712,29 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>252533129</t>
+          <t>244297794</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Găng Tay Hở 2 Ngón Unisex Chống Nắng, Có Thể Sử Dụng Cảm Ứng Điện Thoại</t>
+          <t>Combo 5 Quần Lót Nam Thun Lạnh Lưng To Menlive ML1 – Size M–4XL, Co Giãn 4 Chiều</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/gang-tay-ho-2-ngon-unisex-chong-nang-co-the-su-dung-cam-ung-dien-thoai-p252533129.html?spid=252533130</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-thun-lanh-menlive-p244297794.html?spid=244297815</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1743,28 +1743,28 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>49000</v>
+        <v>150100</v>
       </c>
       <c r="G16" t="n">
-        <v>49000</v>
+        <v>190000</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>39900</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>26.58</v>
       </c>
       <c r="J16" t="n">
-        <v>160</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
-        <v>161</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>49000</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>5</v>
@@ -1776,17 +1776,17 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="R16" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1796,81 +1796,81 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá tăng 39,900đ (+26.6%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>140429170</t>
+          <t>115852451</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bao tay chơi game găng tay 2 ngón cảm ứng điện thoại gamemobile BT01</t>
+          <t>Chai vệ sinh giày đồ da, túi ví, áo, ghế da giúp làm sạch, dưỡng ẩm chống mốc XIMO XI03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bao-tay-choi-game-gang-tay-2-ngon-cam-ung-dien-thoai-gamemobile-bt01-p140429170.html?spid=198934954</t>
+          <t>https://tiki.vn/chai-ve-sinh-giay-do-da-tui-vi-ao-ghe-da-giup-lam-sach-duong-am-chong-moc-ximo-xi03-p115852451.html?spid=262784198</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>17999</v>
+        <v>70000</v>
       </c>
       <c r="G17" t="n">
-        <v>9999</v>
+        <v>75000</v>
       </c>
       <c r="H17" t="n">
-        <v>-8000</v>
+        <v>5000</v>
       </c>
       <c r="I17" t="n">
-        <v>-44.45</v>
+        <v>7.14</v>
       </c>
       <c r="J17" t="n">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="K17" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="L17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>39996</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1880,47 +1880,47 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá giảm 8,000đ (44.4%) | Bán thêm +4 sản phẩm</t>
+          <t>Giá tăng 5,000đ (+7.1%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>244298960</t>
+          <t>279215984</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Quần Mặc Váy Su Thông Hơi Trơn 6530 | Mát Mẻ, Không Lộ, Chống Hớ Hiệu Quả</t>
+          <t>Dép quai Ngang Biti's nam (39-44)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-vay-dai-thong-hoi-6530-p244298960.html?spid=244298972</t>
+          <t>https://tiki.vn/dep-quai-ngang-biti-s-nam-39-44-p279215984.html?spid=279216018</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>33180</v>
+        <v>184000</v>
       </c>
       <c r="G18" t="n">
-        <v>42000</v>
+        <v>184000</v>
       </c>
       <c r="H18" t="n">
-        <v>8820</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>26.58</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1938,23 +1938,23 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1964,24 +1964,24 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá tăng 8,820đ (+26.6%)</t>
+          <t>Rating 0.0→5.0 (+5.00) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>277844658</t>
+          <t>112851354</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Đồ bơi nữ dạng váy duyên dáng kín đáo có quần short liền trong váy</t>
+          <t>Áo ngực học sinh</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/do-boi-nu-dang-vay-duyen-dang-kin-dao-co-quan-short-lien-trong-vay-p277844658.html?spid=278668799</t>
+          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138790</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1995,22 +1995,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>219000</v>
+        <v>40000</v>
       </c>
       <c r="G19" t="n">
-        <v>259000</v>
+        <v>32800</v>
       </c>
       <c r="H19" t="n">
-        <v>40000</v>
+        <v>-7200</v>
       </c>
       <c r="I19" t="n">
-        <v>18.26</v>
+        <v>-18</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,26 +2019,26 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,29 +2048,29 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá tăng 40,000đ (+18.3%)</t>
+          <t>Giá giảm 7,200đ (18.0%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>277996544</t>
+          <t>277274436</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hộp 5 Quần lót nam cotton lụa – Siêu đẹp, mềm mịn, thoáng mát</t>
+          <t>Set áo cổ tròn sát nách phối quần ống suông thanh lịch</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-5-quan-lot-nam-cotton-lua-muji-sieu-dep-mem-min-thoang-mat-p277996544.html?spid=278006738</t>
+          <t>https://tiki.vn/set-ao-co-tron-sat-nach-phoi-quan-ong-suong-thanh-lich-p277274436.html?spid=277274444</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2079,22 +2079,22 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>172000</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>222000</v>
+        <v>199000</v>
       </c>
       <c r="H20" t="n">
-        <v>50000</v>
+        <v>199000</v>
       </c>
       <c r="I20" t="n">
-        <v>29.07</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -2103,53 +2103,53 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Giá tăng 50,000đ (+29.1%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>37126497</t>
+          <t>113145806</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>( 10 cái ) quần lót nữ Su đúc không đường may, hàng đẹp loại xịn W19_503</t>
+          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/set-10-quan-lot-su-duc-khong-duong-may-hang-dep-loai-xin-w19_503-p37126497.html?spid=51720423</t>
+          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2163,22 +2163,22 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>218400</v>
+        <v>117000</v>
       </c>
       <c r="G21" t="n">
-        <v>280000</v>
+        <v>97110</v>
       </c>
       <c r="H21" t="n">
-        <v>61600</v>
+        <v>-19890</v>
       </c>
       <c r="I21" t="n">
-        <v>28.21</v>
+        <v>-17</v>
       </c>
       <c r="J21" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2187,26 +2187,26 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2216,53 +2216,53 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Giá tăng 61,600đ (+28.2%)</t>
+          <t>Giá giảm 19,890đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>140961698</t>
+          <t>113144956</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Giày Lười Nam Da Bò SUNPOLO SUS510 (Đen, Nâu)</t>
+          <t>siêu phẩm áo lót nhật trơn đệm nâng ngực nhẹ</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-luoi-nam-da-bo-sunpolo-sus510-den-nau-p140961698.html?spid=140961714</t>
+          <t>https://tiki.vn/sieu-pham-ao-lot-tron-dem-nang-nguc-nhe-p113144956.html?spid=142116876</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SUNPOLO</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1035000</v>
+        <v>165000</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>136950</v>
       </c>
       <c r="H22" t="n">
-        <v>-1035000</v>
+        <v>-28050</v>
       </c>
       <c r="I22" t="n">
-        <v>-100</v>
+        <v>-17</v>
       </c>
       <c r="J22" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -2274,79 +2274,79 @@
         <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" t="n">
         <v>0</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá giảm 28,050đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>66083356</t>
+          <t>66507793</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Áo phông cổ tròn ALIGRO ALGAPC044</t>
+          <t>Dép Nam Da Bò BIGGBEN Cao Cấp DN260</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-phong-co-tron-aligro-algapc044-p66083356.html?spid=66083362</t>
+          <t>https://tiki.vn/dep-nam-da-bo-biggben-cao-cap-dn260-p66507793.html?spid=66507799</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Aligro</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>369000</v>
       </c>
       <c r="G23" t="n">
-        <v>150000</v>
+        <v>400000</v>
       </c>
       <c r="H23" t="n">
-        <v>150000</v>
+        <v>31000</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -2355,82 +2355,82 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 31,000đ (+8.4%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>278698318</t>
+          <t>177666546</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Set đồ đùi ba lỗ nữ tập thể thao, mặc nhà hàng Quảng Châu loại 1</t>
+          <t>Dép Nam Quai Ngang Da Bò Thật BIGGBEN Cao Cấp DN308</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/set-do-dui-ba-lo-nu-tap-the-thao-mac-nha-hang-quang-chau-loai-1-p278698318.html?spid=278698340</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-that-biggben-cao-cap-dn308-p177666546.html?spid=177666552</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>319000</v>
+        <v>289000</v>
       </c>
       <c r="G24" t="n">
-        <v>335000</v>
+        <v>380000</v>
       </c>
       <c r="H24" t="n">
-        <v>16000</v>
+        <v>91000</v>
       </c>
       <c r="I24" t="n">
-        <v>5.02</v>
+        <v>31.49</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2439,26 +2439,26 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
         <v>0</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2468,24 +2468,24 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Giá tăng 16,000đ (+5.0%)</t>
+          <t>Giá tăng 91,000đ (+31.5%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>63174143</t>
+          <t>250056510</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dép Nam Da Bò BIGGBEN Cao Cấp DN258</t>
+          <t>Dép Nam Quai Ngang BIGGBEN Da Bò Thật Cao Cấp DN332</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-da-bo-biggben-cao-cap-dn258-p63174143.html?spid=63174147</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-biggben-da-bo-that-cao-cap-dn332-p250056510.html?spid=250056524</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2499,22 +2499,22 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>500000</v>
+        <v>369000</v>
       </c>
       <c r="G25" t="n">
-        <v>419000</v>
+        <v>450000</v>
       </c>
       <c r="H25" t="n">
-        <v>-81000</v>
+        <v>81000</v>
       </c>
       <c r="I25" t="n">
-        <v>-16.2</v>
+        <v>21.95</v>
       </c>
       <c r="J25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2523,26 +2523,26 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2552,53 +2552,53 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Giá giảm 81,000đ (16.2%)</t>
+          <t>Giá tăng 81,000đ (+22.0%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>279068959</t>
+          <t>59206687</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Áo thun tay ngắn nam sọc ngang. Regular - ROUTINE 10F25TSS036</t>
+          <t>GIày Sandal Nam Da Bò BIGGBEN Cao Cấp SD105</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-tay-ngan-nam-soc-ngang-regular-routine-10f25tss036-p279068959.html?spid=279068973</t>
+          <t>https://tiki.vn/giay-sandal-nam-da-bo-biggben-cao-cap-sd105-p59206687.html?spid=59206699</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Routine</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>379000</v>
       </c>
       <c r="G26" t="n">
-        <v>379000</v>
+        <v>439000</v>
       </c>
       <c r="H26" t="n">
-        <v>379000</v>
+        <v>60000</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>15.83</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -2607,82 +2607,82 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S26" t="n">
         <v>0</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 60,000đ (+15.8%)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>183895879</t>
+          <t>278872546</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Bình xịt lưu hương chống thối chân, khử mùi giày XIMO, kháng khuẩn, công nghệ Bạc ion (VSG08-1)</t>
+          <t>Áo thun tay ngắn nam.Fitted - ROUTINE 10F25TSS039</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/binh-xit-luu-huong-chong-thoi-chan-khu-mui-giay-ximo-khang-khuan-cong-nghe-bac-ion-vsg08-p183895879.html?spid=252869682</t>
+          <t>https://tiki.vn/ao-thun-tay-ngan-nam-fitted-routine-10f25tss039-p278872546.html?spid=278872558</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>71000</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>66000</v>
+        <v>349000</v>
       </c>
       <c r="H27" t="n">
-        <v>-5000</v>
+        <v>349000</v>
       </c>
       <c r="I27" t="n">
-        <v>-7.04</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>159</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>159</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2691,82 +2691,82 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>0</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Giá giảm 5,000đ (7.0%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>152632563</t>
+          <t>276094684</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Áo Lót Nữ Mút Mỏng Trơn Không Gọng 3281 – Nhẹ Êm, Tự Nhiên, Dễ Mặc Mỗi Ngày</t>
+          <t>Dép Nam Quai Ngang BIGGBEN Da Bò Thật DN356</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-duc-kiem-bra-cao-cap-3281-big-size-p152632563.html?spid=274990712</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-biggben-da-bo-that-dn356-p276094684.html?spid=276094690</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>80190</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>99000</v>
+        <v>389000</v>
       </c>
       <c r="H28" t="n">
-        <v>18810</v>
+        <v>389000</v>
       </c>
       <c r="I28" t="n">
-        <v>23.46</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -2794,63 +2794,63 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Giá tăng 18,810đ (+23.5%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>115852451</t>
+          <t>275233185</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chai vệ sinh giày đồ da, túi ví, áo, ghế da giúp làm sạch, dưỡng ẩm chống mốc XIMO XI03</t>
+          <t>Áo Thun ROUTINE Tay Ngắn Dệt Jacquard Phối Nhãn Form Loose - 10S24TSS014 | LASTORE MENSWEAR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-ve-sinh-giay-do-da-tui-vi-ao-ghe-da-giup-lam-sach-duong-am-chong-moc-ximo-xi03-p115852451.html?spid=262784198</t>
+          <t>https://tiki.vn/ao-thun-routine-tay-ngan-det-jacquard-phoi-nhan-form-loose-10s24tss014-lastore-menswear-p275233185.html?spid=275233197</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>70000</v>
+        <v>399000</v>
       </c>
       <c r="H29" t="n">
-        <v>-5000</v>
+        <v>399000</v>
       </c>
       <c r="I29" t="n">
-        <v>-6.67</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -2859,36 +2859,36 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
         <v>0</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Giá giảm 5,000đ (6.7%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
@@ -2919,16 +2919,16 @@
         </is>
       </c>
       <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
         <v>460000</v>
       </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
       <c r="H30" t="n">
-        <v>-460000</v>
+        <v>460000</v>
       </c>
       <c r="I30" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -2949,7 +2949,7 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -2962,63 +2962,63 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>191694860</t>
+          <t>274350557</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Giày da nam công sở đế cao Bụi Leather G123 - Da bò Nappa cao cấp - Phong cách trẻ trung năng động - Bảo hành 12 tháng</t>
+          <t>Hộp 100 Khăn Lau Kính Nano, Chống Bám Hơi Nước, Chống Bụi Bẩn - Khăn Lau Kính Nano Hộp 100 Miếng Giấy Lau Kính Chống Bám Hơi Nước, Lau Sạch Vân Tay Bụi Bẩn</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-da-nam-cong-so-de-cao-bui-leather-g123-da-bo-nappa-cao-cap-phong-cach-tre-trung-nang-dong-bao-hanh-12-thang-p191694860.html?spid=191694870</t>
+          <t>https://tiki.vn/hop-100-khan-lau-kinh-nano-chong-bam-hoi-nuoc-chong-bui-ban-khan-lau-kinh-nano-hop-100-mieng-giay-lau-kinh-chong-bam-hoi-nuoc-lau-sach-van-tay-bui-ban-p274350557.html?spid=274350558</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bụi Leather</t>
+          <t>fofaHome</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>925000</v>
+        <v>20000</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>17000</v>
       </c>
       <c r="H31" t="n">
-        <v>-925000</v>
+        <v>-3000</v>
       </c>
       <c r="I31" t="n">
-        <v>-100</v>
+        <v>-15</v>
       </c>
       <c r="J31" t="n">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -3030,50 +3030,50 @@
         <v>5</v>
       </c>
       <c r="O31" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P31" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá giảm 3,000đ (15.0%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>275835289</t>
+          <t>183895879</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dép Nam Quai Ngang BIGGBEN Da Bò Thật DN355</t>
+          <t>Bình xịt lưu hương chống thối chân, khử mùi giày XIMO, kháng khuẩn, công nghệ Bạc ion (VSG08-1)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-quai-ngang-biggben-da-bo-that-dn355-p275835289.html?spid=275835315</t>
+          <t>https://tiki.vn/binh-xit-luu-huong-chong-thoi-chan-khu-mui-giay-ximo-khang-khuan-cong-nghe-bac-ion-vsg08-p183895879.html?spid=252869682</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3083,26 +3083,26 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>66000</v>
       </c>
       <c r="G32" t="n">
-        <v>399000</v>
+        <v>71000</v>
       </c>
       <c r="H32" t="n">
-        <v>399000</v>
+        <v>5000</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -3111,53 +3111,53 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="R32" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="S32" t="n">
         <v>0</v>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 5,000đ (+7.6%)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>262085586</t>
+          <t>192419827</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hộp 100 Miếng Khăn Lau Mắt Kính Nano Chống Mờ Sương, Bám Hơi Nước</t>
+          <t>Khăn Lau Kính Nano Hộp 100 Miếng Giấy Lau Kính Chống Bám Hơi Nước, Lau Sạch Vân Tay Bụi Bẩn</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-100-mieng-khan-lau-mat-kinh-nano-chong-mo-suong-bam-hoi-nuoc-p262085586.html?spid=277964244</t>
+          <t>https://tiki.vn/khan-lau-kinh-nano-hop-100-mieng-giay-lau-kinh-chong-bam-hoi-nuoc-lau-sach-van-tay-bui-ban-p192419827.html?spid=278272152</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3183,10 +3183,10 @@
         <v>17.65</v>
       </c>
       <c r="J33" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="K33" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
@@ -3195,26 +3195,26 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O33" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S33" t="n">
         <v>0</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3231,17 +3231,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>246853757</t>
+          <t>78513044</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GĂNG TAY CHỐNG NẮNG CHO NỮ</t>
+          <t>Khăn ống cotton tube co giãn 9 kiểu dùng có video hướng dẫn  TUBE01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://tiki.vn/gang-tay-chong-nang-cho-nu-p246853757.html?spid=273131602</t>
+          <t>https://tiki.vn/khan-ong-cotton-tube-co-gian-9-kieu-dung-co-video-huong-dan-tube01-p78513044.html?spid=78518779</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3251,26 +3251,26 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Song An Eco</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>42000</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>48000</v>
+        <v>15000</v>
       </c>
       <c r="H34" t="n">
-        <v>6000</v>
+        <v>15000</v>
       </c>
       <c r="I34" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -3279,82 +3279,82 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Giá tăng 6,000đ (+14.3%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>192419827</t>
+          <t>163902369</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Khăn Lau Kính Nano Hộp 100 Miếng Giấy Lau Kính Chống Bám Hơi Nước, Lau Sạch Vân Tay Bụi Bẩn</t>
+          <t>Áo Sơ Mi Nam Xanh Dương Kẻ Caro Ngắn Tay Công Sở Trung Niên Thương Hiệu Anton Vải Sợi Tre - YGD566</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://tiki.vn/khan-lau-kinh-nano-hop-100-mieng-giay-lau-kinh-chong-bam-hoi-nuoc-lau-sach-van-tay-bui-ban-p192419827.html?spid=278272152</t>
+          <t>https://tiki.vn/ao-so-mi-nam-xanh-duong-ke-caro-ngan-tay-cong-so-trung-nien-thuong-hieu-anton-vai-soi-tre-ygd566-p163902369.html?spid=163902371</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>SOMIANTON</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>20000</v>
+        <v>355000</v>
       </c>
       <c r="G35" t="n">
-        <v>17000</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>-3000</v>
+        <v>-355000</v>
       </c>
       <c r="I35" t="n">
-        <v>-15</v>
+        <v>-100</v>
       </c>
       <c r="J35" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="K35" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -3366,76 +3366,76 @@
         <v>5</v>
       </c>
       <c r="O35" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
         <v>0</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Giá giảm 3,000đ (15.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>279122825</t>
+          <t>176881225</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Thắt lưng nữ phong cách Hàn Quốc, dây nịt quần tây/quần jean da tổng hợp thanh lịch IDIGO FD2-0052</t>
+          <t>Đồ Bơi Nữ Tay Dài Quần Ôm Thân Tôn Dáng AT221 MayHomes Long Sleeves And Long Pants Women Swimwear Set With UPF 50 Sun Protection</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-nu-phong-cach-han-quoc-day-nit-quan-tay-quan-jean-da-tong-hop-thanh-lich-idigo-fd2-0052-p279122825.html?spid=279122831</t>
+          <t>https://tiki.vn/do-boi-nu-tay-dai-quan-om-than-ton-dang-at221-mayhomes-long-sleeves-and-long-pants-women-swimwear-set-with-upf-50-sun-protection-p176881225.html?spid=176881229</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>IDIGO</t>
+          <t>MAYHOMES</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>288000</v>
       </c>
       <c r="G36" t="n">
-        <v>117090</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>117090</v>
+        <v>-288000</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -3447,16 +3447,16 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>-4.8</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3466,34 +3466,34 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>251424864</t>
+          <t>269878543</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Đồ ngủ nữ Wannabe DNS74 đầm ngủ hai dây cổ tim nền hoa xinh xắn trang nhã</t>
+          <t>Cuộn 8M Băng Dán Cổ Áo Sơ Mi Chống Bẩn Vải Không Dệt Thoáng Khí Bám Dính Tốt Thấm Hút Mồ Hôi</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://tiki.vn/do-ngu-nu-wannabe-dns74-dam-ngu-hai-day-co-tim-nen-hoa-xinh-xan-trang-nha-p251424864.html?spid=270903252</t>
+          <t>https://tiki.vn/cuon-8m-bang-dan-co-ao-so-mi-chong-ban-vai-khong-det-thoang-khi-bam-dinh-tot-tham-hut-mo-hoi-p269878543.html?spid=269878549</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3503,23 +3503,23 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wannabe</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>300000</v>
+        <v>39000</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>-300000</v>
+        <v>-39000</v>
       </c>
       <c r="I37" t="n">
         <v>-100</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -3531,16 +3531,16 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>-0</v>
+        <v>-4.3</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -3567,22 +3567,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>212048690</t>
+          <t>6535821</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NHIỀU MẪU Ghim cài áo đính đá xích cao cấp - ghim cài vest cưới Tien Nguyen</t>
+          <t>Quần Lót Nữ - Quần Đùi Mặc Trong Váy Su Thông Hơi</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://tiki.vn/nhieu-mau-ghim-cai-ao-dinh-da-xich-cao-cap-ghim-cai-vest-cuoi-tien-nguyen-p212048690.html?spid=212048699</t>
+          <t>https://tiki.vn/quan-lot-nu-quan-dui-mac-trong-vay-su-thong-hoi-p6535821.html?spid=51154654</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3591,19 +3591,19 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>159000</v>
+        <v>42000</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>-159000</v>
+        <v>-42000</v>
       </c>
       <c r="I38" t="n">
         <v>-100</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -3615,16 +3615,16 @@
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>-5</v>
+        <v>-4.7</v>
       </c>
       <c r="Q38" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -3651,43 +3651,43 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>278274146</t>
+          <t>273611089</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Củ Cap O.p..p.o 30W_33W_67W Sạc Nhanh Công Nghệ SupperVooc Zin Hãng Cam Kết</t>
+          <t>Xi Đánh Bóng Giày Da Làm Bóng Nhanh Đồ Da, Xi Kem Dưỡng Da Có Đầu Mút Hỗ Trợ - HÀNG CHÍNH HÃNG MINIIN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cu-cap-oppo-30w_33w_67w-sac-nhanh-cong-nghe-suppervooc-zin-chinh-hang-cam-ket-p278274146.html?spid=278292995</t>
+          <t>https://tiki.vn/xi-danh-bong-giay-da-lam-bong-nhanh-do-da-xi-kem-duong-da-co-da-u-mu-t-ho-tro-hang-chinh-hang-miniin-p273611089.html?spid=273611093</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MINIIN</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>165000</v>
+        <v>35000</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>-165000</v>
+        <v>-35000</v>
       </c>
       <c r="I39" t="n">
         <v>-100</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -3699,16 +3699,16 @@
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>-0</v>
+        <v>-3.6</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -3735,17 +3735,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6394813</t>
+          <t>107491961</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Giày Tây Nam BIGGBEN Da Bò Thật GT17</t>
+          <t>Dép Nam Quai Ngang Da Bò BIGGBEN Cao Cấp DN283</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-biggben-da-bo-that-gt17-p6394813.html?spid=6394833</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-biggben-cao-cap-dn283-p107491961.html?spid=107491965</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3759,19 +3759,19 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>720000</v>
+        <v>319000</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>-720000</v>
+        <v>-319000</v>
       </c>
       <c r="I40" t="n">
         <v>-100</v>
       </c>
       <c r="J40" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -3783,16 +3783,16 @@
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>-4.7</v>
+        <v>-0</v>
       </c>
       <c r="Q40" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -3819,43 +3819,43 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>275233185</t>
+          <t>275933718</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Áo Thun ROUTINE Tay Ngắn Dệt Jacquard Phối Nhãn Form Loose - 10S24TSS014 | LASTORE MENSWEAR</t>
+          <t>Giày Sneaker Vải Canvas Nam Nữ E18 White Dincox Shoes Sang Trọng</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-routine-tay-ngan-det-jacquard-phoi-nhan-form-loose-10s24tss014-lastore-menswear-p275233185.html?spid=275233197</t>
+          <t>https://tiki.vn/giay-sneaker-vai-canvas-nam-nu-e18-white-dincox-shoes-sang-trong-p275933718.html?spid=275933722</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Routine</t>
+          <t>DINCOX</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>399000</v>
+        <v>490000</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>-399000</v>
+        <v>-490000</v>
       </c>
       <c r="I41" t="n">
         <v>-100</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -3867,16 +3867,16 @@
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>-0</v>
+        <v>-1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3886,7 +3886,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -3903,43 +3903,43 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>78513044</t>
+          <t>253306906</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Khăn ống cotton tube co giãn 9 kiểu dùng có video hướng dẫn  TUBE01</t>
+          <t>Đón gót giầy gỗ</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://tiki.vn/khan-ong-cotton-tube-co-gian-9-kieu-dung-co-video-huong-dan-tube01-p78513044.html?spid=78518779</t>
+          <t>https://tiki.vn/don-got-giay-p253306906.html?spid=253306912</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Song An Eco</t>
+          <t>DAICAT</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>15000</v>
+        <v>159000</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>-15000</v>
+        <v>-159000</v>
       </c>
       <c r="I42" t="n">
         <v>-100</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -3987,17 +3987,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>275276260</t>
+          <t>154852782</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dép tổ ong ĐỎ nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Giày Lười, Giày Mọi Nam Da Bò SUNPOLO CS5052 (Đen, Nâu)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-do-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276260.html?spid=275276262</t>
+          <t>https://tiki.vn/giay-luoi-nam-da-bo-sunpolo-su5052-den-nau-p154852782.html?spid=154852796</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4007,81 +4007,81 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>SUNPOLO</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>63000</v>
+        <v>1100000</v>
       </c>
       <c r="G43" t="n">
-        <v>63000</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>-1100000</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J43" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
         <v>4</v>
       </c>
-      <c r="L43" t="n">
-        <v>-2</v>
-      </c>
-      <c r="M43" t="n">
-        <v>-126000</v>
-      </c>
-      <c r="N43" t="n">
-        <v>5</v>
-      </c>
       <c r="O43" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="Q43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R43" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S43" t="n">
         <v>0</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>Bán thêm -2 sản phẩm</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>195305781</t>
+          <t>279068959</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Combo 3 quần đùi mặc nhà - Giao màu ngẫu nhiên</t>
+          <t>Áo thun tay ngắn nam sọc ngang. Regular - ROUTINE 10F25TSS036</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-3-quan-dui-mac-nha-giao-mau-ngau-nhien-p195305781.html?spid=195305789</t>
+          <t>https://tiki.vn/ao-thun-tay-ngan-nam-soc-ngang-regular-routine-10f25tss036-p279068959.html?spid=279068973</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4091,81 +4091,81 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Novelty</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>285000</v>
+        <v>379000</v>
       </c>
       <c r="G44" t="n">
-        <v>285000</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>-379000</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J44" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>-285000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O44" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S44" t="n">
         <v>0</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Bán thêm -1 sản phẩm</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>14351068</t>
+          <t>66095198</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Áo thun Nam có cổ thời trang</t>
+          <t>Áo phông cổ tim ALIGRO ALGAPC051</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-nam-co-co-thoi-trang-p14351068.html?spid=14351082</t>
+          <t>https://tiki.vn/ao-phong-co-tim-aligro-algapc051-p66095198.html?spid=66095200</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4175,64 +4175,316 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Aligro</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>160000</v>
+        <v>150000</v>
       </c>
       <c r="G45" t="n">
-        <v>160000</v>
+        <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>-150000</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J45" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>-640000</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="Q45" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>❌ Đã xóa</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Không còn xuất hiện trong danh sách</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>66083356</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Áo phông cổ tròn ALIGRO ALGAPC044</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/ao-phong-co-tron-aligro-algapc044-p66083356.html?spid=66083362</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Thời trang nam</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Aligro</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-150000</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-100</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>❌ Đã xóa</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Không còn xuất hiện trong danh sách</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>277811866</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BỘ Găng Tay Bao Tay Ống Chống Nắng Cao Cấp Unisex MÀU XÁM</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/khan-trum-dau-ninja-fullface-chong-nang-mau-den-p277811866.html?spid=277811867</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Phụ kiện thời trang</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LuckyJQR</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-100</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
         <v>5</v>
       </c>
-      <c r="S45" t="n">
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>-5</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>1</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>❌ Đã xóa</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Không còn xuất hiện trong danh sách</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>102151424</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Kính mát nam EXFASH EF38973 thời trang (62/14/145)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/kinh-mat-nam-exfash-ef38973-thoi-trang-62-14-145-p102151424.html?spid=102151428</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Phụ kiện thời trang</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Exfash</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>529000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-529000</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-100</v>
+      </c>
+      <c r="J48" t="n">
         <v>2</v>
       </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>Bán thêm -4 sản phẩm | Rating 4.7→4.8 (+0.10) | Review thêm +2</t>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>5</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-5</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>1</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>❌ Đã xóa</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-06-23
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V40"/>
+  <dimension ref="A1:V37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,37 +543,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>193978418</t>
+          <t>2302097</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Quần Jean nam Leman xám khói trơn JD13 - Slim Form</t>
+          <t>Combo 3 Đôi Vớ Nam Cotton Thể Thao Donakein 195F3D1M02 (Free Size)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-jean-nam-leman-xam-khoi-tron-jd13-slim-form-p193978418.html?spid=193978434</t>
+          <t>https://tiki.vn/combo-3-doi-vo-nam-cotton-the-thao-donakein-195f3d1m02-free-size-p2302097.html?spid=2340107</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Leman</t>
+          <t>Donakein</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>549000</v>
+        <v>135000</v>
       </c>
       <c r="H2" t="n">
-        <v>549000</v>
+        <v>135000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,13 +582,13 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M2" t="n">
-        <v>34038000</v>
+        <v>7965000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -603,14 +603,14 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="S2" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -627,17 +627,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2710151</t>
+          <t>208746104</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lót giày sức khỏe Spenco Total Support Thin 46-696 cho giày thể thao, công sở nâng vòm hỗ trợ giảm mỏi chân khi đi nhiều, đứng lâu</t>
+          <t>Giày Thể Thao Biti's Nam Hunter X DSMH10500</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/lot-giay-cong-so-giam-dau-moi-chan-spenco-total-suport-thin-46-696-p2710151.html?spid=2710155</t>
+          <t>https://tiki.vn/giay-the-thao-biti-s-nam-hunter-x-dsmh10500-p208746104.html?spid=208746130</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Spenco</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>895000</v>
+        <v>1050000</v>
       </c>
       <c r="H3" t="n">
-        <v>895000</v>
+        <v>1050000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,35 +666,35 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="M3" t="n">
-        <v>17005000</v>
+        <v>5250000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>276634531</t>
+          <t>278820713</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Thể Thao Sêu Dính Dùng Nhiệt Trong Suốt Không Tổn Thương Da, Keo Dính Giày Đa Năng Siêu Bền Chống Nước Tốt Xanh</t>
+          <t>Dép nhựa Biti's nam (39-44)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-the-thao-seu-dinh-dung-nhiet-trong-suot-khong-ton-thuong-da-keo-dinh-giay-da-nang-sieu-ben-chong-nuoc-tot-p276634531.html?spid=276634532</t>
+          <t>https://tiki.vn/dep-nhua-biti-s-nam-39-44-p278820713.html?spid=278820719</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>LuckyJQR</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>160000</v>
+        <v>206000</v>
       </c>
       <c r="H4" t="n">
-        <v>160000</v>
+        <v>206000</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -750,35 +750,35 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="M4" t="n">
-        <v>5600000</v>
+        <v>1030000</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>4.2</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>4.2</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -795,121 +795,121 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>275262532</t>
+          <t>54569520</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Giày Sandal Nam Nữ Chất Liệu Nhựa EVA Mềm, Nhẹ, Êm Chân, Thoải Mái, Chống Trơn Trượt (FORM LỚN ĐẶT LÙI 1 SIZE) Giày đi học - Giày đi làm - Giày đi chơi</t>
+          <t>Quần Lót nam, quần sịp nam lụa Sữa Cao Cấp sp-340</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-sandal-nam-chat-lieu-nhua-eva-mem-nhe-em-chan-thoai-mai-chong-tron-truot-p275262532.html?spid=279226513</t>
+          <t>https://tiki.vn/quan-lot-nam-quan-sip-nam-lua-sua-cao-cap-sp-340-p54569520.html?spid=67859897</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>68640</v>
       </c>
       <c r="G5" t="n">
-        <v>140000</v>
+        <v>88000</v>
       </c>
       <c r="H5" t="n">
-        <v>140000</v>
+        <v>19360</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>28.21</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L5" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>2520000</v>
+        <v>440000</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 19,360đ (+28.2%) | Bán thêm +5 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>277347854</t>
+          <t>253306906</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Thắt lưng nữ DA BÒ THẬT - BEE GEE N8051</t>
+          <t>Đón gót giầy gỗ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-nu-da-bo-that-bee-gee-n8051-p277347854.html?spid=277347856</t>
+          <t>https://tiki.vn/don-got-giay-p253306906.html?spid=253306912</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bee Gee</t>
+          <t>DAICAT</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>150000</v>
+        <v>159000</v>
       </c>
       <c r="H6" t="n">
-        <v>150000</v>
+        <v>159000</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -918,13 +918,13 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="M6" t="n">
-        <v>1500000</v>
+        <v>318000</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -946,7 +946,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -963,37 +963,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>140836685</t>
+          <t>37269401</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Giày Lười Nam Da Bò SUNPOLO MU2588 (Xanh Navy)</t>
+          <t>Combo 5 Quần Lót Nam Thông Hơi Xuất Nhật Mã S02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-luoi-nam-da-bo-sunpolo-mu2588-xanh-navy-p140836685.html?spid=140836687</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-thong-hoi-xuat-nhat-ma-s02-p37269401.html?spid=198496796</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SUNPOLO</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1200000</v>
+        <v>119000</v>
       </c>
       <c r="H7" t="n">
-        <v>1200000</v>
+        <v>119000</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1002,13 +1002,13 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>1200000</v>
+        <v>238000</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1047,34 +1047,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>52184516</t>
+          <t>52758433</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Combo 3 quần lót nam Boxer sợi Organic mềm mịn thoáng mát co giãn 4 chiều MRM Manlywear ( TẶNG Đôi Tất Nam Cao Cấp Giao Ngẫu Nhiên)</t>
+          <t>Combo 5 Đôi Tất Nam Vớ Nam Cổ Dài Sợi Cotton Mix Màu</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-3-qua-n-lo-t-nam-boxer-so-i-cotton-organic-me-m-mi-n-thoa-ng-ma-t-co-gia-n-4-chie-u-mrm-manlywear-tang-doi-tat-nam-cao-cap-giao-ngau-nhien-p52184516.html?spid=52184518</t>
+          <t>https://tiki.vn/combo-5-doi-tat-nam-vo-nam-co-dai-soi-cotton-mix-mau-p52758433.html?spid=67297062</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>JM Jamano</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>199000</v>
+        <v>99000</v>
       </c>
       <c r="G8" t="n">
-        <v>199000</v>
+        <v>99000</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1083,38 +1083,38 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>4333</v>
+        <v>3762</v>
       </c>
       <c r="K8" t="n">
-        <v>4339</v>
+        <v>3763</v>
       </c>
       <c r="L8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>1194000</v>
+        <v>99000</v>
       </c>
       <c r="N8" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="O8" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>1245</v>
+        <v>1001</v>
       </c>
       <c r="R8" t="n">
-        <v>1245</v>
+        <v>1001</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1124,29 +1124,29 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +6 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16375016</t>
+          <t>274036763</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>COMBO HỘP 5 Quần Lót ĐÙI Nam Xuất Nhật Cao Cấp (MIX NGẪU NHIÊN)</t>
+          <t>Tất vớ lười nữ màu trơn Kikiya cao cấp Hàn Quốc W-N-008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-hop-5-quan-lot-dui-nam-xuat-nhat-cao-cap-mix-ngau-nhien-p16375016.html?spid=277961877</t>
+          <t>https://tiki.vn/tat-vo-luoi-nu-mau-tron-kikiya-cao-cap-han-quoc-w-n-008-p274036763.html?spid=274036764</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1158,10 +1158,10 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>251000</v>
+        <v>44100</v>
       </c>
       <c r="H9" t="n">
-        <v>251000</v>
+        <v>44100</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1170,13 +1170,13 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" t="n">
-        <v>753000</v>
+        <v>88200</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1215,34 +1215,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>275276468</t>
+          <t>19843976</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dép tổ ong XANH NAVY nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Combo 10 Đôi Tất Nam Chống Hôi Chân Thời Trang</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-xanh-navy-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276468.html?spid=275276484</t>
+          <t>https://tiki.vn/combo-10-doi-tat-nam-chong-hoi-chan-thoi-trang-p19843976.html?spid=71526312</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>72000</v>
+        <v>79000</v>
       </c>
       <c r="G10" t="n">
-        <v>72000</v>
+        <v>79000</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1251,38 +1251,38 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>13</v>
+        <v>375</v>
       </c>
       <c r="K10" t="n">
-        <v>23</v>
+        <v>376</v>
       </c>
       <c r="L10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>720000</v>
+        <v>79000</v>
       </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="O10" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="R10" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1292,81 +1292,81 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Bán thêm +10 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>278000485</t>
+          <t>183685137</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Áo lót nữ 718 – Mút mỏng thông hơi, không gọng, cài sau 3 móc, co giãn thoải mái</t>
+          <t>Thắt Lưng Dây Nịt Nam Vải Dù US ARMY, Phong Cách Sang Trọng Cổ Điển Mặt Khóa Hợp Kim Thép Chống Ghỉ Cao Cấp -HÀNG CHÍNH HÃNG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-718-mut-mong-thong-hoi-khong-gong-cai-sau-3-moc-co-gian-thoai-mai-p278000485.html?spid=278000491</t>
+          <t>https://tiki.vn/that-lung-day-nit-nam-vai-du-us-army-phong-cach-sang-trong-co-dien-mat-khoa-hop-kim-thep-chong-ghi-cao-cap-hang-chinh-hang-p183685137.html?spid=183685139</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>US ARMY</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>80000</v>
+        <v>79000</v>
       </c>
       <c r="G11" t="n">
-        <v>100000</v>
+        <v>79000</v>
       </c>
       <c r="H11" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>209</v>
       </c>
       <c r="K11" t="n">
-        <v>9</v>
+        <v>210</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>600000</v>
+        <v>79000</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,81 +1376,81 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Giá tăng 20,000đ (+25.0%) | Bán thêm +6 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>278092142</t>
+          <t>107802069</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Quần kiểu nữ ống rộng, chất liệu vải Đũi xước, mềm mịn, mặc mát, Quần Short nữ đẹp Nesa Shop</t>
+          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-kieu-nu-ong-rong-chat-lieu-vai-dui-xuoc-mem-min-mac-mat-quan-short-nu-dep-nesa-shop-p278092142.html?spid=278092148</t>
+          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>55000</v>
+        <v>32000</v>
       </c>
       <c r="G12" t="n">
-        <v>49000</v>
+        <v>32000</v>
       </c>
       <c r="H12" t="n">
-        <v>-6000</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>-10.91</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1029</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>1030</v>
       </c>
       <c r="L12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>392000</v>
+        <v>32000</v>
       </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="O12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,41 +1460,41 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Giá giảm 6,000đ (10.9%) | Bán thêm +8 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>67538621</t>
+          <t>83423370</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
+          <t>Bộ dụng cụ tua vít đa năng sửa kính, mắt kính</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538631</t>
+          <t>https://tiki.vn/bo-dung-cu-tua-vit-da-nang-sua-kinh-mat-kinh-p83423370.html?spid=113070838</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>May 10</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>135000</v>
+        <v>9500</v>
       </c>
       <c r="G13" t="n">
-        <v>135000</v>
+        <v>9500</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1503,38 +1503,38 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>16590</v>
+        <v>89</v>
       </c>
       <c r="K13" t="n">
-        <v>16592</v>
+        <v>90</v>
       </c>
       <c r="L13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>270000</v>
+        <v>9500</v>
       </c>
       <c r="N13" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="O13" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>4842</v>
+        <v>16</v>
       </c>
       <c r="R13" t="n">
-        <v>4842</v>
+        <v>16</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,24 +1544,24 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Bán thêm +2 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>275738156</t>
+          <t>198300891</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mặt Khóa Thắt Lưng Nam Cao Cấp,Mặt Thắt Lưng Nam Khóa Tự Động 203851</t>
+          <t>Khẩu Trang Chống Tia Uv, Khẩu Trang Chống Nắng Upf 50+ - Unisex Nam Nữ Đều Thích Hợp- Vải Mềm Mát Thoáng Khí</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mat-khoa-that-lung-nam-cao-cap-mat-that-lung-nam-khoa-tu-dong-203851-p275738156.html?spid=275738157</t>
+          <t>https://tiki.vn/khau-trang-chong-tia-uv-khau-trang-chong-nang-upf-50-unisex-nam-nu-deu-thich-hop-vai-mem-mat-thoang-khi-p198300891.html?spid=279253596</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1571,54 +1571,54 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TLG Thành Long</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>61250</v>
+        <v>23000</v>
       </c>
       <c r="G14" t="n">
-        <v>61250</v>
+        <v>31000</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>34.78</v>
       </c>
       <c r="J14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>61250</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1628,113 +1628,113 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá tăng 8,000đ (+34.8%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>192985737</t>
+          <t>66095198</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Móc Cài Tai Silicon Siêu Dẻo, Giúp Giữ Gọng Kính Không Bị Tuột Khi Chạy, Nhảy, Chơi Thể Thao, Màu Đen, Trong Suốt</t>
+          <t>Áo phông cổ tim ALIGRO ALGAPC051</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/moc-cai-tai-silicon-sieu-deo-giup-giu-gong-kinh-khong-bi-tuot-khi-chay-nhay-choi-the-thao-mau-den-trong-suot-p192985737.html?spid=192985738</t>
+          <t>https://tiki.vn/ao-phong-co-tim-aligro-algapc051-p66095198.html?spid=66095200</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Blue Light</t>
+          <t>Aligro</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>10000</v>
+        <v>150000</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Bán thêm +6 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>140429170</t>
+          <t>277600025</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bao tay chơi game găng tay 2 ngón cảm ứng điện thoại gamemobile BT01</t>
+          <t>Áo Polo Nam Công Sở Đẹp, Sang Trọng | Hàng Hiệu Cao Cấp PLN05</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bao-tay-choi-game-gang-tay-2-ngon-cam-ung-dien-thoai-gamemobile-bt01-p140429170.html?spid=198934954</t>
+          <t>https://tiki.vn/ao-polo-nam-cong-so-dep-sang-trong-hang-hieu-cao-cap-pln05-p277600025.html?spid=277600091</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1743,10 +1743,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>9999</v>
+        <v>270000</v>
       </c>
       <c r="G16" t="n">
-        <v>9999</v>
+        <v>270000</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1755,38 +1755,38 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O16" t="n">
+        <v>5</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
         <v>1</v>
       </c>
-      <c r="M16" t="n">
-        <v>9999</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1796,29 +1796,29 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>278021672</t>
+          <t>244298960</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Quần Lót Nam Đùi Boxer Lụa Băng Menpro MP9 - Mỏng nhem Thoáng Khí</t>
+          <t>Quần Mặc Váy Su Thông Hơi Trơn 6530 | Mát Mẻ, Không Lộ, Chống Hớ Hiệu Quả</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nam-dui-boxer-lua-bang-menpro-mp9-mong-nhem-thoang-khi-p278021672.html?spid=278021702</t>
+          <t>https://tiki.vn/quan-vay-dai-thong-hoi-6530-p244298960.html?spid=244298972</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1827,16 +1827,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>63200</v>
+        <v>42000</v>
       </c>
       <c r="G17" t="n">
-        <v>79000</v>
+        <v>35280</v>
       </c>
       <c r="H17" t="n">
-        <v>15800</v>
+        <v>-6720</v>
       </c>
       <c r="I17" t="n">
-        <v>25</v>
+        <v>-16</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1880,53 +1880,53 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá tăng 15,800đ (+25.0%)</t>
+          <t>Giá giảm 6,720đ (16.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2212215</t>
+          <t>104791604</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Combo 04 quần lót nam Pro Ben bảng nhỏ MS914</t>
+          <t>Quần lót nữ thái lan 828 – Chất thun lạnh - giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-04-quan-lot-nam-pro-ben-bang-nho-ms914-p2212215.html?spid=53788047</t>
+          <t>https://tiki.vn/quan-lot-nu-thai-lan-828-chat-thun-lanh-giao-mau-ngau-nhien-p104791604.html?spid=270215619</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pro Ben</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>135520</v>
+        <v>44000</v>
       </c>
       <c r="G18" t="n">
-        <v>176000</v>
+        <v>33880</v>
       </c>
       <c r="H18" t="n">
-        <v>40480</v>
+        <v>-10120</v>
       </c>
       <c r="I18" t="n">
-        <v>29.87</v>
+        <v>-23</v>
       </c>
       <c r="J18" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="K18" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="O18" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1964,24 +1964,24 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá tăng 40,480đ (+29.9%)</t>
+          <t>Giá giảm 10,120đ (23.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>244297794</t>
+          <t>7078807</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Combo 5 Quần Lót Nam Thun Lạnh Lưng To Menlive ML1 – Size M–4XL, Co Giãn 4 Chiều</t>
+          <t>Bộ 10 Quần Lót Nam Chéo Nhật Bản Cao Cấp Thoáng Mát (Giao Màu Ngẫu Nhiên)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nam-thun-lanh-menlive-p244297794.html?spid=244297815</t>
+          <t>https://tiki.vn/bo-10-quan-lot-nam-cheo-nhat-ban-cao-cap-thoang-mat-giao-mau-ngau-nhien-p7078807.html?spid=67858801</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1995,22 +1995,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>190000</v>
+        <v>300300</v>
       </c>
       <c r="G19" t="n">
-        <v>159600</v>
+        <v>385000</v>
       </c>
       <c r="H19" t="n">
-        <v>-30400</v>
+        <v>84700</v>
       </c>
       <c r="I19" t="n">
-        <v>-16</v>
+        <v>28.21</v>
       </c>
       <c r="J19" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,10 +2019,10 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,29 +2048,29 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá giảm 30,400đ (16.0%)</t>
+          <t>Giá tăng 84,700đ (+28.2%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>277983818</t>
+          <t>278021672</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Áo Lót Nữ Ren Dày Cài Trước Có Gọng Nâng Ngực Belle VC02 – Combo Đa Màu, Đệm Mút 3 cm, Quyến Rũ &amp; Đỡ Đỡ</t>
+          <t>Quần Lót Nam Đùi Boxer Lụa Băng Menpro MP9 - Mỏng nhem Thoáng Khí</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-ren-day-cai-truoc-co-gong-nang-nguc-belle-vc02-combo-da-mau-dem-mut-3-cm-quyen-ru-do-do-p277983818.html?spid=277983822</t>
+          <t>https://tiki.vn/quan-lot-nam-dui-boxer-lua-bang-menpro-mp9-mong-nhem-thoang-khi-p278021672.html?spid=278021702</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2079,16 +2079,16 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>126000</v>
+        <v>79000</v>
       </c>
       <c r="G20" t="n">
-        <v>150000</v>
+        <v>63200</v>
       </c>
       <c r="H20" t="n">
-        <v>24000</v>
+        <v>-15800</v>
       </c>
       <c r="I20" t="n">
-        <v>19.05</v>
+        <v>-20</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2132,53 +2132,53 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Giá tăng 24,000đ (+19.0%)</t>
+          <t>Giá giảm 15,800đ (20.0%)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>115852451</t>
+          <t>278872546</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chai vệ sinh giày đồ da, túi ví, áo, ghế da giúp làm sạch, dưỡng ẩm chống mốc XIMO XI03</t>
+          <t>Áo thun tay ngắn nam.Fitted - ROUTINE 10F25TSS039</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-ve-sinh-giay-do-da-tui-vi-ao-ghe-da-giup-lam-sach-duong-am-chong-moc-ximo-xi03-p115852451.html?spid=262784198</t>
+          <t>https://tiki.vn/ao-thun-tay-ngan-nam-fitted-routine-10f25tss039-p278872546.html?spid=278872562</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>75000</v>
+        <v>349000</v>
       </c>
       <c r="G21" t="n">
-        <v>70000</v>
+        <v>349000</v>
       </c>
       <c r="H21" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>-6.67</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2187,26 +2187,26 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2216,50 +2216,50 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Giá giảm 5,000đ (6.7%)</t>
+          <t>Rating 0.0→5.0 (+5.00) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>277610005</t>
+          <t>195305781</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Áo Lót 3281 Không Gọng Mút Mỏng Bản 3 Móc Che Khuyết Điểm Đẹp</t>
+          <t>Combo 3 quần đùi mặc nhà - Giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-3281-khong-gong-mut-mong-ban-3-moc-che-khuyet-diem-dep-p277610005.html?spid=277610035</t>
+          <t>https://tiki.vn/combo-3-quan-dui-mac-nha-giao-mau-ngau-nhien-p195305781.html?spid=195305789</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sanny House</t>
+          <t>Novelty</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>285000</v>
       </c>
       <c r="G22" t="n">
-        <v>96000</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>96000</v>
+        <v>-285000</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -2271,16 +2271,16 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -2290,63 +2290,63 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>277969210</t>
+          <t>195304668</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Combo 5 quần lót nữ lọt khe lụa trơn Voronin Q8289 – Mềm mịn, ôm dáng</t>
+          <t>COMBO 2 QUẦN ĐÙI MẶC NHÀ - GIAO MÀU NGẪU NHIÊN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-khe-nu-bang-lua-tron-lien-mach-voronin-q8289-p277969210.html?spid=277969212</t>
+          <t>https://tiki.vn/combo-2-quan-dui-mac-nha-giao-mau-ngau-nhien-p195304668.html?spid=195304672</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Novelty</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>205800</v>
+        <v>190000</v>
       </c>
       <c r="G23" t="n">
-        <v>245000</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>39200</v>
+        <v>-190000</v>
       </c>
       <c r="I23" t="n">
-        <v>19.05</v>
+        <v>-100</v>
       </c>
       <c r="J23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -2374,34 +2374,34 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Giá tăng 39,200đ (+19.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>277919931</t>
+          <t>73862702</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Combo 5 quần lót nữ thun lạnh thông hơi Voronin 2067 – Mát mịn, co giãn 4 chiều, không hằn viền</t>
+          <t>ÁO LÓT NỮ REN MÚT DÀY 2CM DÂY TRƠN NÂNG NGỰC 024B</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nu-thun-lanh-thong-hoi-voronin-2067-mat-min-co-gian-4-chieu-khong-han-vien-p277919931.html?spid=277919932</t>
+          <t>https://tiki.vn/ao-lot-nu-ren-mut-day-2cm-day-tron-nang-nguc-024b-p73862702.html?spid=73862742</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2415,22 +2415,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>159600</v>
+        <v>143590</v>
       </c>
       <c r="G24" t="n">
-        <v>190000</v>
+        <v>173000</v>
       </c>
       <c r="H24" t="n">
-        <v>30400</v>
+        <v>29410</v>
       </c>
       <c r="I24" t="n">
-        <v>19.05</v>
+        <v>20.48</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2439,26 +2439,26 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="S24" t="n">
         <v>0</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2468,53 +2468,53 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Giá tăng 30,400đ (+19.0%)</t>
+          <t>Giá tăng 29,410đ (+20.5%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>199996713</t>
+          <t>115852451</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Quần Âu Nam Công Sở Thương Hiệu Anton Cao Cấp Xếp ly, Chỉnh Cạp Màu Nâu- QA102</t>
+          <t>Chai vệ sinh giày đồ da, túi ví, áo, ghế da giúp làm sạch, dưỡng ẩm chống mốc XIMO XI03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-au-nam-cong-so-thuong-hieu-anton-cao-cap-xep-ly-chinh-cap-mau-nau-qa102-p199996713.html?spid=199996719</t>
+          <t>https://tiki.vn/chai-ve-sinh-giay-do-da-tui-vi-ao-ghe-da-giup-lam-sach-duong-am-chong-moc-ximo-xi03-p115852451.html?spid=262784198</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SOMIANTON</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>368000</v>
+        <v>70000</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>75000</v>
       </c>
       <c r="H25" t="n">
-        <v>-368000</v>
+        <v>5000</v>
       </c>
       <c r="I25" t="n">
-        <v>-100</v>
+        <v>7.14</v>
       </c>
       <c r="J25" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2523,82 +2523,82 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="P25" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá tăng 5,000đ (+7.1%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>72136586</t>
+          <t>278092142</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Giày Tây Nam Da Bò BIGGBEN Cao Cấp GT200</t>
+          <t>Quần kiểu nữ ống rộng, chất liệu vải Đũi xước, mềm mịn, mặc mát, Quần Short nữ đẹp Nesa Shop</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-da-bo-biggben-cao-cap-gt200-p72136586.html?spid=72136606</t>
+          <t>https://tiki.vn/quan-kieu-nu-ong-rong-chat-lieu-vai-dui-xuoc-mem-min-mac-mat-quan-short-nu-dep-nesa-shop-p278092142.html?spid=278092148</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>49000</v>
       </c>
       <c r="G26" t="n">
-        <v>750000</v>
+        <v>55000</v>
       </c>
       <c r="H26" t="n">
-        <v>750000</v>
+        <v>6000</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>12.24</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -2607,82 +2607,82 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S26" t="n">
         <v>0</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 6,000đ (+12.2%)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>270246737</t>
+          <t>59462352</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Giày Tây Nam BIGGBEN Da Bò Thật Cao Cấp GT246</t>
+          <t>Áo ngực mỏng thêu hoa cài trước có gọng</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-biggben-da-bo-that-cao-cap-gt246-p270246737.html?spid=270246761</t>
+          <t>https://tiki.vn/ao-nguc-mong-theu-hoa-cai-truoc-co-gong-p59462352.html?spid=59462384</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>749000</v>
+        <v>70200</v>
       </c>
       <c r="G27" t="n">
-        <v>850000</v>
+        <v>90000</v>
       </c>
       <c r="H27" t="n">
-        <v>101000</v>
+        <v>19800</v>
       </c>
       <c r="I27" t="n">
-        <v>13.48</v>
+        <v>28.21</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2691,26 +2691,26 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="S27" t="n">
         <v>0</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2720,53 +2720,53 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Giá tăng 101,000đ (+13.5%)</t>
+          <t>Giá tăng 19,800đ (+28.2%)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>55150033</t>
+          <t>252533129</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Giày Tây Nam Da Bò BIGGBEN Cao Cấp GT187</t>
+          <t>Găng Tay Hở 2 Ngón Unisex Chống Nắng, Có Thể Sử Dụng Cảm Ứng Điện Thoại</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-da-bo-biggben-cao-cap-gt187-p55150033.html?spid=55150039</t>
+          <t>https://tiki.vn/gang-tay-ho-2-ngon-unisex-chong-nang-co-the-su-dung-cam-ung-dien-thoai-p252533129.html?spid=252533130</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>649000</v>
+        <v>49000</v>
       </c>
       <c r="G28" t="n">
-        <v>750000</v>
+        <v>44000</v>
       </c>
       <c r="H28" t="n">
-        <v>101000</v>
+        <v>-5000</v>
       </c>
       <c r="I28" t="n">
-        <v>15.56</v>
+        <v>-10.2</v>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>162</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>162</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -2775,26 +2775,26 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="S28" t="n">
         <v>0</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2804,53 +2804,53 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Giá tăng 101,000đ (+15.6%)</t>
+          <t>Giá giảm 5,000đ (10.2%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>152632563</t>
+          <t>277347854</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Áo Lót Nữ Mút Mỏng Trơn Không Gọng 3281 – Nhẹ Êm, Tự Nhiên, Dễ Mặc Mỗi Ngày</t>
+          <t>Thắt lưng nữ DA BÒ THẬT - BEE GEE N8051</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-duc-kiem-bra-cao-cap-3281-big-size-p152632563.html?spid=274990712</t>
+          <t>https://tiki.vn/that-lung-nu-da-bo-that-bee-gee-n8051-p277347854.html?spid=277347856</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Bee Gee</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>99000</v>
+        <v>150000</v>
       </c>
       <c r="G29" t="n">
-        <v>82170</v>
+        <v>300000</v>
       </c>
       <c r="H29" t="n">
-        <v>-16830</v>
+        <v>150000</v>
       </c>
       <c r="I29" t="n">
-        <v>-17</v>
+        <v>100</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2888,47 +2888,47 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Giá giảm 16,830đ (17.0%)</t>
+          <t>Giá tăng 150,000đ (+100.0%)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>276945307</t>
+          <t>278851165</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Áo lót nữ Angelavic 529 – Bra thun lạnh tăm, mút liền, cài sau, không gọng, nâng đỡ thoải mái</t>
+          <t>Dép quai ngang Biti's nam (38-43)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-ao-bra-thun-lanh-tam-mut-lien-cai-sau-529-p276945307.html?spid=276945325</t>
+          <t>https://tiki.vn/dep-quai-ngang-biti-s-nam-38-43-p278851165.html?spid=278851187</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>110000</v>
+        <v>237000</v>
       </c>
       <c r="G30" t="n">
-        <v>82500</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>-27500</v>
+        <v>-237000</v>
       </c>
       <c r="I30" t="n">
-        <v>-25</v>
+        <v>-100</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -2943,16 +2943,16 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2962,63 +2962,63 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Giá giảm 27,500đ (25.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>277573177</t>
+          <t>277327053</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[Set 100 chiếc] Khẩu Trang 9A 5 Lớp Chống Nắng, Che Kín Mặt, Bảo Vệ Tia UV - HÀNG CHÍNH HÃNG MINIIN</t>
+          <t>Áo thun tay ngắn nam. Loose - RT 10S25TSS013 | ROUTINE CÀ MAU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://tiki.vn/set-100-chiec-khau-trang-9a-5-lop-chong-nang-che-kin-mat-bao-ve-tia-uv-hang-chinh-hang-miniin-p277573177.html?spid=277573179</t>
+          <t>https://tiki.vn/ao-thun-tay-ngan-nam-loose-rt-10s25tss013-routine-ca-mau-p277327053.html?spid=277327071</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MINIIN</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>65000</v>
+        <v>379000</v>
       </c>
       <c r="G31" t="n">
-        <v>65000</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>-379000</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -3030,76 +3030,76 @@
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>4</v>
+        <v>-0</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Rating 0.0→4.0 (+4.00) | Review thêm +1</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13307720</t>
+          <t>66507793</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Combo 10 Quần lót nam, sịp chéo nam xuất Nhật thời trang cao cấp</t>
+          <t>Dép Nam Da Bò BIGGBEN Cao Cấp DN260</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-10-quan-lot-nam-sip-cheo-nam-xuat-nhat-thoi-trang-cao-cap-p13307720.html?spid=53788749</t>
+          <t>https://tiki.vn/dep-nam-da-bo-biggben-cao-cap-dn260-p66507793.html?spid=66507799</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>296450</v>
+        <v>400000</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>-296450</v>
+        <v>-400000</v>
       </c>
       <c r="I32" t="n">
         <v>-100</v>
       </c>
       <c r="J32" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -3111,16 +3111,16 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>-5</v>
+        <v>-4.6</v>
       </c>
       <c r="Q32" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3147,17 +3147,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>248092080</t>
+          <t>250056510</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Giày lười nam da bò buộc dây Trường Hải màu nâu đề cao 3cm GM446N</t>
+          <t>Dép Nam Quai Ngang BIGGBEN Da Bò Thật Cao Cấp DN332</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-luoi-nam-da-bo-buoc-day-truong-hai-mau-nau-de-cao-3cm-gm446n-p248092080.html?spid=248092084</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-biggben-da-bo-that-cao-cap-dn332-p250056510.html?spid=250056524</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3167,23 +3167,23 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Trường Hải</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>749000</v>
+        <v>450000</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>-749000</v>
+        <v>-450000</v>
       </c>
       <c r="I33" t="n">
         <v>-100</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -3195,16 +3195,16 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>-5</v>
+        <v>-0</v>
       </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3231,43 +3231,43 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>278442851</t>
+          <t>260889428</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Quần Lót Nữ, Combo 6 Quần Lót Su Thạch Mát Lạnh Ngày Hè, Quần Lót Nữ Không Đường Viền - Hàng Nhập Khẩu</t>
+          <t>Khẩu Trang Chống Tia UV - Khẩu trang chống nắng che mặt UPF 50</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nu-combo-6-quan-lot-su-thach-mat-lanh-ngay-he-quan-lot-nu-khong-duong-vien-hang-nhap-khau-p278442851.html?spid=278442852</t>
+          <t>https://tiki.vn/khau-trang-chong-tia-uv-khau-trang-chong-nang-che-mat-upf-50-p260889428.html?spid=279253607</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HT SYS</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>122000</v>
+        <v>19000</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>-122000</v>
+        <v>-19000</v>
       </c>
       <c r="I34" t="n">
         <v>-100</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3315,43 +3315,43 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>278529292</t>
+          <t>78513044</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dép quai ngang Bitis xốp nam</t>
+          <t>Khăn ống cotton tube co giãn 9 kiểu dùng có video hướng dẫn  TUBE01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-quai-ngang-bitis-xop-nam-p278529292.html?spid=278529322</t>
+          <t>https://tiki.vn/khan-ong-cotton-tube-co-gian-9-kieu-dung-co-video-huong-dan-tube01-p78513044.html?spid=78518779</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>Song An Eco</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>126000</v>
+        <v>15000</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>-126000</v>
+        <v>-15000</v>
       </c>
       <c r="I35" t="n">
         <v>-100</v>
       </c>
       <c r="J35" t="n">
-        <v>377</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -3363,16 +3363,16 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>-4.6</v>
+        <v>-0</v>
       </c>
       <c r="Q35" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3399,420 +3399,168 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>270249539</t>
+          <t>193504415</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Giày Tây Nam Tăng Chiều Cao BIGGBEN Da Bò Thật Cao Cấp GT252</t>
+          <t>Combo 2 Áo thun thể thao nam MRM Active Pro thấm hút mồ hôi tốt co dãn thoải mái vận động</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-tang-chieu-cao-biggben-da-bo-that-cao-cap-gt252-p270249539.html?spid=270249555</t>
+          <t>https://tiki.vn/combo-2-ao-thun-the-thao-nam-mrm-active-pro-tham-hut-mo-hoi-tot-co-dan-thoai-mai-van-dong-p193504415.html?spid=193504423</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>MRM Manlywear</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>799000</v>
+        <v>229000</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>229000</v>
       </c>
       <c r="H36" t="n">
-        <v>-799000</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>-916000</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P36" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="R36" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Bán thêm -4 sản phẩm | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>208746104</t>
+          <t>275396535</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Giày Thể Thao Biti's Nam Hunter X DSMH10500</t>
+          <t>Bộ bơi nam quần 2 lớp trẻ trung nam tính thời trang, đồ bơi đồ tập kín đáo chống lộ, chất thoáng khí nhanh khô, áo thun bơi co giãn tốt, có size lớn | BN032</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-the-thao-biti-s-nam-hunter-x-dsmh10500-p208746104.html?spid=208746130</t>
+          <t>https://tiki.vn/bo-boi-nam-quan-2-lop-tre-trung-nam-tinh-thoi-trang-do-boi-do-tap-kin-dao-chong-lo-chat-thoang-khi-nhanh-kho-ao-thun-boi-co-gian-tot-co-size-lon-bn032-p275396535.html?spid=275396555</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1050000</v>
+        <v>310000</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>310000</v>
       </c>
       <c r="H37" t="n">
-        <v>-1050000</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
+        <v>9</v>
+      </c>
+      <c r="K37" t="n">
+        <v>6</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-930000</v>
+      </c>
+      <c r="N37" t="n">
         <v>5</v>
       </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>4</v>
-      </c>
       <c r="O37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P37" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S37" t="n">
         <v>0</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>276545723</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Dép quai kẹp Bitis nam (38-43)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-quai-kep-bitis-nam-38-43-p276545723.html?spid=276545737</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Biti's</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>92000</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>-92000</v>
-      </c>
-      <c r="I38" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J38" t="n">
-        <v>7</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="O38" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" t="n">
-        <v>-4.5</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>2</v>
-      </c>
-      <c r="R38" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>52317590</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Bộ 2 mũ lưỡi trai cho nam ( đen - trắng)</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/bo-2-mu-luoi-trai-cho-nam-den-trang-p52317590.html?spid=162171783</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>LQ luxury</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>49000</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>-49000</v>
-      </c>
-      <c r="I39" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J39" t="n">
-        <v>21</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="n">
-        <v>5</v>
-      </c>
-      <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="n">
-        <v>-5</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>1</v>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
-        <v>0</v>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>278004504</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Combo 5 Quần Lót Nữ Su Tăm Trơn Không Viền Mỏng Nhẹ 892 – Co Giãn 4 Chiều, Thoáng Mát, Không Lộ Viền (Size L/XL/XXL)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nu-su-tam-tron-khong-vien-mong-nhe-892-co-gian-4-chieu-thoang-mat-khong-lo-vien-size-l-xl-xxl-p278004504.html?spid=278004508</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>168000</v>
-      </c>
-      <c r="G40" t="n">
-        <v>230000</v>
-      </c>
-      <c r="H40" t="n">
-        <v>62000</v>
-      </c>
-      <c r="I40" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="J40" t="n">
-        <v>1</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-230000</v>
-      </c>
-      <c r="N40" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
-      <c r="S40" t="n">
-        <v>0</v>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>Giá tăng 62,000đ (+36.9%) | Bán thêm -1 sản phẩm</t>
+          <t>Bán thêm -3 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-06-29
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,17 +543,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>73214429</t>
+          <t>67538621</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Áo Khoác Nam Áo Khoác Dù Nam Nữ Hai Lớp Chống Nước Chống Nắng Chống Gió Phối Nón Cao Cấp QD54 - ShopN6 (Nhiều Màu)</t>
+          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-khoac-nam-ao-khoac-du-nam-nu-hai-lop-chong-nuoc-chong-nang-chong-gio-phoi-non-cao-cap-qd54-shopn6-nhieu-mau-p73214429.html?spid=73214433</t>
+          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538623</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -563,81 +563,81 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>N6</t>
+          <t>May 10</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>135000</v>
       </c>
       <c r="G2" t="n">
-        <v>189000</v>
+        <v>135000</v>
       </c>
       <c r="H2" t="n">
-        <v>189000</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>16583</v>
       </c>
       <c r="K2" t="n">
-        <v>442</v>
+        <v>16599</v>
       </c>
       <c r="L2" t="n">
-        <v>442</v>
+        <v>16</v>
       </c>
       <c r="M2" t="n">
-        <v>83538000</v>
+        <v>2160000</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="O2" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="P2" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="R2" t="n">
-        <v>181</v>
+        <v>4842</v>
       </c>
       <c r="S2" t="n">
-        <v>181</v>
+        <v>0</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +16 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>134757898</t>
+          <t>263276725</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Giày da nam, giày oxford công sở Bụi Leather G106 - Da bò Nappa cao cấp - Bảo hành 12 tháng</t>
+          <t>Chuck Taylor Classic Black Canvas Low | Giày Thể Thao Đen Cổ Thấp M9166C</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-da-nam-giay-oxford-cong-so-bui-leather-g106-da-bo-nappa-cao-cap-bao-hanh-12-thang-p134757898.html?spid=134757930</t>
+          <t>https://tiki.vn/chuck-taylor-classic-black-giay-the-thao-den-co-thap-p263276725.html?spid=263276727</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bụi Leather</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>865000</v>
+        <v>1600000</v>
       </c>
       <c r="H3" t="n">
-        <v>865000</v>
+        <v>1600000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,35 +666,35 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>61415000</v>
+        <v>1600000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="P3" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>136093004</t>
+          <t>275396535</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Áo thun may ô ngắn tay (áo đông xuân) nam</t>
+          <t>Bộ bơi nam quần 2 lớp trẻ trung nam tính thời trang, đồ bơi đồ tập kín đáo chống lộ, chất thoáng khí nhanh khô, áo thun bơi co giãn tốt, có size lớn | BN032</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-may-o-ngan-tay-ao-dong-xuan-nam-p136093004.html?spid=136093008</t>
+          <t>https://tiki.vn/bo-boi-nam-quan-2-lop-tre-trung-nam-tinh-thoi-trang-do-boi-do-tap-kin-dao-chong-lo-chat-thoang-khi-nhanh-kho-ao-thun-boi-co-gian-tot-co-size-lon-bn032-p275396535.html?spid=275396553</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -731,14 +731,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">	OEM</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>69000</v>
+        <v>310000</v>
       </c>
       <c r="G4" t="n">
-        <v>69000</v>
+        <v>310000</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -747,16 +747,16 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>232</v>
+        <v>12</v>
       </c>
       <c r="K4" t="n">
-        <v>258</v>
+        <v>17</v>
       </c>
       <c r="L4" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="M4" t="n">
-        <v>1794000</v>
+        <v>1550000</v>
       </c>
       <c r="N4" t="n">
         <v>5</v>
@@ -768,17 +768,17 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="R4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -788,128 +788,128 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Bán thêm +26 sản phẩm</t>
+          <t>Bán thêm +5 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>174437687</t>
+          <t>277468360</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dép nhựa Bitis nam</t>
+          <t>Mũ Trùm Đầu Chống Nắng Kèm Khẩu Trang Nam Nữ - Nón Che Nắng Chống Tia UV Có Dây Rút</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nhua-bitis-nam-p174437687.html?spid=174437691</t>
+          <t>https://tiki.vn/mu-trum-dau-chong-nang-kem-khau-trang-nam-nu-non-che-nang-chong-tia-uv-co-day-rut-p277468360.html?spid=277468368</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>90000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>105000</v>
+        <v>153000</v>
       </c>
       <c r="H5" t="n">
-        <v>15000</v>
+        <v>153000</v>
       </c>
       <c r="I5" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="M5" t="n">
-        <v>1680000</v>
+        <v>612000</v>
       </c>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
         <v>5</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q5" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Giá tăng 15,000đ (+16.7%) | Bán thêm +16 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>147249168</t>
+          <t>162562752</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dép Nam Quai Ngang HÀ NAM Da Bò Thật Cao Cấp DNA2158</t>
+          <t>Combo 10 quần lót nữ chất liệu cotton chất đẹp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-ha-nam-cao-cap-dna2158-p147249168.html?spid=147249212</t>
+          <t>https://tiki.vn/combo-10-quan-lot-nu-chat-lieu-cotton-chat-dep-p162562752.html?spid=162562761</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HA NAM</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>372000</v>
+        <v>150000</v>
       </c>
       <c r="H6" t="n">
-        <v>372000</v>
+        <v>150000</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -918,13 +918,13 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" t="n">
-        <v>372000</v>
+        <v>300000</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -946,7 +946,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -963,22 +963,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23452446</t>
+          <t>279279665</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Áo Khoác kaki nam</t>
+          <t>Hộp đựng thuốc 20Đ dài slim Foucs YH061</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-khoac-kaki-nam-p23452446.html?spid=113226723</t>
+          <t>https://tiki.vn/hop-dung-thuoc-20d-dai-slim-foucs-yh061-p279279665.html?spid=279279667</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -990,10 +990,10 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>331000</v>
+        <v>99000</v>
       </c>
       <c r="H7" t="n">
-        <v>331000</v>
+        <v>99000</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1002,13 +1002,13 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>331000</v>
+        <v>198000</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1047,34 +1047,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>808362</t>
+          <t>275276422</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bộ 5 Đôi Vớ Nam Modal Công Sở Sọc Đen Donakein 7MM5D5M02</t>
+          <t>Dép tổ ong XANH NGỌC nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-5-doi-vo-nam-modal-cong-so-soc-den-donakein-7mm5d5m02-p808362.html?spid=811320</t>
+          <t>https://tiki.vn/dep-to-ong-xanh-ngoc-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276422.html?spid=275276436</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Donakein</t>
+          <t xml:space="preserve">VAC </t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>199000</v>
+        <v>72000</v>
       </c>
       <c r="G8" t="n">
-        <v>199000</v>
+        <v>72000</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1083,16 +1083,16 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="K8" t="n">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" t="n">
-        <v>199000</v>
+        <v>144000</v>
       </c>
       <c r="N8" t="n">
         <v>5</v>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1124,128 +1124,128 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Bán thêm +2 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>262052731</t>
+          <t>34159085</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Áo thun nam thể thao DO GYM SHOP form ôm body, thun lạnh 4 chiều không xù lông</t>
+          <t>Combo 5 Đôi Tất Cổ Trung Cùng Màu Cotton Thương Hiệu MRM Manlywear</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-nam-the-thao-do-gym-shop-form-om-body-thun-lanh-4-chieu-khong-xu-long-p262052731.html?spid=267343581</t>
+          <t>https://tiki.vn/combo-5-doi-tat-nam-tat-nam-vo-nam-co-dai-cao-cap-mrm-fashion-cung-mau-p34159085.html?spid=34159089</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MRM Manlywear</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>135000</v>
       </c>
       <c r="G9" t="n">
-        <v>159000</v>
+        <v>135000</v>
       </c>
       <c r="H9" t="n">
-        <v>159000</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>4716</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>4717</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>159000</v>
+        <v>135000</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>225209462</t>
+          <t>51299947</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MŨ CHỐNG NẮNG CÓI NỬA ĐẦU RỘNG VÀNH CÁ TÍNH CHO NỮ</t>
+          <t>Áo Sơ Mi Caro TitiShop SM1164 ( Luxury)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mu-chong-nang-coi-nua-dau-rong-vanh-ca-tinh-cho-nu-p225209462.html?spid=247940496</t>
+          <t>https://tiki.vn/ao-so-mi-caro-titishop-sm1164-luxury-p51299947.html?spid=51299949</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Titishop</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>55000</v>
+        <v>79000</v>
       </c>
       <c r="H10" t="n">
-        <v>55000</v>
+        <v>79000</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1254,35 +1254,35 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>110000</v>
+        <v>79000</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1299,17 +1299,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>252533129</t>
+          <t>271973646</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Găng Tay Hở 2 Ngón Unisex Chống Nắng, Có Thể Sử Dụng Cảm Ứng Điện Thoại</t>
+          <t>Miếng dán hình xăm kinh dị hóa trang Halloween vết sẹo xước máu giả vết khâu chảy máu vết thương Legaxi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/gang-tay-ho-2-ngon-unisex-chong-nang-co-the-su-dung-cam-ung-dien-thoai-p252533129.html?spid=252533130</t>
+          <t>https://tiki.vn/mieng-dan-hinh-xam-kinh-di-hoa-trang-halloween-vet-seo-xuoc-mau-gia-vet-khau-chay-mau-vet-thuong-legaxi-p271973646.html?spid=271973648</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1319,14 +1319,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Legaxi</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>49000</v>
+        <v>25000</v>
       </c>
       <c r="G11" t="n">
-        <v>49000</v>
+        <v>25000</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1335,16 +1335,16 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>162</v>
+        <v>5</v>
       </c>
       <c r="K11" t="n">
-        <v>164</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>98000</v>
+        <v>25000</v>
       </c>
       <c r="N11" t="n">
         <v>5</v>
@@ -1356,17 +1356,17 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Bán thêm +2 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>214504425</t>
+          <t>279296102</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Chai Xịt Tạo Bọt Vệ Sinh Giày XIMO Cao Cấp 300ml XVSG02</t>
+          <t>[NEW ARRIVAL] Giày Sneaker Nam Nữ DC48 SHADOW MOVE Dincox Shoes Đế Bằng - Da phối Suede Cao Cấp</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-xit-tao-bot-ve-sinh-giay-ximo-cao-cap-300ml-xvsg02-p214504425.html?spid=252869350</t>
+          <t>https://tiki.vn/new-arrival-giay-sneaker-nam-nu-dc48-shadow-move-dincox-shoes-de-bang-da-phoi-suede-cao-cap-p279296102.html?spid=279296104</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1403,81 +1403,81 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>DINCOX</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>72000</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>72000</v>
+        <v>650000</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>650000</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>338</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>72000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>112851354</t>
+          <t>276945307</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Áo ngực học sinh</t>
+          <t>Áo lót nữ Angelavic 529 – Bra thun lạnh tăm, mút liền, cài sau, không gọng, nâng đỡ thoải mái</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138792</t>
+          <t>https://tiki.vn/ao-lot-nu-ao-bra-thun-lanh-tam-mut-lien-cai-sau-529-p276945307.html?spid=276945325</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1491,22 +1491,22 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>40000</v>
+        <v>82500</v>
       </c>
       <c r="G13" t="n">
-        <v>30400</v>
+        <v>110000</v>
       </c>
       <c r="H13" t="n">
-        <v>-9600</v>
+        <v>27500</v>
       </c>
       <c r="I13" t="n">
-        <v>-24</v>
+        <v>33.33</v>
       </c>
       <c r="J13" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1515,26 +1515,26 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,53 +1544,53 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Giá giảm 9,600đ (24.0%)</t>
+          <t>Giá tăng 27,500đ (+33.3%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>277718250</t>
+          <t>244297794</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Giày Sandal nam cao cấp kiểu dáng mới – GSDNA10</t>
+          <t>Combo 5 Quần Lót Nam Thun Lạnh Lưng To Menlive ML1 – Size M–4XL, Co Giãn 4 Chiều</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-sandal-nam-cao-cap-kieu-dang-moi-gsdna10-p277718250.html?spid=277718278</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-thun-lanh-menlive-p244297794.html?spid=244297815</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bee Gee</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>159600</v>
       </c>
       <c r="G14" t="n">
-        <v>583440</v>
+        <v>190000</v>
       </c>
       <c r="H14" t="n">
-        <v>583440</v>
+        <v>30400</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1599,53 +1599,53 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 30,400đ (+19.0%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>279013580</t>
+          <t>72881856</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Áo sweater thu đông form rộng in hình hài hước "Mập rõ chứ không mập mờ" Mr.buffalo - [HN11] Áo Trắng</t>
+          <t>Quần lót nam thun lạnh không đường may, sịp đùi nam cao cấp kiểu dáng boxer nam ôm sát, chất liệu su thoáng mát, mềm mịn và mỏng nhẹ, quần lót cạp nhỏ đơn giản với màu trơn QLW806</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-sweater-thu-dong-form-rong-in-hinh-hai-huoc-map-ro-chu-khong-map-mo-mr-buffalo-p279013580.html?spid=279013592</t>
+          <t>https://tiki.vn/quan-lot-nam-thun-lanh-khong-duong-may-sip-dui-nam-cao-cap-kieu-dang-boxer-nam-om-sat-chat-lieu-su-thoang-mat-mem-min-va-mong-nhe-quan-lot-cap-nho-don-gian-voi-mau-tron-qlw806-p72881856.html?spid=102551187</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1659,22 +1659,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>160000</v>
+        <v>69000</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>69000</v>
       </c>
       <c r="H15" t="n">
-        <v>-160000</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1683,82 +1683,82 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P15" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>113145806</t>
+          <t>51297510</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
+          <t>Áo Sơ Mi Caro TitiShop SM1161 ( Luxury)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
+          <t>https://tiki.vn/ao-so-mi-caro-titishop-sm1161-luxury-p51297510.html?spid=51297512</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Titishop</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>117000</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>88920</v>
+        <v>79000</v>
       </c>
       <c r="H16" t="n">
-        <v>-28080</v>
+        <v>79000</v>
       </c>
       <c r="I16" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -1767,82 +1767,82 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Giá giảm 28,080đ (24.0%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>107802069</t>
+          <t>136093004</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
+          <t>Áo thun may ô ngắn tay (áo đông xuân) nam</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
+          <t>https://tiki.vn/ao-thun-may-o-ngan-tay-ao-dong-xuan-nam-p136093004.html?spid=136093008</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t xml:space="preserve">	OEM</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>26000</v>
+        <v>69000</v>
       </c>
       <c r="G17" t="n">
-        <v>42000</v>
+        <v>89000</v>
       </c>
       <c r="H17" t="n">
-        <v>16000</v>
+        <v>20000</v>
       </c>
       <c r="I17" t="n">
-        <v>61.54</v>
+        <v>28.99</v>
       </c>
       <c r="J17" t="n">
-        <v>1033</v>
+        <v>258</v>
       </c>
       <c r="K17" t="n">
-        <v>1033</v>
+        <v>258</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,26 +1851,26 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O17" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="R17" t="n">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1880,53 +1880,53 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá tăng 16,000đ (+61.5%)</t>
+          <t>Giá tăng 20,000đ (+29.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>278004504</t>
+          <t>277420779</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Combo 5 Quần Lót Nữ Su Tăm Trơn Không Viền Mỏng Nhẹ 892 – Co Giãn 4 Chiều, Thoáng Mát, Không Lộ Viền (Size L/XL/XXL)</t>
+          <t>Khẩu Trang Chống Nắng Cao Cấp UPF 50+,Khẩu Trang Chống Nám Chống Tia UV, Bảo Vệ Da Hiệu Quả - HÀNG CHÍNH HÃNG MINIIN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nu-su-tam-tron-khong-vien-mong-nhe-892-co-gian-4-chieu-thoang-mat-khong-lo-vien-size-l-xl-xxl-p278004504.html?spid=278004508</t>
+          <t>https://tiki.vn/khau-trang-chong-nang-enaide-cao-cap-upf-50-chong-tia-uv-bao-ve-da-hieu-qua-hang-chinh-hang-miniin-p277420779.html?spid=277420793</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MINIIN</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>230000</v>
+        <v>55000</v>
       </c>
       <c r="G18" t="n">
-        <v>188600</v>
+        <v>27000</v>
       </c>
       <c r="H18" t="n">
-        <v>-41400</v>
+        <v>-28000</v>
       </c>
       <c r="I18" t="n">
-        <v>-18</v>
+        <v>-50.91</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1964,29 +1964,29 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá giảm 41,400đ (18.0%)</t>
+          <t>Giá giảm 28,000đ (50.9%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>113144956</t>
+          <t>279100044</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>siêu phẩm áo lót nhật trơn đệm nâng ngực nhẹ</t>
+          <t>Chai Xịt Khử Mùi Giày Dép 260ML</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/sieu-pham-ao-lot-tron-dem-nang-nguc-nhe-p113144956.html?spid=142116876</t>
+          <t>https://tiki.vn/chai-xit-khu-mui-giay-dep-260ml-p279100044.html?spid=279100045</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1995,22 +1995,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>165000</v>
+        <v>48000</v>
       </c>
       <c r="G19" t="n">
-        <v>123750</v>
+        <v>59000</v>
       </c>
       <c r="H19" t="n">
-        <v>-41250</v>
+        <v>11000</v>
       </c>
       <c r="I19" t="n">
-        <v>-25</v>
+        <v>22.92</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,26 +2019,26 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,41 +2048,41 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá giảm 41,250đ (25.0%)</t>
+          <t>Giá tăng 11,000đ (+22.9%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31638135</t>
+          <t>112814658</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Combo 4 quần lót nam Boxer sợi cạp 1cm sợi tre tự nhiên mềm mịn thấm hút mồ hôi, co giãn 4 chiều MRM Manlywear - Màu ngẫu nhiên</t>
+          <t>Thắt Lưng Nam Dây Vải Dù Phong Cách Lính U379 US ARMY, Khóa Cài Tự Động Dễ Dàng Điều Chỉnh Theo Vòng Bụng- HÀNG CHÍNH HÃNG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-4-quan-sip-dui-nam-quan-lot-nam-boxer-soi-tre-mem-min-sieu-thoang-mat-co-gian-4-chieu-cao-cap-cap-1cm-mrm-fashion-3-mau-p31638135.html?spid=31638146</t>
+          <t>https://tiki.vn/that-lung-nam-day-vai-du-phong-cach-linh-u379-us-army-khoa-cai-tu-dong-de-dang-dieu-chinh-theo-vong-bung-hang-chinh-hang-p112814658.html?spid=174134932</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>US ARMY</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>255000</v>
+        <v>99000</v>
       </c>
       <c r="G20" t="n">
-        <v>255000</v>
+        <v>99000</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -2091,10 +2091,10 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>5855</v>
+        <v>75</v>
       </c>
       <c r="K20" t="n">
-        <v>5855</v>
+        <v>75</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -2103,26 +2103,26 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="O20" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>1371</v>
+        <v>28</v>
       </c>
       <c r="R20" t="n">
-        <v>1372</v>
+        <v>29</v>
       </c>
       <c r="S20" t="n">
         <v>1</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2139,22 +2139,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>279100044</t>
+          <t>276146188</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chai Xịt Khử Mùi Giày Dép 260ML</t>
+          <t>Combo đồ bơi nam quần 2 lớp kèm kính mũ bơi, túi đựng đồ và bịt tai kẹp mũi, set bơi đầy đủ tiện lợi cho nam giới, quần bơi 2 lớp &amp; kính chống đọng sương | BN032</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-xit-khu-mui-giay-dep-260ml-p279100044.html?spid=279100045</t>
+          <t>https://tiki.vn/combo-do-boi-nam-quan-2-lop-kem-kinh-mu-boi-tui-dung-do-va-bit-tai-kep-mui-set-boi-day-du-tien-loi-cho-nam-gioi-quan-boi-2-lop-kinh-chong-dong-suong-bn032-p276146188.html?spid=276146212</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2163,22 +2163,22 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>59000</v>
+        <v>350000</v>
       </c>
       <c r="G21" t="n">
-        <v>48000</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>-11000</v>
+        <v>-350000</v>
       </c>
       <c r="I21" t="n">
-        <v>-18.64</v>
+        <v>-100</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
@@ -2206,54 +2206,54 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Giá giảm 11,000đ (18.6%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>279295872</t>
+          <t>75728341</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Giày Da Sneaker Nam Nữ DC39 Oreo Dincox Shoes Đế Bằng - Microfiber Leather</t>
+          <t>Áo Sơ Mi Nam Titishop SM1281</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-da-sneaker-nam-nu-dc39-oreo-dincox-shoes-de-bang-microfiber-leather-p279295872.html?spid=279295884</t>
+          <t>https://tiki.vn/ao-so-mi-nam-titishop-sm1281-p75728341.html?spid=75728349</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DINCOX</t>
+          <t>Titishop</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>660000</v>
+        <v>59000</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>-660000</v>
+        <v>-59000</v>
       </c>
       <c r="I22" t="n">
         <v>-100</v>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2307,43 +2307,43 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>276561845</t>
+          <t>152632563</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Giày thể thao Bitis hunter nam (40-45)</t>
+          <t>Áo Lót Nữ Mút Mỏng Trơn Không Gọng 3281 – Nhẹ Êm, Tự Nhiên, Dễ Mặc Mỗi Ngày</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-the-thao-bitis-hunter-nam-40-45-p276561845.html?spid=276561867</t>
+          <t>https://tiki.vn/ao-lot-duc-kiem-bra-cao-cap-3281-big-size-p152632563.html?spid=274990712</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>869000</v>
+        <v>82170</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>-869000</v>
+        <v>-82170</v>
       </c>
       <c r="I23" t="n">
         <v>-100</v>
       </c>
       <c r="J23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -2355,16 +2355,16 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>-5</v>
+        <v>-0</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2391,43 +2391,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>160418420</t>
+          <t>163806087</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ÁO CHỐNG NẮNG NAM THÔNG HƠI VẢI KIM CƯƠNG</t>
+          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-chong-nang-nam-thong-hoi-vai-kim-cuong-p160418420.html?spid=174620121</t>
+          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-p163806087.html?spid=253461440</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>165000</v>
+        <v>59000</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>-165000</v>
+        <v>-59000</v>
       </c>
       <c r="I24" t="n">
         <v>-100</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -2439,16 +2439,16 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2475,17 +2475,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>279149590</t>
+          <t>273550361</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Keo Dán Sửa Chữa Giày Siêu Chắc Shoe Glue Plr80 60Ml Đa Năng</t>
+          <t>Lót giày sức khỏe cho chân vòm cao Spenco Ground Control High Arch ôm sát vòm chân</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-sua-chua-giay-sieu-chac-shoe-glue-plr80-60ml-da-nang-p279149590.html?spid=279149591</t>
+          <t>https://tiki.vn/lot-giay-y-khoa-spenco-ground-control-high-arch-p273550361.html?spid=273550365</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2495,23 +2495,23 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Spenco</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>49000</v>
+        <v>895000</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>-49000</v>
+        <v>-895000</v>
       </c>
       <c r="I25" t="n">
         <v>-100</v>
       </c>
       <c r="J25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -2523,16 +2523,16 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>-5</v>
+        <v>-0</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2559,43 +2559,43 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>277342816</t>
+          <t>273097909</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Áo thun tay ngắn nam. Regular - RT 10F24TSS070R1 | ROUTINE CÀ MAU</t>
+          <t>Tròng kính cận/viễn/loạn mỏng 1.60 chemi đổi màu thời trang OURESS</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-tay-ngan-nam-regular-rt-10f24tss070r1-routine-ca-mau-p277342816.html?spid=277342840</t>
+          <t>https://tiki.vn/trong-kinh-can-vien-loan-mong-1-60-chemi-doi-mau-thoi-trang-ouress-p273097909.html?spid=273097910</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Routine</t>
+          <t>OURESS</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>349000</v>
+        <v>1100000</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>-349000</v>
+        <v>-1100000</v>
       </c>
       <c r="I26" t="n">
         <v>-100</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2643,17 +2643,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16212451</t>
+          <t>225209462</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Combo 6 Quần tất da nữ siêu dai và mịn</t>
+          <t>MŨ CHỐNG NẮNG CÓI NỬA ĐẦU RỘNG VÀNH CÁ TÍNH CHO NỮ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-6-quan-tat-da-nu-sieu-dai-va-min-p16212451.html?spid=44145983</t>
+          <t>https://tiki.vn/mu-chong-nang-coi-nua-dau-rong-vanh-ca-tinh-cho-nu-p225209462.html?spid=247940496</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2663,23 +2663,23 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TOMAN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>144000</v>
+        <v>55000</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>-144000</v>
+        <v>-55000</v>
       </c>
       <c r="I27" t="n">
         <v>-100</v>
       </c>
       <c r="J27" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -2691,16 +2691,16 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="Q27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2721,174 +2721,6 @@
       <c r="V27" t="inlineStr">
         <is>
           <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>275276334</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Dép tổ ong XÁM nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-to-ong-xam-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276334.html?spid=275276350</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VAC </t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>72000</v>
-      </c>
-      <c r="G28" t="n">
-        <v>72000</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>87</v>
-      </c>
-      <c r="K28" t="n">
-        <v>85</v>
-      </c>
-      <c r="L28" t="n">
-        <v>-2</v>
-      </c>
-      <c r="M28" t="n">
-        <v>-144000</v>
-      </c>
-      <c r="N28" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O28" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>4</v>
-      </c>
-      <c r="R28" t="n">
-        <v>4</v>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Bán thêm -2 sản phẩm</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>274937386</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Bộ bơi nữ big size cao cấp, mẫu 2 mảnh áo cộc tay có khóa kéo trước, quần boxer trẻ trung, chất thun bơi lạnh Lycra co giãn đa chiều, dày dặn mịn mát, chống thấm nước nhanh khô | KT110</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/bo-boi-nu-big-size-cao-cap-mau-2-manh-ao-coc-tay-co-khoa-keo-truoc-quan-boxer-tre-trung-chat-thun-boi-lanh-lycra-co-gian-da-chieu-day-dan-min-mat-chong-tham-nuoc-nhanh-kho-kt110-p274937386.html?spid=274937410</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>480000</v>
-      </c>
-      <c r="G29" t="n">
-        <v>480000</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="n">
-        <v>12</v>
-      </c>
-      <c r="K29" t="n">
-        <v>9</v>
-      </c>
-      <c r="L29" t="n">
-        <v>-3</v>
-      </c>
-      <c r="M29" t="n">
-        <v>-1440000</v>
-      </c>
-      <c r="N29" t="n">
-        <v>5</v>
-      </c>
-      <c r="O29" t="n">
-        <v>5</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>1</v>
-      </c>
-      <c r="R29" t="n">
-        <v>1</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Bán thêm -3 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-06-30
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -543,185 +543,185 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>67538621</t>
+          <t>24030500</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
+          <t>Bộ 5 quần lót nữ basic Comfort Modal MILEY LINGERIE - Màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538623</t>
+          <t>https://tiki.vn/bo-5-quan-lot-nu-basic-comfort-modal-miley-lingerie-mau-ngau-nhien-p24030500.html?spid=24030504</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>May 10</t>
+          <t>Miley Lingerie</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>135000</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>135000</v>
+        <v>320000</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>320000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>16583</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>16599</v>
+        <v>72</v>
       </c>
       <c r="L2" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="M2" t="n">
-        <v>2160000</v>
+        <v>23040000</v>
       </c>
       <c r="N2" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>4842</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>4842</v>
+        <v>12</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Bán thêm +16 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>263276725</t>
+          <t>277573177</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chuck Taylor Classic Black Canvas Low | Giày Thể Thao Đen Cổ Thấp M9166C</t>
+          <t>[Set 100 chiếc] Khẩu Trang 9A 5 Lớp Chống Nắng, Che Kín Mặt, Bảo Vệ Tia UV - HÀNG CHÍNH HÃNG MINIIN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chuck-taylor-classic-black-giay-the-thao-den-co-thap-p263276725.html?spid=263276727</t>
+          <t>https://tiki.vn/set-100-chiec-khau-trang-9a-5-lop-chong-nang-che-kin-mat-bao-ve-tia-uv-hang-chinh-hang-miniin-p277573177.html?spid=277573181</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>MINIIN</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>65000</v>
       </c>
       <c r="G3" t="n">
-        <v>1600000</v>
+        <v>59000</v>
       </c>
       <c r="H3" t="n">
-        <v>1600000</v>
+        <v>-6000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>-9.23</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K3" t="n">
+        <v>21</v>
+      </c>
+      <c r="L3" t="n">
+        <v>16</v>
+      </c>
+      <c r="M3" t="n">
+        <v>944000</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
         <v>1</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>5</v>
-      </c>
-      <c r="P3" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 6,000đ (9.2%) | Bán thêm +16 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>275396535</t>
+          <t>14351068</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bộ bơi nam quần 2 lớp trẻ trung nam tính thời trang, đồ bơi đồ tập kín đáo chống lộ, chất thoáng khí nhanh khô, áo thun bơi co giãn tốt, có size lớn | BN032</t>
+          <t>Áo thun Nam có cổ thời trang</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-boi-nam-quan-2-lop-tre-trung-nam-tinh-thoi-trang-do-boi-do-tap-kin-dao-chong-lo-chat-thoang-khi-nhanh-kho-ao-thun-boi-co-gian-tot-co-size-lon-bn032-p275396535.html?spid=275396553</t>
+          <t>https://tiki.vn/ao-thun-nam-co-co-thoi-trang-p14351068.html?spid=14351092</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -735,10 +735,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>310000</v>
+        <v>160000</v>
       </c>
       <c r="G4" t="n">
-        <v>310000</v>
+        <v>160000</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -747,38 +747,38 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" t="n">
+        <v>640000</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="O4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" t="n">
-        <v>1550000</v>
-      </c>
-      <c r="N4" t="n">
+      <c r="R4" t="n">
         <v>5</v>
       </c>
-      <c r="O4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R4" t="n">
-        <v>2</v>
-      </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -788,29 +788,29 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Bán thêm +5 sản phẩm</t>
+          <t>Bán thêm +4 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>277468360</t>
+          <t>244297794</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mũ Trùm Đầu Chống Nắng Kèm Khẩu Trang Nam Nữ - Nón Che Nắng Chống Tia UV Có Dây Rút</t>
+          <t>Combo 5 Quần Lót Nam Thun Lạnh Lưng To Menlive ML1 – Size M–4XL, Co Giãn 4 Chiều</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mu-trum-dau-chong-nang-kem-khau-trang-nam-nu-non-che-nang-chong-tia-uv-co-day-rut-p277468360.html?spid=277468368</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-thun-lanh-menlive-p244297794.html?spid=244297815</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -819,82 +819,82 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>190000</v>
       </c>
       <c r="G5" t="n">
-        <v>153000</v>
+        <v>148200</v>
       </c>
       <c r="H5" t="n">
-        <v>153000</v>
+        <v>-41800</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>-22</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>612000</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O5" t="n">
         <v>5</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 41,800đ (22.0%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>162562752</t>
+          <t>16375016</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Combo 10 quần lót nữ chất liệu cotton chất đẹp</t>
+          <t>COMBO HỘP 5 Quần Lót ĐÙI Nam Xuất Nhật Cao Cấp (MIX NGẪU NHIÊN)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-10-quan-lot-nu-chat-lieu-cotton-chat-dep-p162562752.html?spid=162562761</t>
+          <t>https://tiki.vn/combo-hop-5-quan-lot-dui-nam-xuat-nhat-cao-cap-mix-ngau-nhien-p16375016.html?spid=277961877</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -903,28 +903,28 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>251000</v>
       </c>
       <c r="G6" t="n">
-        <v>150000</v>
+        <v>198290</v>
       </c>
       <c r="H6" t="n">
-        <v>150000</v>
+        <v>-52710</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -946,39 +946,39 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 52,710đ (21.0%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>279279665</t>
+          <t>277919931</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hộp đựng thuốc 20Đ dài slim Foucs YH061</t>
+          <t>Combo 5 quần lót nữ thun lạnh thông hơi Voronin 2067 – Mát mịn, co giãn 4 chiều, không hằn viền</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-dung-thuoc-20d-dai-slim-foucs-yh061-p279279665.html?spid=279279667</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nu-thun-lanh-thong-hoi-voronin-2067-mat-min-co-gian-4-chieu-khong-han-vien-p277919931.html?spid=277919932</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -987,134 +987,134 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>190000</v>
       </c>
       <c r="G7" t="n">
-        <v>99000</v>
+        <v>150100</v>
       </c>
       <c r="H7" t="n">
-        <v>99000</v>
+        <v>-39900</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
         <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>198000</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 39,900đ (21.0%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>275276422</t>
+          <t>74421501</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dép tổ ong XANH NGỌC nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>ÁO LÓT NỮ MỎNG CÓ GỌNG CÀI TRƯỚC VIỀN REN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-xanh-ngoc-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276422.html?spid=275276436</t>
+          <t>https://tiki.vn/ao-lot-nu-mong-co-gong-cai-truoc-vien-ren-p74421501.html?spid=74421553</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>72000</v>
+        <v>118500</v>
       </c>
       <c r="G8" t="n">
-        <v>72000</v>
+        <v>160000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>41500</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>35.02</v>
       </c>
       <c r="J8" t="n">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="K8" t="n">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>144000</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O8" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="R8" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1124,81 +1124,81 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +2 sản phẩm</t>
+          <t>Giá tăng 41,500đ (+35.0%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>34159085</t>
+          <t>244298352</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combo 5 Đôi Tất Cổ Trung Cùng Màu Cotton Thương Hiệu MRM Manlywear</t>
+          <t>Quần Gen Ôm Bụng Dạng Đùi Có Thanh Chống Cuộn Voronin 8292 – Siêu Gọn, Siêu Định Hình</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-doi-tat-nam-tat-nam-vo-nam-co-dai-cao-cap-mrm-fashion-cung-mau-p34159085.html?spid=34159089</t>
+          <t>https://tiki.vn/quan-gen-chong-cuon-dui-8292-p244298352.html?spid=244298362</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>135000</v>
+        <v>122000</v>
       </c>
       <c r="G9" t="n">
-        <v>135000</v>
+        <v>97600</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>-24400</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="J9" t="n">
-        <v>4716</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>4717</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>135000</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1208,24 +1208,24 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá giảm 24,400đ (20.0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>51299947</t>
+          <t>278021672</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Áo Sơ Mi Caro TitiShop SM1164 ( Luxury)</t>
+          <t>Quần Lót Nam Đùi Boxer Lụa Băng Menpro MP9 - Mỏng nhem Thoáng Khí</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-caro-titishop-sm1164-luxury-p51299947.html?spid=51299949</t>
+          <t>https://tiki.vn/quan-lot-nam-dui-boxer-lua-bang-menpro-mp9-mong-nhem-thoang-khi-p278021672.html?spid=278021690</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1235,32 +1235,32 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Titishop</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>63200</v>
       </c>
       <c r="G10" t="n">
         <v>79000</v>
       </c>
       <c r="H10" t="n">
-        <v>79000</v>
+        <v>15800</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>79000</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -1282,51 +1282,51 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 15,800đ (+25.0%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>271973646</t>
+          <t>67538621</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Miếng dán hình xăm kinh dị hóa trang Halloween vết sẹo xước máu giả vết khâu chảy máu vết thương Legaxi</t>
+          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mieng-dan-hinh-xam-kinh-di-hoa-trang-halloween-vet-seo-xuoc-mau-gia-vet-khau-chay-mau-vet-thuong-legaxi-p271973646.html?spid=271973648</t>
+          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538623</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Legaxi</t>
+          <t>May 10</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>25000</v>
+        <v>135000</v>
       </c>
       <c r="G11" t="n">
-        <v>25000</v>
+        <v>135000</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1335,38 +1335,38 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>16599</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>16599</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="O11" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>4842</v>
       </c>
       <c r="R11" t="n">
-        <v>2</v>
+        <v>4843</v>
       </c>
       <c r="S11" t="n">
         <v>1</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,47 +1376,47 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm | Review thêm +1</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>279296102</t>
+          <t>277983818</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[NEW ARRIVAL] Giày Sneaker Nam Nữ DC48 SHADOW MOVE Dincox Shoes Đế Bằng - Da phối Suede Cao Cấp</t>
+          <t>Áo Lót Nữ Ren Dày Cài Trước Có Gọng Nâng Ngực Belle VC02 – Combo Đa Màu, Đệm Mút 3 cm, Quyến Rũ &amp; Đỡ Đỡ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/new-arrival-giay-sneaker-nam-nu-dc48-shadow-move-dincox-shoes-de-bang-da-phoi-suede-cao-cap-p279296102.html?spid=279296104</t>
+          <t>https://tiki.vn/ao-lot-nu-ren-day-cai-truoc-co-gong-nang-nguc-belle-vc02-combo-da-mau-dem-mut-3-cm-quyen-ru-do-do-p277983818.html?spid=277983822</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>DINCOX</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="G12" t="n">
-        <v>650000</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>650000</v>
+        <v>-150000</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -1437,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1450,34 +1450,34 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>276945307</t>
+          <t>278883514</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Áo lót nữ Angelavic 529 – Bra thun lạnh tăm, mút liền, cài sau, không gọng, nâng đỡ thoải mái</t>
+          <t>Áo sơ mi xếp 3 li kết ngọc tay dài</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-ao-bra-thun-lanh-tam-mut-lien-cai-sau-529-p276945307.html?spid=276945325</t>
+          <t>https://tiki.vn/ao-so-mi-xep-3-li-ket-ngoc-tay-dai-p278883514.html?spid=278883520</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1491,16 +1491,16 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>82500</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>110000</v>
+        <v>125000</v>
       </c>
       <c r="H13" t="n">
-        <v>27500</v>
+        <v>125000</v>
       </c>
       <c r="I13" t="n">
-        <v>33.33</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1534,63 +1534,63 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Giá tăng 27,500đ (+33.3%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>244297794</t>
+          <t>115852451</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Combo 5 Quần Lót Nam Thun Lạnh Lưng To Menlive ML1 – Size M–4XL, Co Giãn 4 Chiều</t>
+          <t>Chai vệ sinh giày đồ da, túi ví, áo, ghế da giúp làm sạch, dưỡng ẩm chống mốc XIMO XI03</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nam-thun-lanh-menlive-p244297794.html?spid=244297815</t>
+          <t>https://tiki.vn/chai-ve-sinh-giay-do-da-tui-vi-ao-ghe-da-giup-lam-sach-duong-am-chong-moc-ximo-xi03-p115852451.html?spid=262784198</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>159600</v>
+        <v>75000</v>
       </c>
       <c r="G14" t="n">
-        <v>190000</v>
+        <v>70000</v>
       </c>
       <c r="H14" t="n">
-        <v>30400</v>
+        <v>-5000</v>
       </c>
       <c r="I14" t="n">
-        <v>19.05</v>
+        <v>-6.67</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="K14" t="n">
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1599,26 +1599,26 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O14" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1628,29 +1628,29 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Giá tăng 30,400đ (+19.0%)</t>
+          <t>Giá giảm 5,000đ (6.7%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>72881856</t>
+          <t>244297862</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Quần lót nam thun lạnh không đường may, sịp đùi nam cao cấp kiểu dáng boxer nam ôm sát, chất liệu su thoáng mát, mềm mịn và mỏng nhẹ, quần lót cạp nhỏ đơn giản với màu trơn QLW806</t>
+          <t>Áo Lót Nữ Bra Ống Su Gân Viền Ren Cài Sau 4003 – Seamless, Co Giãn 4 Chiều</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nam-thun-lanh-khong-duong-may-sip-dui-nam-cao-cap-kieu-dang-boxer-nam-om-sat-chat-lieu-su-thoang-mat-mem-min-va-mong-nhe-quan-lot-cap-nho-don-gian-voi-mau-tron-qlw806-p72881856.html?spid=102551187</t>
+          <t>https://tiki.vn/ao-bra-ong-su-gan-cai-sau-4003-p244297862.html?spid=244297867</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1659,22 +1659,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>69000</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>69000</v>
+        <v>36800</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>36800</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1683,73 +1683,73 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Review thêm +1</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>51297510</t>
+          <t>279295829</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Áo Sơ Mi Caro TitiShop SM1161 ( Luxury)</t>
+          <t>Giày Sneaker Da - GAT Shoes Nam Nữ DC36 White Dune Dincox Shoes</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-caro-titishop-sm1161-luxury-p51297510.html?spid=51297512</t>
+          <t>https://tiki.vn/giay-sneaker-da-gat-shoes-nam-nu-dc36-white-dune-dincox-shoes-p279295829.html?spid=279295837</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Titishop</t>
+          <t>DINCOX</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>79000</v>
+        <v>600000</v>
       </c>
       <c r="H16" t="n">
-        <v>79000</v>
+        <v>600000</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1803,46 +1803,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>136093004</t>
+          <t>278957623</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Áo thun may ô ngắn tay (áo đông xuân) nam</t>
+          <t>Dép quai kẹp Biti's nam (size 38-43)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-may-o-ngan-tay-ao-dong-xuan-nam-p136093004.html?spid=136093008</t>
+          <t>https://tiki.vn/dep-quai-kep-biti-s-nam-size-38-43-p278957623.html?spid=278957641</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">	OEM</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>69000</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>89000</v>
+        <v>232000</v>
       </c>
       <c r="H17" t="n">
-        <v>20000</v>
+        <v>232000</v>
       </c>
       <c r="I17" t="n">
-        <v>28.99</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,53 +1851,53 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá tăng 20,000đ (+29.0%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>277420779</t>
+          <t>278863219</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Khẩu Trang Chống Nắng Cao Cấp UPF 50+,Khẩu Trang Chống Nám Chống Tia UV, Bảo Vệ Da Hiệu Quả - HÀNG CHÍNH HÃNG MINIIN</t>
+          <t>Dây Lưng Nam Thắt Lưng Da Chính Hãng GENCE LG52 Chất Liệu Da Bò Cao Cấp Màu Nâu</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/khau-trang-chong-nang-enaide-cao-cap-upf-50-chong-tia-uv-bao-ve-da-hieu-qua-hang-chinh-hang-miniin-p277420779.html?spid=277420793</t>
+          <t>https://tiki.vn/day-lung-nam-that-lung-da-chinh-hang-gence-lg52-chat-lieu-da-bo-cao-cap-mau-nau-p278863219.html?spid=278863220</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1907,26 +1907,26 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MINIIN</t>
+          <t>Gence</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>27000</v>
+        <v>715000</v>
       </c>
       <c r="H18" t="n">
-        <v>-28000</v>
+        <v>715000</v>
       </c>
       <c r="I18" t="n">
-        <v>-50.91</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1954,39 +1954,39 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá giảm 28,000đ (50.9%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>279100044</t>
+          <t>146589320</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chai Xịt Khử Mùi Giày Dép 260ML</t>
+          <t>Cài tóc pha lê kim cương sang trọng - bờm tóc pha lê - quà tặng cho bạn gái</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-xit-khu-mui-giay-dep-260ml-p279100044.html?spid=279100045</t>
+          <t>https://tiki.vn/cai-toc-pha-le-kim-cuong-sang-trong-bom-toc-pha-le-qua-tang-cho-ban-gai-p146589320.html?spid=146589326</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1995,50 +1995,50 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>48000</v>
+        <v>68000</v>
       </c>
       <c r="G19" t="n">
-        <v>59000</v>
+        <v>68000</v>
       </c>
       <c r="H19" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>22.92</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
+        <v>130</v>
+      </c>
+      <c r="K19" t="n">
+        <v>130</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="O19" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>18</v>
+      </c>
+      <c r="R19" t="n">
+        <v>19</v>
+      </c>
+      <c r="S19" t="n">
         <v>1</v>
       </c>
-      <c r="K19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="n">
-        <v>0</v>
-      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,53 +2048,53 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá tăng 11,000đ (+22.9%)</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>112814658</t>
+          <t>147249168</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Thắt Lưng Nam Dây Vải Dù Phong Cách Lính U379 US ARMY, Khóa Cài Tự Động Dễ Dàng Điều Chỉnh Theo Vòng Bụng- HÀNG CHÍNH HÃNG</t>
+          <t>Dép Nam Quai Ngang HÀ NAM Da Bò Thật Cao Cấp DNA2158</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-nam-day-vai-du-phong-cach-linh-u379-us-army-khoa-cai-tu-dong-de-dang-dieu-chinh-theo-vong-bung-hang-chinh-hang-p112814658.html?spid=174134932</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-ha-nam-cao-cap-dna2158-p147249168.html?spid=147249212</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>US ARMY</t>
+          <t>HA NAM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>99000</v>
+        <v>372000</v>
       </c>
       <c r="G20" t="n">
-        <v>99000</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>-372000</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J20" t="n">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -2103,73 +2103,73 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q20" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Review thêm +1</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>276146188</t>
+          <t>277718250</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Combo đồ bơi nam quần 2 lớp kèm kính mũ bơi, túi đựng đồ và bịt tai kẹp mũi, set bơi đầy đủ tiện lợi cho nam giới, quần bơi 2 lớp &amp; kính chống đọng sương | BN032</t>
+          <t>Giày Sandal nam cao cấp kiểu dáng mới – GSDNA10</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-do-boi-nam-quan-2-lop-kem-kinh-mu-boi-tui-dung-do-va-bit-tai-kep-mui-set-boi-day-du-tien-loi-cho-nam-gioi-quan-boi-2-lop-kinh-chong-dong-suong-bn032-p276146188.html?spid=276146212</t>
+          <t>https://tiki.vn/giay-sandal-nam-cao-cap-kieu-dang-moi-gsdna10-p277718250.html?spid=277718278</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Bee Gee</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>350000</v>
+        <v>583440</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>-350000</v>
+        <v>-583440</v>
       </c>
       <c r="I21" t="n">
         <v>-100</v>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2223,37 +2223,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>75728341</t>
+          <t>244298960</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Áo Sơ Mi Nam Titishop SM1281</t>
+          <t>Quần Mặc Váy Su Thông Hơi Trơn 6530 | Mát Mẻ, Không Lộ, Chống Hớ Hiệu Quả</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nam-titishop-sm1281-p75728341.html?spid=75728349</t>
+          <t>https://tiki.vn/quan-vay-dai-thong-hoi-6530-p244298960.html?spid=244298972</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Titishop</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>59000</v>
+        <v>35280</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>-59000</v>
+        <v>-35280</v>
       </c>
       <c r="I22" t="n">
         <v>-100</v>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2307,17 +2307,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>152632563</t>
+          <t>279292197</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Áo Lót Nữ Mút Mỏng Trơn Không Gọng 3281 – Nhẹ Êm, Tự Nhiên, Dễ Mặc Mỗi Ngày</t>
+          <t>Quần Lọt Khe Thêu Nơ Ren Lưới Xuyên Thấu Đính Nơ Sau Xinh Xắn</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-duc-kiem-bra-cao-cap-3281-big-size-p152632563.html?spid=274990712</t>
+          <t>https://tiki.vn/quan-lot-khe-theu-no-ren-luoi-xuyen-thau-dinh-no-sau-xinh-xan-p279292197.html?spid=279292199</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2327,23 +2327,23 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Sanny House</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>82170</v>
+        <v>82500</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>-82170</v>
+        <v>-82500</v>
       </c>
       <c r="I23" t="n">
         <v>-100</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2391,43 +2391,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>163806087</t>
+          <t>275632752</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da</t>
+          <t>Thắt lưng nam da bò nguyên chất mặt khóa tự động hợp kim cao cấp</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-p163806087.html?spid=253461440</t>
+          <t>https://tiki.vn/that-lung-nam-da-bo-nguyen-chat-mat-khoa-tu-dong-hop-kim-cao-cap-p275632752.html?spid=275632754</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>ANANSHOP688</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>59000</v>
+        <v>190000</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>-59000</v>
+        <v>-190000</v>
       </c>
       <c r="I24" t="n">
         <v>-100</v>
       </c>
       <c r="J24" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -2439,16 +2439,16 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>-5</v>
+        <v>-4.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2475,17 +2475,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>273550361</t>
+          <t>275276374</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Lót giày sức khỏe cho chân vòm cao Spenco Ground Control High Arch ôm sát vòm chân</t>
+          <t>Dép tổ ong XANH RÊU nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/lot-giay-y-khoa-spenco-ground-control-high-arch-p273550361.html?spid=273550365</t>
+          <t>https://tiki.vn/dep-to-ong-xanh-reu-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276374.html?spid=275276382</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2495,170 +2495,170 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Spenco</t>
+          <t xml:space="preserve">VAC </t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>895000</v>
+        <v>72000</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>72000</v>
       </c>
       <c r="H25" t="n">
-        <v>-895000</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>-72000</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="P25" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Bán thêm -1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>273097909</t>
+          <t>174437687</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tròng kính cận/viễn/loạn mỏng 1.60 chemi đổi màu thời trang OURESS</t>
+          <t>Dép nhựa Bitis nam</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/trong-kinh-can-vien-loan-mong-1-60-chemi-doi-mau-thoi-trang-ouress-p273097909.html?spid=273097910</t>
+          <t>https://tiki.vn/dep-nhua-bitis-nam-p174437687.html?spid=174437689</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OURESS</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1100000</v>
+        <v>105000</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>89000</v>
       </c>
       <c r="H26" t="n">
-        <v>-1100000</v>
+        <v>-16000</v>
       </c>
       <c r="I26" t="n">
-        <v>-100</v>
+        <v>-15.24</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-267000</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P26" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="S26" t="n">
         <v>0</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá giảm 16,000đ (15.2%) | Bán thêm -3 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>225209462</t>
+          <t>104791604</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MŨ CHỐNG NẮNG CÓI NỬA ĐẦU RỘNG VÀNH CÁ TÍNH CHO NỮ</t>
+          <t>Quần lót nữ thái lan 828 – Chất thun lạnh - giao màu ngẫu nhiên</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/mu-chong-nang-coi-nua-dau-rong-vanh-ca-tinh-cho-nu-p225209462.html?spid=247940496</t>
+          <t>https://tiki.vn/quan-lot-nu-thai-lan-828-chat-thun-lanh-giao-mau-ngau-nhien-p104791604.html?spid=270215621</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2667,60 +2667,60 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>55000</v>
+        <v>33880</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>36520</v>
       </c>
       <c r="H27" t="n">
-        <v>-55000</v>
+        <v>2640</v>
       </c>
       <c r="I27" t="n">
-        <v>-100</v>
+        <v>7.79</v>
       </c>
       <c r="J27" t="n">
+        <v>41</v>
+      </c>
+      <c r="K27" t="n">
+        <v>24</v>
+      </c>
+      <c r="L27" t="n">
+        <v>-17</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-620840</v>
+      </c>
+      <c r="N27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q27" t="n">
         <v>2</v>
       </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
+      <c r="R27" t="n">
         <v>3</v>
       </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>-3</v>
-      </c>
-      <c r="Q27" t="n">
+      <c r="S27" t="n">
         <v>1</v>
       </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá tăng 2,640đ (+7.8%) | Bán thêm -17 sản phẩm | Rating 4.5→4.7 (+0.20) | Review thêm +1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-07-05
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V53"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,37 +543,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7997276</t>
+          <t>58362412</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Giày Sneaker Unisex Converse Chuck Taylor All Star 1970s All Hi 2018 - White (Size</t>
+          <t>Áo khoác da cá GOKING 6 túi cho nam nữ, form unisex. Chống lanh, giữ ấm, chống nắng, chống tia UV hiệu quả</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-sneaker-unisex-converse-chuck-taylor-all-star-1970s-all-white-hi-2018-p7997276.html?spid=26499478</t>
+          <t>https://tiki.vn/ao-khoac-nam-goking-chuyen-chong-nang-6-tui-tien-dung-vai-day-cong-nghe-nhat-ban-cao-cap-p58362412.html?spid=58362420</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>GOKING</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2000000</v>
+        <v>339000</v>
       </c>
       <c r="H2" t="n">
-        <v>2000000</v>
+        <v>339000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,13 +582,13 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="L2" t="n">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="M2" t="n">
-        <v>78000000</v>
+        <v>28476000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -603,14 +603,14 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="S2" t="n">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -627,17 +627,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7995403</t>
+          <t>126091279</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Giày Converse Chuck Taylor All Star Classic Hi Top - 121184</t>
+          <t>Giày Mọi, Giày Lười Nam Da Bò SUNPOLO SU5059 Hiện đại (Đen)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-converse-chuck-taylor-all-star-classic-hi-top-121184-p7995403.html?spid=20342953</t>
+          <t>https://tiki.vn/giay-moi-giay-luoi-nam-da-bo-sunpolo-su5059-hien-dai-den-p126091279.html?spid=126091289</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Converse</t>
+          <t>SUNPOLO</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1550000</v>
+        <v>1100000</v>
       </c>
       <c r="H3" t="n">
-        <v>1550000</v>
+        <v>1100000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>34100000</v>
+        <v>8800000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -687,14 +687,14 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>112188948</t>
+          <t>132286309</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dép Nam Quai Ngang HA NAM Da Bò Thật Cao Cấp DNA2074</t>
+          <t>Bộ Dụng Cụ Đánh Giày 7 Món Có Kèm Sẵn 2 Hộp Xi Tiện Dụng- Đánh Bóng Mới - Hàng Loại 1- Chính Hãng MINIIN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-cao-cap-dna2074-p112188948.html?spid=112188950</t>
+          <t>https://tiki.vn/bo-dung-cu-danh-giay-7-mon-co-kem-san-2-hop-xi-tien-dung-danh-bong-moi-hang-loai-1-chinh-hang-miniin-p132286309.html?spid=132286315</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HA NAM</t>
+          <t>MINIIN</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>380000</v>
+        <v>99000</v>
       </c>
       <c r="H4" t="n">
-        <v>380000</v>
+        <v>99000</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -750,13 +750,13 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L4" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M4" t="n">
-        <v>21280000</v>
+        <v>5247000</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -771,14 +771,14 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="S4" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -795,22 +795,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>181566777</t>
+          <t>26652440</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Áo sơ mi nam sọc tay ngắn dáng ôm body chuẩn form nhiều màu sắc - MON01</t>
+          <t>1 Hộp Khăn Lau Kính Mắt - Màn Hình Điện Tử</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nam-soc-tay-ngan-dang-om-body-chuan-form-nhieu-mau-sac-mon01-p181566777.html?spid=181566813</t>
+          <t>https://tiki.vn/1-hop-khan-lau-kinh-mat-man-hinh-dien-tu-p26652440.html?spid=146386798</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -822,10 +822,10 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>137500</v>
+        <v>99000</v>
       </c>
       <c r="H5" t="n">
-        <v>137500</v>
+        <v>99000</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -834,13 +834,13 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="L5" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="M5" t="n">
-        <v>3162500</v>
+        <v>2673000</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -855,14 +855,14 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -879,17 +879,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>52758100</t>
+          <t>183685137</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Combo 5 Đôi Tất Nam Vớ Nam Cổ Dài Sợi Cotton Cùng Màu</t>
+          <t>Thắt Lưng Dây Nịt Nam Vải Dù US ARMY, Phong Cách Sang Trọng Cổ Điển Mặt Khóa Hợp Kim Thép Chống Ghỉ Cao Cấp -HÀNG CHÍNH HÃNG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-doi-tat-nam-vo-nam-co-dai-soi-cotton-cung-mau-p52758100.html?spid=67294705</t>
+          <t>https://tiki.vn/that-lung-day-nit-nam-vai-du-us-army-phong-cach-sang-trong-co-dien-mat-khoa-hop-kim-thep-chong-ghi-cao-cap-hang-chinh-hang-p183685137.html?spid=183685139</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -899,54 +899,54 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JM Jamano</t>
+          <t>US ARMY</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>99000</v>
+        <v>79000</v>
       </c>
       <c r="G6" t="n">
-        <v>175000</v>
+        <v>79000</v>
       </c>
       <c r="H6" t="n">
-        <v>76000</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>76.77</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>4207</v>
+        <v>210</v>
       </c>
       <c r="K6" t="n">
-        <v>4211</v>
+        <v>222</v>
       </c>
       <c r="L6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="M6" t="n">
-        <v>700000</v>
+        <v>948000</v>
       </c>
       <c r="N6" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="O6" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>859</v>
+        <v>59</v>
       </c>
       <c r="R6" t="n">
-        <v>859</v>
+        <v>59</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -956,29 +956,29 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Giá tăng 76,000đ (+76.8%) | Bán thêm +4 sản phẩm</t>
+          <t>Bán thêm +12 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>189528669</t>
+          <t>191422227</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Áo sơ mi nữ rộng dài tay phong cách hàn quốc trẻ trung năng động vải lụa mềm mịn -MURD05</t>
+          <t>Cột tóc scrunchies màu cánh dán ánh kim size trung</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nu-rong-dai-tay-phong-cach-han-quoc-tre-trung-nang-dong-vai-lua-mem-min-murd05-p189528669.html?spid=189528683</t>
+          <t>https://tiki.vn/day-cot-toc-scrunchies-mau-canh-dan-anh-kim-size-trung-p191422227.html?spid=191422228</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -987,28 +987,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>24900</v>
       </c>
       <c r="G7" t="n">
-        <v>115500</v>
+        <v>24900</v>
       </c>
       <c r="H7" t="n">
-        <v>115500</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="L7" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="M7" t="n">
-        <v>693000</v>
+        <v>821700</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1030,219 +1030,219 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +33 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>107802069</t>
+          <t>201594583</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
+          <t>Áo Thun Nam Dài Tay Aligro Chất Liệu Cotton Cao Cấp, Siêu Mềm Mại, Dày Dặn, Cực Dễ Chịu, Thấm Hút Tốt ALGAPD055</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
+          <t>https://tiki.vn/ao-thun-nam-dai-tay-aligro-chat-lieu-cotton-cao-cap-sieu-mem-mai-day-dan-cuc-de-chiu-tham-hut-tot-algapd055-p201594583.html?spid=201594593</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>Aligro</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>42000</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>42000</v>
+        <v>335000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>335000</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1033</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1041</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>336000</v>
+        <v>335000</v>
       </c>
       <c r="N8" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +8 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>278149879</t>
+          <t>107802069</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combo 5 quần lót nữ du lịch dùng 1 lần Size L 45-55kg</t>
+          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-bao-quan-lot-mien-giat-tien-loi-travel-mate-nu-5-cai-bao-size-m-vong-mong-84-94-cm-p278149879.html?spid=278149880</t>
+          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LuckyJQR</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>42000</v>
       </c>
       <c r="G9" t="n">
-        <v>110000</v>
+        <v>42000</v>
       </c>
       <c r="H9" t="n">
-        <v>110000</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1041</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>1047</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M9" t="n">
-        <v>220000</v>
+        <v>252000</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +6 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>183498218</t>
+          <t>272408652</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nón Kết Nam Lính Mỹ U558 Thêu AIR FORCE Chóp Tròn , Nón Lưỡi Trai Nam Vải Kaki Cao Cấp Thời Trang US ARMY Phong Cách Lính Mỹ - HÀNG CHÍNH HÃNG</t>
+          <t>Áo Thun T-shirt Nam Cổ Tròn TRẮNG, ĐEN 100% Cotton Cao Cấp, Trẻ Trung, Thanh Lịch - Gold Rhino</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/non-ket-nam-linh-my-u558-theu-air-force-chop-tron-non-luoi-trai-nam-vai-kaki-cao-cap-thoi-trang-us-army-phong-cach-linh-my-hang-chinh-hang-p183498218.html?spid=183498220</t>
+          <t>https://tiki.vn/ao-thun-nam-t-shirt-mau-trang-co-tron-100-cotton-tre-trung-thanh-lich-p272408652.html?spid=272408850</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>US ARMY</t>
+          <t>Gold Rhino</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>94500</v>
+        <v>209000</v>
       </c>
       <c r="G10" t="n">
-        <v>94500</v>
+        <v>209000</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1251,38 +1251,38 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>259</v>
+        <v>10</v>
       </c>
       <c r="K10" t="n">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>189000</v>
+        <v>209000</v>
       </c>
       <c r="N10" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1292,81 +1292,81 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Bán thêm +2 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>275276374</t>
+          <t>49210060</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dép tổ ong XANH RÊU nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Vỉ 3 Kẹp Tóc Càng Cua PASTEL 3 Chấu Loại Xịn MP120.3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-xanh-reu-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276374.html?spid=275276390</t>
+          <t>https://tiki.vn/vi-3-kep-toc-cang-cua-pastel-3-chau-loai-xin-mp120-3-p49210060.html?spid=51138209</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>72000</v>
+        <v>34900</v>
       </c>
       <c r="G11" t="n">
-        <v>75000</v>
+        <v>34900</v>
       </c>
       <c r="H11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>4.17</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>38</v>
+        <v>531</v>
       </c>
       <c r="K11" t="n">
-        <v>40</v>
+        <v>532</v>
       </c>
       <c r="L11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>150000</v>
+        <v>34900</v>
       </c>
       <c r="N11" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="O11" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Giá tăng 3,000đ (+4.2%) | Bán thêm +2 sản phẩm</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>190142008</t>
+          <t>54569520</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Áo sơ mi nam form rộng cổ tàu cổ trụ tay dài Giấu Nút phong cách hàn quốc trẻ trung lịch lãm-MRDT02</t>
+          <t>Quần Lót nam, quần sịp nam lụa Sữa Cao Cấp sp-340</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nam-form-rong-co-tau-co-tru-tay-dai-giau-nut-phong-cach-han-quoc-tre-trung-lich-lam-mrdt02-p190142008.html?spid=190142020</t>
+          <t>https://tiki.vn/quan-lot-nam-quan-sip-nam-lua-sua-cao-cap-sp-340-p54569520.html?spid=67859897</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1407,50 +1407,50 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>115000</v>
+        <v>88000</v>
       </c>
       <c r="G12" t="n">
-        <v>121000</v>
+        <v>67760</v>
       </c>
       <c r="H12" t="n">
-        <v>6000</v>
+        <v>-20240</v>
       </c>
       <c r="I12" t="n">
-        <v>5.22</v>
+        <v>-23</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>121000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,81 +1460,81 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Giá tăng 6,000đ (+5.2%) | Bán thêm +1 sản phẩm</t>
+          <t>Giá giảm 20,240đ (23.0%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>126144478</t>
+          <t>103049077</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Đón gót giày bằng sừng bóng đẹp (DGH903) Đón gót giày mọi tư thế Cho giày Nam &amp; Nữ - Tiện lợi</t>
+          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/don-got-giay-bang-sung-bong-dep-dgh903-don-got-giay-moi-tu-the-cho-giay-nam-nu-p126144478.html?spid=163423850</t>
+          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HAHANCO</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>59000</v>
+        <v>185000</v>
       </c>
       <c r="G13" t="n">
-        <v>59000</v>
+        <v>153550</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>-31450</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>-17</v>
       </c>
       <c r="J13" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="K13" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>59000</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,24 +1544,24 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá giảm 31,450đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>73163978</t>
+          <t>279491793</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hộp miếng dán ngực Silicon màu xanh 5 đôi</t>
+          <t>Đầm xoè linen cao cấp,độ bền cao,mát mịn,thấm hút mồ hôi,may viền tỉ mỉ,sản xuất độc quyền tại Kiều Oanh Designer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-mieng-dan-nguc-silicon-mau-xanh-5-doi-p73163978.html?spid=117659470</t>
+          <t>https://tiki.vn/dam-xoe-linen-cao-cap-do-ben-cao-mat-min-tham-hut-mo-hoi-may-vien-ti-mi-san-xuat-doc-quyen-tai-kieu-oanh-designer-p279491793.html?spid=279491958</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1571,86 +1571,86 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LQ luxury</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>55000</v>
+        <v>860000</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>860000</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>190129715</t>
+          <t>73862702</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Áo sơ mi nam cổ tàu cổ trụ form rộng tay dài trẻ trung thanh lịch vải lụa mềm mịn mát ít nhăn- MRDT01</t>
+          <t>ÁO LÓT NỮ REN MÚT DÀY 2CM DÂY TRƠN NÂNG NGỰC 024B</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nam-co-tau-co-tru-form-rong-tay-dai-tre-trung-thanh-lich-vai-lua-mem-min-mat-it-nhan-mrdt01-p190129715.html?spid=190129725</t>
+          <t>https://tiki.vn/ao-lot-nu-ren-mut-day-2cm-day-tron-nang-nguc-024b-p73862702.html?spid=73862720</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1659,22 +1659,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>115000</v>
+        <v>173000</v>
       </c>
       <c r="G15" t="n">
-        <v>121000</v>
+        <v>140130</v>
       </c>
       <c r="H15" t="n">
-        <v>6000</v>
+        <v>-32870</v>
       </c>
       <c r="I15" t="n">
-        <v>5.22</v>
+        <v>-19</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1692,17 +1692,17 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="R15" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1712,29 +1712,29 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Giá tăng 6,000đ (+5.2%)</t>
+          <t>Giá giảm 32,870đ (19.0%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>103049077</t>
+          <t>278004504</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
+          <t>Combo 5 Quần Lót Nữ Su Tăm Trơn Không Viền Mỏng Nhẹ 892 – Co Giãn 4 Chiều, Thoáng Mát, Không Lộ Viền (Size L/XL/XXL)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nu-su-tam-tron-khong-vien-mong-nhe-892-co-gian-4-chieu-thoang-mat-khong-lo-vien-size-l-xl-xxl-p278004504.html?spid=278004508</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1743,22 +1743,22 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>140600</v>
+        <v>188600</v>
       </c>
       <c r="G16" t="n">
-        <v>185000</v>
+        <v>230000</v>
       </c>
       <c r="H16" t="n">
-        <v>44400</v>
+        <v>41400</v>
       </c>
       <c r="I16" t="n">
-        <v>31.58</v>
+        <v>21.95</v>
       </c>
       <c r="J16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -1767,26 +1767,26 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1796,53 +1796,53 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Giá tăng 44,400đ (+31.6%)</t>
+          <t>Giá tăng 41,400đ (+22.0%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>279256558</t>
+          <t>74421501</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Áo polo nam tay ngắn phối cố Form Fitted - ROUTINE 10F25POL028</t>
+          <t>ÁO LÓT NỮ MỎNG CÓ GỌNG CÀI TRƯỚC VIỀN REN</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-polo-nam-tay-ngan-phoi-co-form-fitted-routine-10f25pol028-p279256558.html?spid=279256564</t>
+          <t>https://tiki.vn/ao-lot-nu-mong-co-gong-cai-truoc-vien-ren-p74421501.html?spid=74421553</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Routine</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>160000</v>
       </c>
       <c r="G17" t="n">
-        <v>579000</v>
+        <v>129600</v>
       </c>
       <c r="H17" t="n">
-        <v>579000</v>
+        <v>-30400</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>-19</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,53 +1851,53 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 30,400đ (19.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>91388606</t>
+          <t>7078807</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ÁO THUN NAM CAO CẤP CỔ BẺ PEGA IN</t>
+          <t>Bộ 10 Quần Lót Nam Chéo Nhật Bản Cao Cấp Thoáng Mát (Giao Màu Ngẫu Nhiên)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/product-p91388606.html?spid=113227822</t>
+          <t>https://tiki.vn/bo-10-quan-lot-nam-cheo-nhat-ban-cao-cap-thoang-mat-giao-mau-ngau-nhien-p7078807.html?spid=67858717</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1911,22 +1911,22 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>385000</v>
       </c>
       <c r="G18" t="n">
-        <v>454900</v>
+        <v>296450</v>
       </c>
       <c r="H18" t="n">
-        <v>454900</v>
+        <v>-88550</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>-23</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1935,53 +1935,53 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 88,550đ (23.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>133160820</t>
+          <t>113144956</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Quần Lót Su Đúc Nữ (Hàng Loại 1) Không Đường Mai, Thun Lạnh, SIêu Co Dãn, Được Chọn Màu</t>
+          <t>siêu phẩm áo lót nhật trơn đệm nâng ngực nhẹ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-su-duc-nu-hang-loai-1-khong-duong-mai-thun-lanh-sieu-co-dan-duoc-chon-mau-p133160820.html?spid=198901960</t>
+          <t>https://tiki.vn/sieu-pham-ao-lot-tron-dem-nang-nguc-nhe-p113144956.html?spid=142116876</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1995,22 +1995,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>22680</v>
+        <v>123750</v>
       </c>
       <c r="G19" t="n">
-        <v>28000</v>
+        <v>165000</v>
       </c>
       <c r="H19" t="n">
-        <v>5320</v>
+        <v>41250</v>
       </c>
       <c r="I19" t="n">
-        <v>23.46</v>
+        <v>33.33</v>
       </c>
       <c r="J19" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,24 +2048,24 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá tăng 5,320đ (+23.5%)</t>
+          <t>Giá tăng 41,250đ (+33.3%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>201934265</t>
+          <t>56041700</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Combo 2 Áo khoác gió nam chống nắng trượt nước cản gió cản bụi hiệu quả MRM Manlywear</t>
+          <t>Quần bơi nam cao cấp, đồ bơi nam boxer đẹp</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-2-ao-khoac-gio-nam-giu-nhiet-chong-nuoc-can-gio-can-bui-hieu-qua-mrm-manlywear-p201934265.html?spid=201934281</t>
+          <t>https://tiki.vn/quan-boi-nam-cao-cap-do-boi-nam-boxer-dep-p56041700.html?spid=56041702</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2075,23 +2075,23 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="G20" t="n">
-        <v>899000</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>899000</v>
+        <v>-200000</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -2103,16 +2103,16 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2122,34 +2122,34 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>274505062</t>
+          <t>52054230</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Áo polo thể thao Phiten polo (light) - Đen</t>
+          <t>combo 5 quần sịp chéo cotton nam xuất nhật túi zip bạc</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-polo-the-thao-phiten-polo-light-p274505062.html?spid=274505078</t>
+          <t>https://tiki.vn/combo-5-quan-sip-cheo-cotton-nam-xuat-nhat-tui-zip-bac-p52054230.html?spid=73622918</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2159,23 +2159,23 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Phiten</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>189000</v>
       </c>
       <c r="G21" t="n">
-        <v>1780000</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1780000</v>
+        <v>-189000</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
@@ -2206,63 +2206,63 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>174001966</t>
+          <t>173635485</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Quần Jean nam Leman xanh trơn JD03 - Slim Form</t>
+          <t>Giày Lười Nam Tăng Chiều Cao Da Bò Thật BIGGBEN Cao Cấp GM270</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-jean-nam-leman-xanh-tron-jd03-slim-form-p174001966.html?spid=174001978</t>
+          <t>https://tiki.vn/giay-luoi-nam-tang-chieu-cao-da-bo-that-biggben-cao-cap-gm269-p173635485.html?spid=278818066</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Leman</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>549000</v>
+        <v>999000</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1700000</v>
       </c>
       <c r="H22" t="n">
-        <v>-549000</v>
+        <v>701000</v>
       </c>
       <c r="I22" t="n">
-        <v>-100</v>
+        <v>70.17</v>
       </c>
       <c r="J22" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -2274,70 +2274,70 @@
         <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S22" t="n">
         <v>0</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá tăng 701,000đ (+70.2%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>276827848</t>
+          <t>275042862</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Quần Jean Ống Rộng Classic Carolina Blue Aaa Jeans</t>
+          <t>GIÀY CHẠY BỘ VÀ ĐI BỘ ĐỊA HÌNH SLM X-ADVENTURE OLIVE NIGHT - L47386000</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-jean-o-ng-rong-classic-carolina-blue-aaa-jeans-p276827848.html?spid=276827850</t>
+          <t>https://tiki.vn/giay-chay-bo-va-di-bo-dia-hinh-slm-x-adventure-olive-night-l47386000-p275042862.html?spid=275042868</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TRIPLE A</t>
+          <t>Salomon</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>650000</v>
+        <v>3800000</v>
       </c>
       <c r="H23" t="n">
-        <v>650000</v>
+        <v>3800000</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2391,17 +2391,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>112851354</t>
+          <t>113145806</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Áo ngực học sinh</t>
+          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138792</t>
+          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2415,22 +2415,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>30400</v>
+        <v>88920</v>
       </c>
       <c r="G24" t="n">
-        <v>42000</v>
+        <v>117000</v>
       </c>
       <c r="H24" t="n">
-        <v>11600</v>
+        <v>28080</v>
       </c>
       <c r="I24" t="n">
-        <v>38.16</v>
+        <v>31.58</v>
       </c>
       <c r="J24" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="K24" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2439,26 +2439,26 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
         <v>0</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2468,24 +2468,24 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Giá tăng 11,600đ (+38.2%)</t>
+          <t>Giá tăng 28,080đ (+31.6%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>108220832</t>
+          <t>144236336</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bra dán ngực bàn tay P29 (kèm dây trong)</t>
+          <t>COMBO 5 ÁO LÓT VẢI KHÔNG GỌNG KHÔNG MÚT (SIZE 32-42)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bra-dan-nguc-ban-tay-p29-kem-day-trong-p108220832.html?spid=242370964</t>
+          <t>https://tiki.vn/combo-5-ao-lot-vai-khong-gong-khong-mut-size-32-42-p144236336.html?spid=146366320</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2499,22 +2499,22 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>56250</v>
+        <v>210000</v>
       </c>
       <c r="G25" t="n">
-        <v>75000</v>
+        <v>174300</v>
       </c>
       <c r="H25" t="n">
-        <v>18750</v>
+        <v>-35700</v>
       </c>
       <c r="I25" t="n">
-        <v>33.33</v>
+        <v>-17</v>
       </c>
       <c r="J25" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2532,17 +2532,17 @@
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2552,53 +2552,53 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Giá tăng 18,750đ (+33.3%)</t>
+          <t>Giá giảm 35,700đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>214706031</t>
+          <t>276086848</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Áo lót áo ngực Thái lan có gọng mút kép nâng ngực tạo khe, áo lót nữ thông hơi hàng CAO CẤP</t>
+          <t>Cục bông trang trí nhiều màu sắc chọn lựa (tùy chọn màu sắc) (hàng có sẵn giao nhanh) (Hàng Chính Hãng)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-ao-nguc-thai-lan-co-gong-mut-kep-nang-nguc-tao-khe-ao-lot-nu-thong-hoi-hang-cao-cap-p214706031.html?spid=215408041</t>
+          <t>https://tiki.vn/cuc-bong-trang-tri-nhieu-mau-sac-chon-lua-tuy-chon-mau-sac-hang-co-san-giao-nhanh-hang-chinh-hang-p276086848.html?spid=276086851</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Bilaha</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>97200</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>120000</v>
+        <v>70000</v>
       </c>
       <c r="H26" t="n">
-        <v>22800</v>
+        <v>70000</v>
       </c>
       <c r="I26" t="n">
-        <v>23.46</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -2626,39 +2626,39 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Giá tăng 22,800đ (+23.5%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>187278904</t>
+          <t>192642640</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Áo sơ mi nữ form rộng tay dài phồng hot trend hàn quốc trẻ trung thanh lịch vải lụa mềm mịn-MUD02</t>
+          <t>Cài tóc bảng nhỏ 1 cm - cài tóc nam nữ - cài tóc đơn giản</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-so-mi-nu-form-rong-tay-dai-phong-hot-trend-han-quoc-tre-trung-thanh-lich-vai-lua-mem-min-mud02-p187278904.html?spid=187278918</t>
+          <t>https://tiki.vn/cai-toc-bang-nho-1-cm-cai-toc-nam-nu-cai-toc-don-gian-p192642640.html?spid=192642674</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2667,22 +2667,22 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>230000</v>
+        <v>24000</v>
       </c>
       <c r="G27" t="n">
-        <v>135000</v>
+        <v>24000</v>
       </c>
       <c r="H27" t="n">
-        <v>-95000</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>-41.3</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="K27" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2691,26 +2691,26 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O27" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="R27" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2720,53 +2720,53 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Giá giảm 95,000đ (41.3%)</t>
+          <t>Review thêm +2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>174585329</t>
+          <t>38160273</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Áo lót nâng ngực boya mút mỏng, Áo ngực boya nâng ngực cài sau 522BT</t>
+          <t>Giày Boot Nam BIGGBEN Da Bò Thật Cao Cấp BT2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nang-nguc-boya-mut-mong-ao-nguc-boya-nang-nguc-cai-sau-522bt-p174585329.html?spid=203717976</t>
+          <t>https://tiki.vn/giay-boot-nam-biggben-da-bo-that-cao-cap-bt2-p38160273.html?spid=38160275</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>BIGGBEN</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>85050</v>
+        <v>2000000</v>
       </c>
       <c r="G28" t="n">
-        <v>105000</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>19950</v>
+        <v>-2000000</v>
       </c>
       <c r="I28" t="n">
-        <v>23.46</v>
+        <v>-100</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -2775,82 +2775,82 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="Q28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
         <v>0</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Giá tăng 19,950đ (+23.5%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>158732070</t>
+          <t>278957623</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>❈✣♚Combo 10 quần lót nữ su đúc cao cấp không đường may, chất mát lạnh, mềm mịn, thoáng</t>
+          <t>Dép quai kẹp Biti's nam (size 38-43)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-10-quan-lot-nu-su-duc-cao-cap-khong-duong-may-chat-mat-lanh-mem-min-thoang-p158732070.html?spid=242324041</t>
+          <t>https://tiki.vn/dep-quai-kep-biti-s-nam-size-38-43-p278957623.html?spid=278957641</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Biti's</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>240000</v>
+        <v>232000</v>
       </c>
       <c r="G29" t="n">
-        <v>320000</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>80000</v>
+        <v>-232000</v>
       </c>
       <c r="I29" t="n">
-        <v>33.33</v>
+        <v>-100</v>
       </c>
       <c r="J29" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -2859,82 +2859,82 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
         <v>0</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Giá tăng 80,000đ (+33.3%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>275276309</t>
+          <t>276827848</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dép tổ ong ĐEN nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Quần Jean Ống Rộng Classic Carolina Blue Aaa Jeans</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-den-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276309.html?spid=275276319</t>
+          <t>https://tiki.vn/quan-jean-o-ng-rong-classic-carolina-blue-aaa-jeans-p276827848.html?spid=276827850</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>TRIPLE A</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>72000</v>
+        <v>650000</v>
       </c>
       <c r="G30" t="n">
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>3000</v>
+        <v>-650000</v>
       </c>
       <c r="I30" t="n">
-        <v>4.17</v>
+        <v>-100</v>
       </c>
       <c r="J30" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -2949,7 +2949,7 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -2962,34 +2962,34 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Giá tăng 3,000đ (+4.2%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>275276422</t>
+          <t>277744886</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dép tổ ong XANH NGỌC nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Giày Da Nam Italy - 1720BIA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-xanh-ngoc-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276422.html?spid=275276436</t>
+          <t>https://tiki.vn/giay-da-nam-italy-1720bia-p277744886.html?spid=277744894</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2999,26 +2999,26 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>Gianni Conti</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>72000</v>
+        <v>4000000</v>
       </c>
       <c r="G31" t="n">
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>3000</v>
+        <v>-4000000</v>
       </c>
       <c r="I31" t="n">
-        <v>4.17</v>
+        <v>-100</v>
       </c>
       <c r="J31" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -3027,82 +3027,82 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Giá tăng 3,000đ (+4.2%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>274804274</t>
+          <t>278449303</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dép tổ ong [Size 31-34] KÈM STICKER NGẪU NHIÊN vật liệu EVA cao cấp siêu bền, siêu nhẹ, chống trơn trượt</t>
+          <t xml:space="preserve">Mấy Xajy Bột Khô Siêu Khỏe 3000W – Bột Mịn Siêu Tốc, Nghiêjn Ngjũ Cốc &amp; Hạt Khô Đa Năng, đèn trang trí   đồng hồ treo tường </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-size-31-34-kem-sticker-ngau-nhien-vat-lieu-eva-cao-cap-sieu-ben-sieu-nhe-chong-tron-truot-p274804274.html?spid=274804515</t>
+          <t>https://tiki.vn/may-xajy-bot-kho-sieu-khoe-3000w-bot-min-sieu-toc-nghiejn-ngju-coc-hat-kho-da-nang-den-trang-tri-dong-ho-treo-tuong-p278449303.html?spid=278449304</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>65000</v>
+        <v>1288000</v>
       </c>
       <c r="G32" t="n">
-        <v>73000</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>8000</v>
+        <v>-1288000</v>
       </c>
       <c r="I32" t="n">
-        <v>12.31</v>
+        <v>-100</v>
       </c>
       <c r="J32" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -3130,60 +3130,60 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Giá tăng 8,000đ (+12.3%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>276558531</t>
+          <t>68491184</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Giày thể thao Bitis Hunter (39-45) 969k</t>
+          <t>Kính râm Nam thời trang + Tặng Tuavit Kính Xinh Mini đa năng</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-the-thao-bitis-hunter-39-45-969k-p276558531.html?spid=276558541</t>
+          <t>https://tiki.vn/kinh-ram-nam-thoi-trang-tang-tuavit-kinh-xinh-mini-da-nang-p68491184.html?spid=68491185</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>HOKO</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>169000</v>
       </c>
       <c r="G33" t="n">
-        <v>969000</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>969000</v>
+        <v>-169000</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -3201,7 +3201,7 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -3214,34 +3214,34 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>275276260</t>
+          <t>272224450</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dép tổ ong ĐỎ nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+          <t>Dép quai ngang nam, nữ siêu nhẹ DUWA - Hàng chính hãng - TK9056</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-to-ong-do-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276260.html?spid=275276270</t>
+          <t>https://tiki.vn/dep-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk9056-p272224450.html?spid=272224458</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3251,54 +3251,54 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC </t>
+          <t>DUWA</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>72000</v>
+        <v>159000</v>
       </c>
       <c r="G34" t="n">
-        <v>75000</v>
+        <v>159000</v>
       </c>
       <c r="H34" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>4.17</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>4</v>
       </c>
       <c r="K34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>-318000</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="O34" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -3308,59 +3308,59 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Giá tăng 3,000đ (+4.2%)</t>
+          <t>Bán thêm -2 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>262796074</t>
+          <t>278000485</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Chai vệ sinh đồ da làm sạch, dưỡng ẩm chống mốc, kháng khuẩn giày, túi ví, áo, ghế da 150ml</t>
+          <t>Áo lót nữ 718 – Mút mỏng thông hơi, không gọng, cài sau 3 móc, co giãn thoải mái</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://tiki.vn/chai-ve-sinh-do-da-lam-sach-duong-am-chong-moc-khang-khuan-giay-tui-vi-ao-ghe-da-150ml-p262796074.html?spid=262796075</t>
+          <t>https://tiki.vn/ao-lot-nu-718-mut-mong-thong-hoi-khong-gong-cai-sau-3-moc-co-gian-thoai-mai-p278000485.html?spid=278000517</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>70000</v>
+        <v>100000</v>
       </c>
       <c r="G35" t="n">
-        <v>75000</v>
+        <v>100000</v>
       </c>
       <c r="H35" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>7.14</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>-400000</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -3392,1519 +3392,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Giá tăng 5,000đ (+7.1%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>275276334</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Dép tổ ong XÁM nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-to-ong-xam-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276334.html?spid=275276350</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VAC </t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>72000</v>
-      </c>
-      <c r="G36" t="n">
-        <v>75000</v>
-      </c>
-      <c r="H36" t="n">
-        <v>3000</v>
-      </c>
-      <c r="I36" t="n">
-        <v>4.17</v>
-      </c>
-      <c r="J36" t="n">
-        <v>85</v>
-      </c>
-      <c r="K36" t="n">
-        <v>85</v>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O36" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>4</v>
-      </c>
-      <c r="R36" t="n">
-        <v>4</v>
-      </c>
-      <c r="S36" t="n">
-        <v>0</v>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>Giá tăng 3,000đ (+4.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>275276468</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Dép tổ ong XANH NAVY nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-to-ong-xanh-navy-vat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276468.html?spid=275276484</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VAC </t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>72000</v>
-      </c>
-      <c r="G37" t="n">
-        <v>75000</v>
-      </c>
-      <c r="H37" t="n">
-        <v>3000</v>
-      </c>
-      <c r="I37" t="n">
-        <v>4.17</v>
-      </c>
-      <c r="J37" t="n">
-        <v>23</v>
-      </c>
-      <c r="K37" t="n">
-        <v>23</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>5</v>
-      </c>
-      <c r="O37" t="n">
-        <v>5</v>
-      </c>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>1</v>
-      </c>
-      <c r="R37" t="n">
-        <v>1</v>
-      </c>
-      <c r="S37" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>Giá tăng 3,000đ (+4.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>192642401</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Giày Thể Thao Nam Biti's Hunter X LITEPLEX DSMH09800</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/giay-the-thao-nam-biti-s-hunter-x-liteplex-dsmh09800-p192642401.html?spid=192642413</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Biti's</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>1010000</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>-1010000</v>
-      </c>
-      <c r="I38" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J38" t="n">
-        <v>4</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" t="n">
-        <v>4</v>
-      </c>
-      <c r="O38" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" t="n">
-        <v>-4</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>1</v>
-      </c>
-      <c r="R38" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>252533129</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Găng Tay Hở 2 Ngón Unisex Chống Nắng, Có Thể Sử Dụng Cảm Ứng Điện Thoại</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/gang-tay-ho-2-ngon-unisex-chong-nang-co-the-su-dung-cam-ung-dien-thoai-p252533129.html?spid=252533130</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>19600</v>
-      </c>
-      <c r="G39" t="n">
-        <v>49000</v>
-      </c>
-      <c r="H39" t="n">
-        <v>29400</v>
-      </c>
-      <c r="I39" t="n">
-        <v>150</v>
-      </c>
-      <c r="J39" t="n">
-        <v>164</v>
-      </c>
-      <c r="K39" t="n">
-        <v>164</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="n">
-        <v>5</v>
-      </c>
-      <c r="O39" t="n">
-        <v>5</v>
-      </c>
-      <c r="P39" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>19</v>
-      </c>
-      <c r="R39" t="n">
-        <v>19</v>
-      </c>
-      <c r="S39" t="n">
-        <v>0</v>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>Giá tăng 29,400đ (+150.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>52154918</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trâm Cài Áo Nữ Hình Hoa Mẫu Đơn Trang Nhã Sang Trọng </t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/tram-cai-ao-nu-hinh-hoa-mau-don-trang-nha-sang-trong-p52154918.html?spid=52154919</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>29600</v>
-      </c>
-      <c r="G40" t="n">
-        <v>69000</v>
-      </c>
-      <c r="H40" t="n">
-        <v>39400</v>
-      </c>
-      <c r="I40" t="n">
-        <v>133.11</v>
-      </c>
-      <c r="J40" t="n">
-        <v>26</v>
-      </c>
-      <c r="K40" t="n">
-        <v>26</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" t="n">
-        <v>5</v>
-      </c>
-      <c r="O40" t="n">
-        <v>5</v>
-      </c>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>9</v>
-      </c>
-      <c r="R40" t="n">
-        <v>9</v>
-      </c>
-      <c r="S40" t="n">
-        <v>0</v>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>Giá tăng 39,400đ (+133.1%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>277420779</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Khẩu Trang Chống Nắng Cao Cấp UPF 50+,Khẩu Trang Chống Nám Chống Tia UV, Bảo Vệ Da Hiệu Quả - HÀNG CHÍNH HÃNG MINIIN</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/khau-trang-chong-nang-enaide-cao-cap-upf-50-chong-tia-uv-bao-ve-da-hieu-qua-hang-chinh-hang-miniin-p277420779.html?spid=277420791</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>MINIIN</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>27000</v>
-      </c>
-      <c r="G41" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" t="n">
-        <v>7</v>
-      </c>
-      <c r="K41" t="n">
-        <v>7</v>
-      </c>
-      <c r="L41" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" t="n">
-        <v>1</v>
-      </c>
-      <c r="P41" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" t="n">
-        <v>1</v>
-      </c>
-      <c r="S41" t="n">
-        <v>1</v>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Rating 0.0→1.0 (+1.00) | Review thêm +1</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>35087712</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Quần lót nam thun lạnh không đường may, sịp nam tam giác cao cấp chất liệu thoáng mát, mềm mịn QLW606</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/quan-lot-nam-thun-lanh-su-qlw606-p35087712.html?spid=116563301</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>69000</v>
-      </c>
-      <c r="G42" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="n">
-        <v>-69000</v>
-      </c>
-      <c r="I42" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J42" t="n">
-        <v>434</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" t="n">
-        <v>-4.8</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>86</v>
-      </c>
-      <c r="R42" t="n">
-        <v>0</v>
-      </c>
-      <c r="S42" t="n">
-        <v>0</v>
-      </c>
-      <c r="T42" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>134757633</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Áo Sơ Mi Form Rộng GIẤU NÚT Tay Dài Hàn Quốc Áo Unisex Nam Nữ Vải Lụa Mềm Mịn Thoáng Mát Ít Nhăn - SMD02</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-so-mi-form-rong-giau-nut-tay-dai-han-quoc-ao-unisex-nam-nu-vai-lua-mem-min-thoang-mat-it-nhan-smd02-p134757633.html?spid=134757665</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>125000</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>-125000</v>
-      </c>
-      <c r="I43" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J43" t="n">
-        <v>99</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" t="n">
-        <v>0</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="O43" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" t="n">
-        <v>-4.7</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>34</v>
-      </c>
-      <c r="R43" t="n">
-        <v>0</v>
-      </c>
-      <c r="S43" t="n">
-        <v>0</v>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>177502414</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Áo sơ mi trơn form rộng tay dài unisex nam nữ kiểu cổ bẻ phong cách hàn quốc trẻ trung - MRD03</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-so-mi-tron-form-rong-tay-dai-unisex-nam-nu-kieu-co-be-phong-cach-han-quoc-tre-trung-mrd03-p177502414.html?spid=177502428</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>115500</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>-115500</v>
-      </c>
-      <c r="I44" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J44" t="n">
-        <v>9</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
-        <v>0</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>0</v>
-      </c>
-      <c r="R44" t="n">
-        <v>0</v>
-      </c>
-      <c r="S44" t="n">
-        <v>0</v>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>72881856</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Quần lót nam thun lạnh không đường may, sịp đùi nam cao cấp kiểu dáng boxer nam ôm sát, chất liệu su thoáng mát, mềm mịn và mỏng nhẹ, quần lót cạp nhỏ đơn giản với màu trơn QLW806</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/quan-lot-nam-thun-lanh-khong-duong-may-sip-dui-nam-cao-cap-kieu-dang-boxer-nam-om-sat-chat-lieu-su-thoang-mat-mem-min-va-mong-nhe-quan-lot-cap-nho-don-gian-voi-mau-tron-qlw806-p72881856.html?spid=102551187</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>69000</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>-69000</v>
-      </c>
-      <c r="I45" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J45" t="n">
-        <v>143</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="n">
-        <v>-4.5</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>36</v>
-      </c>
-      <c r="R45" t="n">
-        <v>0</v>
-      </c>
-      <c r="S45" t="n">
-        <v>0</v>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>7997237</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Giày Converse Chuck Taylor All Star 1970s Low Top - 162058V</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/giay-converse-chuck-taylor-all-star-1970s-low-top-162058v-p7997237.html?spid=20296398</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Converse</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>1900000</v>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>-1900000</v>
-      </c>
-      <c r="I46" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J46" t="n">
-        <v>231</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
-        <v>0</v>
-      </c>
-      <c r="M46" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" t="n">
-        <v>5</v>
-      </c>
-      <c r="O46" t="n">
-        <v>0</v>
-      </c>
-      <c r="P46" t="n">
-        <v>-5</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>73</v>
-      </c>
-      <c r="R46" t="n">
-        <v>0</v>
-      </c>
-      <c r="S46" t="n">
-        <v>0</v>
-      </c>
-      <c r="T46" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>186271142</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Quần lót chất ren phối đáy cotton cao cấp sexy</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/quan-lot-chat-ren-phoi-day-cotton-cao-cap-sexy-p186271142.html?spid=186271150</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>35000</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>-35000</v>
-      </c>
-      <c r="I47" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J47" t="n">
-        <v>4</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
-        <v>0</v>
-      </c>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>0</v>
-      </c>
-      <c r="R47" t="n">
-        <v>0</v>
-      </c>
-      <c r="S47" t="n">
-        <v>0</v>
-      </c>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>192947717</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Áo sơ mi nữ form rộng tay ngắn chuẩn form hàn quốc trẻ trung năng động vải lạu mềm mại ít nhăn-MURN02</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-so-mi-nu-form-rong-tay-ngan-chuan-form-han-quoc-tre-trung-nang-dong-vai-lau-mem-mai-it-nhan-murn02-p192947717.html?spid=192947757</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>115000</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" t="n">
-        <v>-115000</v>
-      </c>
-      <c r="I48" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J48" t="n">
-        <v>3</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="n">
-        <v>5</v>
-      </c>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="n">
-        <v>-5</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>1</v>
-      </c>
-      <c r="R48" t="n">
-        <v>0</v>
-      </c>
-      <c r="S48" t="n">
-        <v>0</v>
-      </c>
-      <c r="T48" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>189527267</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Áo sơ mi nữ tay dài form rộng phong cách trẻ trung hàn quốc vải lụa mềm mịn mát -MURD04</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-so-mi-nu-tay-dai-form-rong-phong-cach-tre-trung-han-quoc-vai-lua-mem-min-mat-murd04-p189527267.html?spid=189527319</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F49" t="n">
-        <v>115500</v>
-      </c>
-      <c r="G49" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" t="n">
-        <v>-115500</v>
-      </c>
-      <c r="I49" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J49" t="n">
-        <v>7</v>
-      </c>
-      <c r="K49" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" t="n">
-        <v>5</v>
-      </c>
-      <c r="O49" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" t="n">
-        <v>-5</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>1</v>
-      </c>
-      <c r="R49" t="n">
-        <v>0</v>
-      </c>
-      <c r="S49" t="n">
-        <v>0</v>
-      </c>
-      <c r="T49" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>275042862</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>GIÀY CHẠY BỘ VÀ ĐI BỘ ĐỊA HÌNH SLM X-ADVENTURE OLIVE NIGHT - L47386000</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/giay-chay-bo-va-di-bo-dia-hinh-slm-x-adventure-olive-night-l47386000-p275042862.html?spid=275042868</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Salomon</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>3800000</v>
-      </c>
-      <c r="G50" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" t="n">
-        <v>-3800000</v>
-      </c>
-      <c r="I50" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J50" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" t="n">
-        <v>0</v>
-      </c>
-      <c r="M50" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" t="n">
-        <v>0</v>
-      </c>
-      <c r="S50" t="n">
-        <v>0</v>
-      </c>
-      <c r="T50" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>279277580</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Giày sandal thể thao, sandal học sinh VN2224 size 35-45 chính hãng VINASAN. Hàng Việt Nam xuất khẩu</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/giay-sandal-the-thao-sandal-hoc-sinh-vn2224-size-35-45-chinh-hang-vinasan-hang-viet-nam-xuat-khau-p279277580.html?spid=279277678</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>VINASAN</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>245000</v>
-      </c>
-      <c r="G51" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" t="n">
-        <v>-245000</v>
-      </c>
-      <c r="I51" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" t="n">
-        <v>0</v>
-      </c>
-      <c r="P51" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" t="n">
-        <v>0</v>
-      </c>
-      <c r="S51" t="n">
-        <v>0</v>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>274795145</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Dép tổ ong [Size 39-43] KÈM STICKER NGẪU NHIÊN vật liệu EVA cao cấp siêu bền, siêu nhẹ, chống trơn trượt</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-to-ong-size-39-43-kem-sticker-ngau-nhien-vat-lieu-eva-cao-cap-sieu-ben-sieu-nhe-chong-tron-truot-p274795145.html?spid=274803734</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VAC </t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>77000</v>
-      </c>
-      <c r="G52" t="n">
-        <v>83000</v>
-      </c>
-      <c r="H52" t="n">
-        <v>6000</v>
-      </c>
-      <c r="I52" t="n">
-        <v>7.79</v>
-      </c>
-      <c r="J52" t="n">
-        <v>51</v>
-      </c>
-      <c r="K52" t="n">
-        <v>50</v>
-      </c>
-      <c r="L52" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M52" t="n">
-        <v>-83000</v>
-      </c>
-      <c r="N52" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="O52" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="P52" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>5</v>
-      </c>
-      <c r="R52" t="n">
-        <v>5</v>
-      </c>
-      <c r="S52" t="n">
-        <v>0</v>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>Giá tăng 6,000đ (+7.8%) | Bán thêm -1 sản phẩm</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>262803154</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Đầm ngủ WANNABE DNS71 váy ngủ 2 dây cúp ngực lót mút mỏng tạo dáng cho người mặc in hoa ngọt ngào nữ tính quyến rũ</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/do-ngu-nu-wannabe-dns71-dam-ngu-hai-day-ra-cup-lot-mut-nu-tinh-quyen-ru-p262803154.html?spid=271126198</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Wannabe</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>390000</v>
-      </c>
-      <c r="G53" t="n">
-        <v>390000</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="n">
-        <v>8</v>
-      </c>
-      <c r="K53" t="n">
-        <v>6</v>
-      </c>
-      <c r="L53" t="n">
-        <v>-2</v>
-      </c>
-      <c r="M53" t="n">
-        <v>-780000</v>
-      </c>
-      <c r="N53" t="n">
-        <v>5</v>
-      </c>
-      <c r="O53" t="n">
-        <v>5</v>
-      </c>
-      <c r="P53" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>2</v>
-      </c>
-      <c r="R53" t="n">
-        <v>2</v>
-      </c>
-      <c r="S53" t="n">
-        <v>0</v>
-      </c>
-      <c r="T53" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>Bán thêm -2 sản phẩm</t>
+          <t>Bán thêm -4 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-07-06
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,17 +543,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>58362412</t>
+          <t>279287522</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Áo khoác da cá GOKING 6 túi cho nam nữ, form unisex. Chống lanh, giữ ấm, chống nắng, chống tia UV hiệu quả</t>
+          <t>Bộ áo điều hòa KITO NEWPRO KT10 thế hệ mới nhất 2026 quạt 24V siêu bên ,chống chai ,chống phồng</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-khoac-nam-goking-chuyen-chong-nang-6-tui-tien-dung-vai-day-cong-nghe-nhat-ban-cao-cap-p58362412.html?spid=58362420</t>
+          <t>https://tiki.vn/bo-ao-dieu-hoa-kito-newpro-kt10-the-he-moi-nhat-2026-quat-24v-sieu-ben-chong-chai-chong-phong-p279287522.html?spid=279287524</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GOKING</t>
+          <t>Kito</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1070000</v>
       </c>
       <c r="G2" t="n">
-        <v>339000</v>
+        <v>1070000</v>
       </c>
       <c r="H2" t="n">
-        <v>339000</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,62 +582,62 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="M2" t="n">
-        <v>28476000</v>
+        <v>9630000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +9 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>126091279</t>
+          <t>228132185</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Giày Mọi, Giày Lười Nam Da Bò SUNPOLO SU5059 Hiện đại (Đen)</t>
+          <t>Dép Nam Quai Ngang HÀ NAM Da Bò Thật Cao Cấp DNA2210</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-moi-giay-luoi-nam-da-bo-sunpolo-su5059-hien-dai-den-p126091279.html?spid=126091289</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-that-ha-nam-cao-cap-dna2210-p228132185.html?spid=228132221</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SUNPOLO</t>
+          <t>HA NAM</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1100000</v>
+        <v>450000</v>
       </c>
       <c r="H3" t="n">
-        <v>1100000</v>
+        <v>450000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M3" t="n">
-        <v>8800000</v>
+        <v>1800000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -687,14 +687,14 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,17 +711,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>132286309</t>
+          <t>276814141</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bộ Dụng Cụ Đánh Giày 7 Món Có Kèm Sẵn 2 Hộp Xi Tiện Dụng- Đánh Bóng Mới - Hàng Loại 1- Chính Hãng MINIIN</t>
+          <t>New Arrivals | Giày Da Sneaker Nam Nữ DC39 COCO MILK DINCOX Shoes Đế Bằng - Microfiber Leather</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-dung-cu-danh-giay-7-mon-co-kem-san-2-hop-xi-tien-dung-danh-bong-moi-hang-loai-1-chinh-hang-miniin-p132286309.html?spid=132286315</t>
+          <t>https://tiki.vn/new-arrivals-giay-da-sneaker-nam-nu-dc39-coco-milk-dincox-shoes-de-bang-microfiber-leather-p276814141.html?spid=276814174</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -731,81 +731,81 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MINIIN</t>
+          <t>DINCOX</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>660000</v>
       </c>
       <c r="G4" t="n">
-        <v>99000</v>
+        <v>660000</v>
       </c>
       <c r="H4" t="n">
-        <v>99000</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>5247000</v>
+        <v>660000</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O4" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>26652440</t>
+          <t>34159085</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1 Hộp Khăn Lau Kính Mắt - Màn Hình Điện Tử</t>
+          <t>Combo 5 Đôi Tất Cổ Trung Cùng Màu Cotton Thương Hiệu MRM Manlywear</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/1-hop-khan-lau-kinh-mat-man-hinh-dien-tu-p26652440.html?spid=146386798</t>
+          <t>https://tiki.vn/combo-5-doi-tat-nam-tat-nam-vo-nam-co-dai-cao-cap-mrm-fashion-cung-mau-p34159085.html?spid=34159089</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -815,81 +815,81 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>MRM Manlywear</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>149000</v>
       </c>
       <c r="G5" t="n">
-        <v>99000</v>
+        <v>149000</v>
       </c>
       <c r="H5" t="n">
-        <v>99000</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>4717</v>
       </c>
       <c r="K5" t="n">
-        <v>27</v>
+        <v>4720</v>
       </c>
       <c r="L5" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>2673000</v>
+        <v>447000</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O5" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>901</v>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>901</v>
       </c>
       <c r="S5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +3 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>183685137</t>
+          <t>68491184</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Thắt Lưng Dây Nịt Nam Vải Dù US ARMY, Phong Cách Sang Trọng Cổ Điển Mặt Khóa Hợp Kim Thép Chống Ghỉ Cao Cấp -HÀNG CHÍNH HÃNG</t>
+          <t>Kính râm Nam thời trang + Tặng Tuavit Kính Xinh Mini đa năng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-day-nit-nam-vai-du-us-army-phong-cach-sang-trong-co-dien-mat-khoa-hop-kim-thep-chong-ghi-cao-cap-hang-chinh-hang-p183685137.html?spid=183685139</t>
+          <t>https://tiki.vn/kinh-ram-nam-thoi-trang-tang-tuavit-kinh-xinh-mini-da-nang-p68491184.html?spid=68491185</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -899,138 +899,138 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>US ARMY</t>
+          <t>HOKO</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>79000</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>79000</v>
+        <v>169000</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>169000</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>222</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="M6" t="n">
-        <v>948000</v>
+        <v>338000</v>
       </c>
       <c r="N6" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Bán thêm +12 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>191422227</t>
+          <t>107802069</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cột tóc scrunchies màu cánh dán ánh kim size trung</t>
+          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/day-cot-toc-scrunchies-mau-canh-dan-anh-kim-size-trung-p191422227.html?spid=191422228</t>
+          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ximo</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>24900</v>
+        <v>42000</v>
       </c>
       <c r="G7" t="n">
-        <v>24900</v>
+        <v>27000</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>-15000</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>-35.71</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>1047</v>
       </c>
       <c r="K7" t="n">
-        <v>37</v>
+        <v>1048</v>
       </c>
       <c r="L7" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>821700</v>
+        <v>27000</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1040,44 +1040,44 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Bán thêm +33 sản phẩm</t>
+          <t>Giá giảm 15,000đ (35.7%) | Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>201594583</t>
+          <t>158565446</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Áo Thun Nam Dài Tay Aligro Chất Liệu Cotton Cao Cấp, Siêu Mềm Mại, Dày Dặn, Cực Dễ Chịu, Thấm Hút Tốt ALGAPD055</t>
+          <t>Áo Lót Nữ, Áo Ngực Trơn Mút Dày Hàng Thái Lan Hãng.A2280</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-nam-dai-tay-aligro-chat-lieu-cotton-cao-cap-sieu-mem-mai-day-dan-cuc-de-chiu-tham-hut-tot-algapd055-p201594583.html?spid=201594593</t>
+          <t>https://tiki.vn/ao-lot-nu-ao-nguc-tron-mut-day-hang-thai-lan-hang-a2280-p158565446.html?spid=276838010</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aligro</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>335000</v>
+        <v>87400</v>
       </c>
       <c r="H8" t="n">
-        <v>335000</v>
+        <v>87400</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1086,13 +1086,13 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>335000</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1131,74 +1131,74 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>107802069</t>
+          <t>276945307</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Keo Dán Giày Nhiệt XIMO Trong Suốt Siêu Dính Dùng Không Tổn Thương Da XKDG06</t>
+          <t>Áo lót nữ Angelavic 529 – Bra thun lạnh tăm, mút liền, cài sau, không gọng, nâng đỡ thoải mái</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-ximo-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-xkdg06-p107802069.html?spid=252869410</t>
+          <t>https://tiki.vn/ao-lot-nu-ao-bra-thun-lanh-tam-mut-lien-cai-sau-529-p276945307.html?spid=276945325</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ximo</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>42000</v>
+        <v>110000</v>
       </c>
       <c r="G9" t="n">
-        <v>42000</v>
+        <v>83600</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>-26400</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="J9" t="n">
-        <v>1041</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1047</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>252000</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1208,41 +1208,41 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Bán thêm +6 sản phẩm</t>
+          <t>Giá giảm 26,400đ (24.0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>272408652</t>
+          <t>277610005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Áo Thun T-shirt Nam Cổ Tròn TRẮNG, ĐEN 100% Cotton Cao Cấp, Trẻ Trung, Thanh Lịch - Gold Rhino</t>
+          <t>Áo Lót 3281 Không Gọng Mút Mỏng Bản 3 Móc Che Khuyết Điểm Đẹp</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-nam-t-shirt-mau-trang-co-tron-100-cotton-tre-trung-thanh-lich-p272408652.html?spid=272408850</t>
+          <t>https://tiki.vn/ao-lot-3281-khong-gong-mut-mong-ban-3-moc-che-khuyet-diem-dep-p277610005.html?spid=277610045</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gold Rhino</t>
+          <t>Sanny House</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>209000</v>
+        <v>96000</v>
       </c>
       <c r="G10" t="n">
-        <v>209000</v>
+        <v>96000</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1251,38 +1251,38 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
         <v>1</v>
       </c>
-      <c r="M10" t="n">
-        <v>209000</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1292,29 +1292,29 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Rating 0.0→5.0 (+5.00) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>49210060</t>
+          <t>16375016</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vỉ 3 Kẹp Tóc Càng Cua PASTEL 3 Chấu Loại Xịn MP120.3</t>
+          <t>COMBO HỘP 5 Quần Lót ĐÙI Nam Xuất Nhật Cao Cấp (MIX NGẪU NHIÊN)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/vi-3-kep-toc-cang-cua-pastel-3-chau-loai-xin-mp120-3-p49210060.html?spid=51138209</t>
+          <t>https://tiki.vn/combo-hop-5-quan-lot-dui-nam-xuat-nhat-cao-cap-mix-ngau-nhien-p16375016.html?spid=277961877</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1323,50 +1323,50 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>34900</v>
+        <v>198290</v>
       </c>
       <c r="G11" t="n">
-        <v>34900</v>
+        <v>274000</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>75710</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>38.18</v>
       </c>
       <c r="J11" t="n">
-        <v>531</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>532</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>34900</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá tăng 75,710đ (+38.2%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>54569520</t>
+          <t>277996544</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Quần Lót nam, quần sịp nam lụa Sữa Cao Cấp sp-340</t>
+          <t>Hộp 5 Quần lót nam cotton lụa – Siêu đẹp, mềm mịn, thoáng mát</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nam-quan-sip-nam-lua-sua-cao-cap-sp-340-p54569520.html?spid=67859897</t>
+          <t>https://tiki.vn/hop-5-quan-lot-nam-cotton-lua-muji-sieu-dep-mem-min-thoang-mat-p277996544.html?spid=278006734</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1407,22 +1407,22 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>88000</v>
+        <v>172200</v>
       </c>
       <c r="G12" t="n">
-        <v>67760</v>
+        <v>220000</v>
       </c>
       <c r="H12" t="n">
-        <v>-20240</v>
+        <v>47800</v>
       </c>
       <c r="I12" t="n">
-        <v>-23</v>
+        <v>27.76</v>
       </c>
       <c r="J12" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1440,17 +1440,17 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,24 +1460,24 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Giá giảm 20,240đ (23.0%)</t>
+          <t>Giá tăng 47,800đ (+27.8%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>103049077</t>
+          <t>16546849</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
+          <t>Combo 5 Quần Lót Nam Tam Giác Nhật</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-tam-giac-nhat-p16546849.html?spid=53006035</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1491,22 +1491,22 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>185000</v>
+        <v>161700</v>
       </c>
       <c r="G13" t="n">
-        <v>153550</v>
+        <v>210000</v>
       </c>
       <c r="H13" t="n">
-        <v>-31450</v>
+        <v>48300</v>
       </c>
       <c r="I13" t="n">
-        <v>-17</v>
+        <v>29.87</v>
       </c>
       <c r="J13" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1515,26 +1515,26 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="R13" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,29 +1544,29 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Giá giảm 31,450đ (17.0%)</t>
+          <t>Giá tăng 48,300đ (+29.9%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>279491793</t>
+          <t>7078807</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Đầm xoè linen cao cấp,độ bền cao,mát mịn,thấm hút mồ hôi,may viền tỉ mỉ,sản xuất độc quyền tại Kiều Oanh Designer</t>
+          <t>Bộ 10 Quần Lót Nam Chéo Nhật Bản Cao Cấp Thoáng Mát (Giao Màu Ngẫu Nhiên)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dam-xoe-linen-cao-cap-do-ben-cao-mat-min-tham-hut-mo-hoi-may-vien-ti-mi-san-xuat-doc-quyen-tai-kieu-oanh-designer-p279491793.html?spid=279491958</t>
+          <t>https://tiki.vn/bo-10-quan-lot-nam-cheo-nhat-ban-cao-cap-thoang-mat-giao-mau-ngau-nhien-p7078807.html?spid=67858717</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1575,22 +1575,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>296450</v>
       </c>
       <c r="G14" t="n">
-        <v>860000</v>
+        <v>420000</v>
       </c>
       <c r="H14" t="n">
-        <v>860000</v>
+        <v>123550</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>41.68</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1599,53 +1599,53 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 123,550đ (+41.7%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>73862702</t>
+          <t>143940811</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ÁO LÓT NỮ REN MÚT DÀY 2CM DÂY TRƠN NÂNG NGỰC 024B</t>
+          <t>Đồ bộ Tole lửng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-ren-mut-day-2cm-day-tron-nang-nguc-024b-p73862702.html?spid=73862720</t>
+          <t>https://tiki.vn/do-bo-tole-lung-p143940811.html?spid=278943919</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1659,22 +1659,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>173000</v>
+        <v>100000</v>
       </c>
       <c r="G15" t="n">
-        <v>140130</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>-32870</v>
+        <v>-100000</v>
       </c>
       <c r="I15" t="n">
-        <v>-19</v>
+        <v>-100</v>
       </c>
       <c r="J15" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1683,53 +1683,53 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q15" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Giá giảm 32,870đ (19.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>278004504</t>
+          <t>279491793</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Combo 5 Quần Lót Nữ Su Tăm Trơn Không Viền Mỏng Nhẹ 892 – Co Giãn 4 Chiều, Thoáng Mát, Không Lộ Viền (Size L/XL/XXL)</t>
+          <t>Đầm xoè linen cao cấp,độ bền cao,mát mịn,thấm hút mồ hôi,may viền tỉ mỉ,sản xuất độc quyền tại Kiều Oanh Designer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-lot-nu-su-tam-tron-khong-vien-mong-nhe-892-co-gian-4-chieu-thoang-mat-khong-lo-vien-size-l-xl-xxl-p278004504.html?spid=278004508</t>
+          <t>https://tiki.vn/dam-xoe-linen-cao-cap-do-ben-cao-mat-min-tham-hut-mo-hoi-may-vien-ti-mi-san-xuat-doc-quyen-tai-kieu-oanh-designer-p279491793.html?spid=279491958</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1743,16 +1743,16 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>188600</v>
+        <v>860000</v>
       </c>
       <c r="G16" t="n">
-        <v>230000</v>
+        <v>790000</v>
       </c>
       <c r="H16" t="n">
-        <v>41400</v>
+        <v>-70000</v>
       </c>
       <c r="I16" t="n">
-        <v>21.95</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1796,24 +1796,24 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Giá tăng 41,400đ (+22.0%)</t>
+          <t>Giá giảm 70,000đ (8.1%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>74421501</t>
+          <t>113145806</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ÁO LÓT NỮ MỎNG CÓ GỌNG CÀI TRƯỚC VIỀN REN</t>
+          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-mong-co-gong-cai-truoc-vien-ren-p74421501.html?spid=74421553</t>
+          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1827,22 +1827,22 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>160000</v>
+        <v>117000</v>
       </c>
       <c r="G17" t="n">
-        <v>129600</v>
+        <v>97110</v>
       </c>
       <c r="H17" t="n">
-        <v>-30400</v>
+        <v>-19890</v>
       </c>
       <c r="I17" t="n">
-        <v>-19</v>
+        <v>-17</v>
       </c>
       <c r="J17" t="n">
-        <v>153</v>
+        <v>4</v>
       </c>
       <c r="K17" t="n">
-        <v>153</v>
+        <v>4</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,26 +1851,26 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>4.7</v>
+        <v>1</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1880,29 +1880,29 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá giảm 30,400đ (19.0%)</t>
+          <t>Giá giảm 19,890đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7078807</t>
+          <t>112851354</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bộ 10 Quần Lót Nam Chéo Nhật Bản Cao Cấp Thoáng Mát (Giao Màu Ngẫu Nhiên)</t>
+          <t>Áo ngực học sinh</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-10-quan-lot-nam-cheo-nhat-ban-cao-cap-thoang-mat-giao-mau-ngau-nhien-p7078807.html?spid=67858717</t>
+          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138792</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1911,22 +1911,22 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>385000</v>
+        <v>42000</v>
       </c>
       <c r="G18" t="n">
-        <v>296450</v>
+        <v>35280</v>
       </c>
       <c r="H18" t="n">
-        <v>-88550</v>
+        <v>-6720</v>
       </c>
       <c r="I18" t="n">
-        <v>-23</v>
+        <v>-16</v>
       </c>
       <c r="J18" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="K18" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1935,26 +1935,26 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="O18" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R18" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1964,24 +1964,24 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá giảm 88,550đ (23.0%)</t>
+          <t>Giá giảm 6,720đ (16.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>113144956</t>
+          <t>278157402</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>siêu phẩm áo lót nhật trơn đệm nâng ngực nhẹ</t>
+          <t>Áo sơ mi kiểu tay lỡ cổ đức, chất liệu Đũi tơ mềm mát, thấm hút mồ hôi, áo kiểu nữ dễ thương, NeSa Shop AT12</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/sieu-pham-ao-lot-tron-dem-nang-nguc-nhe-p113144956.html?spid=142116876</t>
+          <t>https://tiki.vn/ao-so-mi-kieu-tay-lo-co-duc-chat-lieu-dui-to-mem-mat-tham-hut-mo-hoi-ao-kieu-nu-de-thuong-nesa-shop-at12-p278157402.html?spid=278157438</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1995,22 +1995,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>123750</v>
+        <v>168000</v>
       </c>
       <c r="G19" t="n">
-        <v>165000</v>
+        <v>168000</v>
       </c>
       <c r="H19" t="n">
-        <v>41250</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>33.33</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,26 +2019,26 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q19" t="n">
         <v>1</v>
       </c>
       <c r="R19" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" t="n">
         <v>1</v>
       </c>
-      <c r="S19" t="n">
-        <v>0</v>
-      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,50 +2048,50 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá tăng 41,250đ (+33.3%)</t>
+          <t>Rating 4.0→4.5 (+0.50) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>56041700</t>
+          <t>276827848</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Quần bơi nam cao cấp, đồ bơi nam boxer đẹp</t>
+          <t>Quần Jean Ống Rộng Classic Carolina Blue Aaa Jeans</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-boi-nam-cao-cap-do-boi-nam-boxer-dep-p56041700.html?spid=56041702</t>
+          <t>https://tiki.vn/quan-jean-o-ng-rong-classic-carolina-blue-aaa-jeans-p276827848.html?spid=276827850</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>TRIPLE A</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>650000</v>
       </c>
       <c r="H20" t="n">
-        <v>-200000</v>
+        <v>650000</v>
       </c>
       <c r="I20" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>134</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -2103,16 +2103,16 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2122,118 +2122,118 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>52054230</t>
+          <t>275631855</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>combo 5 quần sịp chéo cotton nam xuất nhật túi zip bạc</t>
+          <t>Thắt lưng nam da bò nguyên chất mặt khóa tự động hợp kim cao cấp</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-sip-cheo-cotton-nam-xuat-nhat-tui-zip-bac-p52054230.html?spid=73622918</t>
+          <t>https://tiki.vn/that-lung-nam-da-bo-nguyen-chat-mat-khoa-tu-dong-hop-kim-cao-cap-p275631855.html?spid=275631857</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>ANANSHOP688</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>189000</v>
+        <v>199000</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>199000</v>
       </c>
       <c r="H21" t="n">
-        <v>-189000</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
+        <v>36</v>
+      </c>
+      <c r="K21" t="n">
+        <v>36</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>9</v>
+      </c>
+      <c r="R21" t="n">
+        <v>10</v>
+      </c>
+      <c r="S21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0</v>
-      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Rating 4.6→4.5 (-0.10) | Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>173635485</t>
+          <t>152246210</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Giày Lười Nam Tăng Chiều Cao Da Bò Thật BIGGBEN Cao Cấp GM270</t>
+          <t>Giày mọi nam da bò thật BIGGBEN cao cấp GM266</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-luoi-nam-tang-chieu-cao-da-bo-that-biggben-cao-cap-gm269-p173635485.html?spid=278818066</t>
+          <t>https://tiki.vn/giay-moi-nam-da-bo-that-biggben-cao-cap-gm266-p152246210.html?spid=152246220</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2247,22 +2247,22 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>999000</v>
+        <v>599000</v>
       </c>
       <c r="G22" t="n">
-        <v>1700000</v>
+        <v>800000</v>
       </c>
       <c r="H22" t="n">
-        <v>701000</v>
+        <v>201000</v>
       </c>
       <c r="I22" t="n">
-        <v>70.17</v>
+        <v>33.56</v>
       </c>
       <c r="J22" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -2271,26 +2271,26 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S22" t="n">
         <v>0</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2300,50 +2300,50 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Giá tăng 701,000đ (+70.2%)</t>
+          <t>Giá tăng 201,000đ (+33.6%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>275042862</t>
+          <t>124273951</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GIÀY CHẠY BỘ VÀ ĐI BỘ ĐỊA HÌNH SLM X-ADVENTURE OLIVE NIGHT - L47386000</t>
+          <t>Bộ Búi Tóc Đa Năng 4 Món Giúp Bạn Có Kiểu Tóc Xinh</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-chay-bo-va-di-bo-dia-hinh-slm-x-adventure-olive-night-l47386000-p275042862.html?spid=275042868</t>
+          <t>https://tiki.vn/bo-bui-toc-da-nang-4-mon-giup-ban-co-kieu-toc-xinh-p124273951.html?spid=124273958</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Salomon</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>19000</v>
       </c>
       <c r="G23" t="n">
-        <v>3800000</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>3800000</v>
+        <v>-19000</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -2355,16 +2355,16 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2374,39 +2374,39 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>113145806</t>
+          <t>278449303</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
+          <t xml:space="preserve">Mấy Xajy Bột Khô Siêu Khỏe 3000W – Bột Mịn Siêu Tốc, Nghiêjn Ngjũ Cốc &amp; Hạt Khô Đa Năng, đèn trang trí   đồng hồ treo tường </t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
+          <t>https://tiki.vn/may-xajy-bot-kho-sieu-khoe-3000w-bot-min-sieu-toc-nghiejn-ngju-coc-hat-kho-da-nang-den-trang-tri-dong-ho-treo-tuong-p278449303.html?spid=278449304</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2415,22 +2415,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>88920</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>117000</v>
+        <v>1288000</v>
       </c>
       <c r="H24" t="n">
-        <v>28080</v>
+        <v>1288000</v>
       </c>
       <c r="I24" t="n">
-        <v>31.58</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2439,58 +2439,58 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="n">
         <v>0</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Giá tăng 28,080đ (+31.6%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>144236336</t>
+          <t>174175573</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>COMBO 5 ÁO LÓT VẢI KHÔNG GỌNG KHÔNG MÚT (SIZE 32-42)</t>
+          <t>Combo sỉ 5 quần lót  nam cao cấp</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-ao-lot-vai-khong-gong-khong-mut-size-32-42-p144236336.html?spid=146366320</t>
+          <t>https://tiki.vn/combo-si-5-quan-lot-nam-cao-cap-p174175573.html?spid=174175578</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2499,22 +2499,22 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>210000</v>
+        <v>150000</v>
       </c>
       <c r="G25" t="n">
-        <v>174300</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>-35700</v>
+        <v>-150000</v>
       </c>
       <c r="I25" t="n">
-        <v>-17</v>
+        <v>-100</v>
       </c>
       <c r="J25" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K25" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2523,79 +2523,79 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q25" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Giá giảm 35,700đ (17.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>276086848</t>
+          <t>113144956</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cục bông trang trí nhiều màu sắc chọn lựa (tùy chọn màu sắc) (hàng có sẵn giao nhanh) (Hàng Chính Hãng)</t>
+          <t>siêu phẩm áo lót nhật trơn đệm nâng ngực nhẹ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cuc-bong-trang-tri-nhieu-mau-sac-chon-lua-tuy-chon-mau-sac-hang-co-san-giao-nhanh-hang-chinh-hang-p276086848.html?spid=276086851</t>
+          <t>https://tiki.vn/sieu-pham-ao-lot-tron-dem-nang-nguc-nhe-p113144956.html?spid=142116876</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bilaha</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>165000</v>
       </c>
       <c r="G26" t="n">
-        <v>70000</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>70000</v>
+        <v>-165000</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -2607,16 +2607,16 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2626,34 +2626,34 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>192642640</t>
+          <t>275738497</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cài tóc bảng nhỏ 1 cm - cài tóc nam nữ - cài tóc đơn giản</t>
+          <t>Mặt Khóa Thắt Lưng Nam Cao Cấp,Mặt Thắt Lưng Nam Khóa Tự Động 203859</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cai-toc-bang-nho-1-cm-cai-toc-nam-nu-cai-toc-don-gian-p192642640.html?spid=192642674</t>
+          <t>https://tiki.vn/mat-khoa-that-lung-nam-cao-cap-mat-that-lung-nam-khoa-tu-dong-203859-p275738497.html?spid=275738498</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2663,26 +2663,26 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>TLG Thành Long</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>24000</v>
+        <v>61400</v>
       </c>
       <c r="G27" t="n">
-        <v>24000</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>-61400</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J27" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="K27" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2694,50 +2694,50 @@
         <v>5</v>
       </c>
       <c r="O27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Review thêm +2</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>38160273</t>
+          <t>126091279</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Giày Boot Nam BIGGBEN Da Bò Thật Cao Cấp BT2</t>
+          <t>Giày Mọi, Giày Lười Nam Da Bò SUNPOLO SU5059 Hiện đại (Đen)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-boot-nam-biggben-da-bo-that-cao-cap-bt2-p38160273.html?spid=38160275</t>
+          <t>https://tiki.vn/giay-moi-giay-luoi-nam-da-bo-sunpolo-su5059-hien-dai-den-p126091279.html?spid=126091289</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2747,23 +2747,23 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>SUNPOLO</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2000000</v>
+        <v>1100000</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>-2000000</v>
+        <v>-1100000</v>
       </c>
       <c r="I28" t="n">
         <v>-100</v>
       </c>
       <c r="J28" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -2775,13 +2775,13 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2811,52 +2811,52 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>278957623</t>
+          <t>274586950</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dép quai kẹp Biti's nam (size 38-43)</t>
+          <t>Set 100 Miếng dán chống mồ hôi nách, miếng dán ngăn mồ hôi nách siêu thâm hút cho Nam và Nữ che tên sản phẩm</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-quai-kep-biti-s-nam-size-38-43-p278957623.html?spid=278957641</t>
+          <t>https://tiki.vn/set-100-mieng-dan-chong-mo-hoi-nach-mieng-dan-ngan-mo-hoi-nach-sieu-tham-hut-cho-nam-va-nu-che-ten-san-pham-p274586950.html?spid=274586956</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Biti's</t>
+          <t>FTAKY</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>232000</v>
+        <v>199000</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>99000</v>
       </c>
       <c r="H29" t="n">
-        <v>-232000</v>
+        <v>-100000</v>
       </c>
       <c r="I29" t="n">
-        <v>-100</v>
+        <v>-50.25</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>-198000</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -2878,521 +2878,101 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá giảm 100,000đ (50.3%) | Bán thêm -2 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>276827848</t>
+          <t>49733157</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Quần Jean Ống Rộng Classic Carolina Blue Aaa Jeans</t>
+          <t>Quần bơi nam giới dáng vừa, độ dài trên gối, chất thun bơi lạnh dày đẹp, co giãn 4 chiều ôm đùi gọn gàng dễ chịu, thoáng mát nhanh khô | BN005</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-jean-o-ng-rong-classic-carolina-blue-aaa-jeans-p276827848.html?spid=276827850</t>
+          <t>https://tiki.vn/quan-boi-nam-dang-lung-mau-moi-2020-vai-boi-day-dan-dep-co-gian-4-chieu-bn005-p49733157.html?spid=49733161</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TRIPLE A</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>650000</v>
+        <v>115000</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>115000</v>
       </c>
       <c r="H30" t="n">
-        <v>-650000</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>-920000</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="O30" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="P30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="S30" t="n">
         <v>0</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>277744886</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Giày Da Nam Italy - 1720BIA</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/giay-da-nam-italy-1720bia-p277744886.html?spid=277744894</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Gianni Conti</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>-4000000</v>
-      </c>
-      <c r="I31" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>278449303</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mấy Xajy Bột Khô Siêu Khỏe 3000W – Bột Mịn Siêu Tốc, Nghiêjn Ngjũ Cốc &amp; Hạt Khô Đa Năng, đèn trang trí   đồng hồ treo tường </t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/may-xajy-bot-kho-sieu-khoe-3000w-bot-min-sieu-toc-nghiejn-ngju-coc-hat-kho-da-nang-den-trang-tri-dong-ho-treo-tuong-p278449303.html?spid=278449304</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>1288000</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>-1288000</v>
-      </c>
-      <c r="I32" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>68491184</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Kính râm Nam thời trang + Tặng Tuavit Kính Xinh Mini đa năng</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/kinh-ram-nam-thoi-trang-tang-tuavit-kinh-xinh-mini-da-nang-p68491184.html?spid=68491185</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>HOKO</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>169000</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>-169000</v>
-      </c>
-      <c r="I33" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J33" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>272224450</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Dép quai ngang nam, nữ siêu nhẹ DUWA - Hàng chính hãng - TK9056</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/dep-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk9056-p272224450.html?spid=272224458</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>DUWA</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>159000</v>
-      </c>
-      <c r="G34" t="n">
-        <v>159000</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" t="n">
-        <v>2</v>
-      </c>
-      <c r="L34" t="n">
-        <v>-2</v>
-      </c>
-      <c r="M34" t="n">
-        <v>-318000</v>
-      </c>
-      <c r="N34" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="O34" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>2</v>
-      </c>
-      <c r="R34" t="n">
-        <v>2</v>
-      </c>
-      <c r="S34" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>Bán thêm -2 sản phẩm</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>278000485</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Áo lót nữ 718 – Mút mỏng thông hơi, không gọng, cài sau 3 móc, co giãn thoải mái</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-lot-nu-718-mut-mong-thong-hoi-khong-gong-cai-sau-3-moc-co-gian-thoai-mai-p278000485.html?spid=278000517</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>100000</v>
-      </c>
-      <c r="G35" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>9</v>
-      </c>
-      <c r="K35" t="n">
-        <v>5</v>
-      </c>
-      <c r="L35" t="n">
-        <v>-4</v>
-      </c>
-      <c r="M35" t="n">
-        <v>-400000</v>
-      </c>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>Bán thêm -4 sản phẩm</t>
+          <t>Bán thêm -8 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-07-12
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V31"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,17 +543,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>132230478</t>
+          <t>7997300</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Giày Lười Nam Da Bò SUNPOLO CS5054 Trẻ trung, thanh lịch (Đen, Nâu)</t>
+          <t>Giày Converse Chuck Taylor All Star 1970s Hi Top - 162050V</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-luoi-nam-da-bo-sunpolo-cs5054-tre-trung-thanh-lich-den-nau-p132230478.html?spid=132230492</t>
+          <t>https://tiki.vn/giay-converse-chuck-taylor-all-star-1970s-hi-top-162050v-p7997300.html?spid=13727356</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SUNPOLO</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1100000</v>
+        <v>2000000</v>
       </c>
       <c r="H2" t="n">
-        <v>1100000</v>
+        <v>2000000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,35 +582,35 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>16</v>
+        <v>200</v>
       </c>
       <c r="L2" t="n">
-        <v>16</v>
+        <v>200</v>
       </c>
       <c r="M2" t="n">
-        <v>17600000</v>
+        <v>400000000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="P2" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="S2" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -627,37 +627,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>197062475</t>
+          <t>7995370</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Áo khoác măng tô nam cổ đứng dáng ngắn khóa kéo chất vải kaki đẹp NMT34</t>
+          <t>Giày Converse Chuck Taylor All Star Classic Hi Top - 121186</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-khoac-mang-to-nam-co-dung-dang-ngan-khoa-keo-chat-vai-kaki-dep-nmt34-p197062475.html?spid=197062507</t>
+          <t>https://tiki.vn/giay-converse-chuck-taylor-all-star-classic-hi-top-121186-p7995370.html?spid=20315038</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>936000</v>
+        <v>1550000</v>
       </c>
       <c r="H3" t="n">
-        <v>936000</v>
+        <v>1550000</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,35 +666,35 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>92</v>
       </c>
       <c r="L3" t="n">
-        <v>7</v>
+        <v>92</v>
       </c>
       <c r="M3" t="n">
-        <v>6552000</v>
+        <v>142600000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P3" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -711,37 +711,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>270474726</t>
+          <t>96301779</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bộ đồ bơi nam ngắn tay + quần boxer 2 lớp, họa tiết mạnh mẽ, set quần áo đi biển, đi bơi cho nam giới, chất thun bơi dày dặn mịn mát đẹp | BN031</t>
+          <t>Dép Bít Mũi Nam HÀ NAM Da Bò Thật Cao Cấp GSB2068</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-do-boi-nam-ngan-tay-quan-boxer-2-lop-hoa-tiet-manh-me-set-quan-ao-di-bien-di-boi-cho-nam-gioi-chat-thun-boi-day-dan-min-mat-dep-bn031-p270474726.html?spid=275928740</t>
+          <t>https://tiki.vn/dep-bit-mui-nam-sabo-nam-da-bo-that-de-cao-su-gsb2068-p96301779.html?spid=96301783</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>HA NAM</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>420000</v>
+        <v>468000</v>
       </c>
       <c r="H4" t="n">
-        <v>420000</v>
+        <v>468000</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -750,35 +750,35 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M4" t="n">
-        <v>3780000</v>
+        <v>5148000</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P4" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="S4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -795,37 +795,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>55953905</t>
+          <t>13307720</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Giày tây tăng chiều cao Trường Hải da bò cao cấp cao 6.5 cm trường Hải GTN0125</t>
+          <t>Combo 10 Quần lót nam, sịp chéo nam xuất Nhật thời trang cao cấp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-tang-chieu-cao-truong-hai-da-bo-cao-cap-cao-6-5-cm-de-cao-su-giay-duoc-gia-cong-tai-xuong-truong-hai-gtn0125-p55953905.html?spid=55953907</t>
+          <t>https://tiki.vn/combo-10-quan-lot-nam-sip-cheo-nam-xuat-nhat-thoi-trang-cao-cap-p13307720.html?spid=278703711</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Trường Hải</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>645000</v>
+        <v>336000</v>
       </c>
       <c r="H5" t="n">
-        <v>645000</v>
+        <v>336000</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -834,13 +834,13 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M5" t="n">
-        <v>2580000</v>
+        <v>2688000</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -855,14 +855,14 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -879,37 +879,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>48310107</t>
+          <t>193095213</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Giày Mọi Nam Da Bò BIGGBEN GM219</t>
+          <t>Kính Râm Kính Mát Nam Nữ TF Mắt To Gọng Nhựa Dẻo TR90 Mắt Màu Vàng, Xanh Dương, Đen Chống Tia UV - BLUE LIGHT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-moi-nam-da-bo-biggben-gm219-p48310107.html?spid=48310111</t>
+          <t>https://tiki.vn/kinh-ram-kinh-mat-nam-nu-tf-mat-to-gong-nhua-deo-tr90-mat-mau-vang-xanh-duong-den-chong-tia-uv-blue-light-p193095213.html?spid=193095217</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>Blue Light</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>800000</v>
+        <v>185000</v>
       </c>
       <c r="H6" t="n">
-        <v>800000</v>
+        <v>185000</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -918,35 +918,35 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="L6" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M6" t="n">
-        <v>2400000</v>
+        <v>2035000</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -963,37 +963,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>107491961</t>
+          <t>277877891</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dép Nam Quai Ngang Da Bò BIGGBEN Cao Cấp DN283</t>
+          <t>Móc Nối Tăng Size Áo Ngực 3 Móc 59S – Phụ Kiện Nới Rộng Bra Linh Hoạt</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-biggben-cao-cap-dn283-p107491961.html?spid=107491981</t>
+          <t>https://tiki.vn/moc-noi-tang-size-ao-nguc-3-moc-59s-phu-kien-noi-rong-bra-linh-hoat-p277877891.html?spid=277877895</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>395000</v>
+        <v>20000</v>
       </c>
       <c r="H7" t="n">
-        <v>395000</v>
+        <v>20000</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1002,35 +1002,35 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
+        <v>19</v>
+      </c>
+      <c r="L7" t="n">
+        <v>19</v>
+      </c>
+      <c r="M7" t="n">
+        <v>380000</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4</v>
+      </c>
+      <c r="P7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
         <v>1</v>
       </c>
-      <c r="L7" t="n">
+      <c r="S7" t="n">
         <v>1</v>
       </c>
-      <c r="M7" t="n">
-        <v>395000</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1047,34 +1047,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>114739740</t>
+          <t>113215403</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cột tóc srunchies mẫu mới màu hồng phấn đẹp</t>
+          <t>Lót giày vải lưới Hương Quế, quế thật, quế thơm, tốt cho sức khỏe</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cot-toc-srunchies-mau-moi-mau-hong-phan-dep-p114739740.html?spid=114739748</t>
+          <t>https://tiki.vn/lot-giay-vai-luoi-huong-que-que-that-que-thom-tot-cho-suc-khoe-p113215403.html?spid=113215415</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Hương quế</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>25000</v>
+        <v>38000</v>
       </c>
       <c r="G8" t="n">
-        <v>25000</v>
+        <v>38000</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1083,38 +1083,38 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="K8" t="n">
-        <v>220</v>
+        <v>184</v>
       </c>
       <c r="L8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M8" t="n">
-        <v>250000</v>
+        <v>190000</v>
       </c>
       <c r="N8" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="O8" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="R8" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1124,125 +1124,125 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Bán thêm +10 sản phẩm</t>
+          <t>Bán thêm +5 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>199607832</t>
+          <t>19843976</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combo 4 Quần Lót Ren Miley Lingerie Màu Trắng Đen - FLS03</t>
+          <t>Combo 10 Đôi Tất Nam Chống Hôi Chân Thời Trang</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-4-quan-lot-ren-miley-lingerie-mau-trang-den-fls03-p199607832.html?spid=199607836</t>
+          <t>https://tiki.vn/combo-10-doi-tat-nam-chong-hoi-chan-thoi-trang-p19843976.html?spid=71526312</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Miley Lingerie</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>79000</v>
       </c>
       <c r="G9" t="n">
-        <v>216000</v>
+        <v>79000</v>
       </c>
       <c r="H9" t="n">
-        <v>216000</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>378</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>216000</v>
+        <v>79000</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Bán thêm +1 sản phẩm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>67538621</t>
+          <t>212471303</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Combo 5 quần ĐÙI May 10 giao màu ngẫu nhiên</t>
+          <t>Sét 8 Kẹp Tóc Size To Phong Cách Hàn Quốc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-quan-dui-may-10-p67538621.html?spid=67538623</t>
+          <t>https://tiki.vn/set-8-kep-toc-size-to-phong-cach-han-quoc-p212471303.html?spid=212471304</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>May 10</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>135000</v>
+        <v>59000</v>
       </c>
       <c r="G10" t="n">
-        <v>135000</v>
+        <v>59000</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1251,38 +1251,38 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>16601</v>
+        <v>13</v>
       </c>
       <c r="K10" t="n">
-        <v>16602</v>
+        <v>14</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>135000</v>
+        <v>59000</v>
       </c>
       <c r="N10" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="O10" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>4843</v>
+        <v>2</v>
       </c>
       <c r="R10" t="n">
-        <v>4843</v>
+        <v>2</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1299,142 +1299,142 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19843976</t>
+          <t>278704460</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Combo 10 Đôi Tất Nam Chống Hôi Chân Thời Trang</t>
+          <t>Áo Thun Basic Tay Ngắn Nam Ninomaxx 2505012</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-10-doi-tat-nam-chong-hoi-chan-thoi-trang-p19843976.html?spid=71526312</t>
+          <t>https://tiki.vn/ao-thun-basic-tay-ngan-nam-ninomaxx-2505012-p278704460.html?spid=278704476</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ninomaxx</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>79000</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>79000</v>
+        <v>269000</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>269000</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>376</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>377</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>79000</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>187249357</t>
+          <t>16651795</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cặp Cài Tai Giữ Mắt Kính Bằng Silicon Chống Trượt Tiện Dụng</t>
+          <t>️[5 Quần] ComBo 5 Quần Lót Nam THUN LẠNH Lưng Bự Hàng Việt Nam Cao Cấp</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cap-cai-tai-giu-mat-kinh-bang-silicon-chong-truot-tien-dung-p187249357.html?spid=187249358</t>
+          <t>https://tiki.vn/5-quan-combo-5-quan-lot-nam-thun-lanh-lung-bu-hang-viet-nam-cao-cap-p16651795.html?spid=51148102</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OURESS</t>
+          <t>MENLIVE</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>10000</v>
+        <v>190000</v>
       </c>
       <c r="G12" t="n">
-        <v>10000</v>
+        <v>159600</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>-30400</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="J12" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="K12" t="n">
-        <v>88</v>
+        <v>9</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,29 +1460,29 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Bán thêm +3 sản phẩm</t>
+          <t>Giá giảm 30,400đ (16.0%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>83423370</t>
+          <t>16546849</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bộ dụng cụ tua vít đa năng sửa kính, mắt kính</t>
+          <t>Combo 5 Quần Lót Nam Tam Giác Nhật</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-dung-cu-tua-vit-da-nang-sua-kinh-mat-kinh-p83423370.html?spid=113070838</t>
+          <t>https://tiki.vn/combo-5-quan-lot-nam-tam-giac-nhat-p16546849.html?spid=53006035</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1491,50 +1491,50 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9500</v>
+        <v>210000</v>
       </c>
       <c r="G13" t="n">
-        <v>9500</v>
+        <v>170100</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>-39900</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>-19</v>
       </c>
       <c r="J13" t="n">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="K13" t="n">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>9500</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="O13" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="R13" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,24 +1544,24 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Bán thêm +1 sản phẩm</t>
+          <t>Giá giảm 39,900đ (19.0%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>277996544</t>
+          <t>54569520</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hộp 5 Quần lót nam cotton lụa – Siêu đẹp, mềm mịn, thoáng mát</t>
+          <t>Quần Lót nam, quần sịp nam lụa Sữa Cao Cấp sp-340</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-5-quan-lot-nam-cotton-lua-muji-sieu-dep-mem-min-thoang-mat-p277996544.html?spid=278006734</t>
+          <t>https://tiki.vn/quan-lot-nam-quan-sip-nam-lua-sua-cao-cap-sp-340-p54569520.html?spid=67859897</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1575,22 +1575,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>220000</v>
+        <v>67760</v>
       </c>
       <c r="G14" t="n">
-        <v>169400</v>
+        <v>88000</v>
       </c>
       <c r="H14" t="n">
-        <v>-50600</v>
+        <v>20240</v>
       </c>
       <c r="I14" t="n">
-        <v>-23</v>
+        <v>29.87</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1608,17 +1608,17 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1628,24 +1628,24 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Giá giảm 50,600đ (23.0%)</t>
+          <t>Giá tăng 20,240đ (+29.9%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>278021672</t>
+          <t>127197643</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Quần Lót Nam Đùi Boxer Lụa Băng Menpro MP9 - Mỏng nhem Thoáng Khí</t>
+          <t>Bộ Quần Áo Nam Lính Mỹ US ARMY  Kiểu Dáng Túi Hộp, Chất Liệu Kaki Cao Cấp Phong Cách Lính Cực Ngầu (Tặng dây lưng) - HÀNG CHÍNH HÃNG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-nam-dui-boxer-lua-bang-menpro-mp9-mong-nhem-thoang-khi-p278021672.html?spid=278021690</t>
+          <t>https://tiki.vn/bo-quan-ao-nam-linh-my-us-army-kieu-dang-tui-hop-chat-lieu-kaki-cao-cap-phong-cach-linh-cuc-ngau-tang-day-lung-hang-chinh-hang-p127197643.html?spid=182094568</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1655,26 +1655,26 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>US ARMY</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>79000</v>
+        <v>899000</v>
       </c>
       <c r="G15" t="n">
-        <v>63200</v>
+        <v>899000</v>
       </c>
       <c r="H15" t="n">
-        <v>-15800</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1683,26 +1683,26 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1712,53 +1712,53 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Giá giảm 15,800đ (20.0%)</t>
+          <t>Review thêm +1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>262817701</t>
+          <t>103049077</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Giày Mọi Nam Đế Âm Da Bò Thật TiTi ĐÔ Cao Cấp GDA2021</t>
+          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-moi-nam-de-am-titi-do-da-bo-that-cao-cap-gda2021-p262817701.html?spid=262817709</t>
+          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HA NAM</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>153550</v>
       </c>
       <c r="G16" t="n">
-        <v>760000</v>
+        <v>185000</v>
       </c>
       <c r="H16" t="n">
-        <v>760000</v>
+        <v>31450</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>20.48</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -1767,58 +1767,58 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 31,450đ (+20.5%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>59462352</t>
+          <t>16375016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Áo ngực mỏng thêu hoa cài trước có gọng</t>
+          <t>COMBO HỘP 5 Quần Lót ĐÙI Nam Xuất Nhật Cao Cấp (MIX NGẪU NHIÊN)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-nguc-mong-theu-hoa-cai-truoc-co-gong-p59462352.html?spid=59462384</t>
+          <t>https://tiki.vn/combo-hop-5-quan-lot-dui-nam-xuat-nhat-cao-cap-mix-ngau-nhien-p16375016.html?spid=277961877</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1827,22 +1827,22 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>90000</v>
+        <v>274000</v>
       </c>
       <c r="G17" t="n">
-        <v>90000</v>
+        <v>210980</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>-63020</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>-23</v>
       </c>
       <c r="J17" t="n">
-        <v>204</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>204</v>
+        <v>3</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,26 +1851,26 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1880,53 +1880,53 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Review thêm +5</t>
+          <t>Giá giảm 63,020đ (23.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>279104033</t>
+          <t>278850221</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Áo lót nữ form ba lỗ thông hơi trơn big size 1397 – Size XXL–3XL</t>
+          <t>Quần Jean Thời Trang Basic Nam Ống Đứng Ninomaxx 2508004</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-form-ba-lo-thong-hoi-tron-big-size-1397-size-xxl-3xl-p279104033.html?spid=279104035</t>
+          <t>https://tiki.vn/quan-jean-thoi-trang-basic-nam-ong-dung-ninomaxx-2508004-p278850221.html?spid=278850229</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Ninomaxx</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>108000</v>
+        <v>769000</v>
       </c>
       <c r="G18" t="n">
-        <v>86400</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>-21600</v>
+        <v>-769000</v>
       </c>
       <c r="I18" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="J18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1935,82 +1935,82 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá giảm 21,600đ (20.0%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>91973812</t>
+          <t>274795145</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Áo Lót Nữ Su Đúc Hình Lá Không Gọng Đệm Dày Nâng Ngực A01 có ảnh thật</t>
+          <t>Dép tổ ong [Size 39-43] KÈM STICKER NGẪU NHIÊN vật liệu EVA cao cấp siêu bền, siêu nhẹ, chống trơn trượt</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-su-duc-hinh-la-khong-gong-dem-day-nang-nguc-a01-co-anh-that-p91973812.html?spid=279055013</t>
+          <t>https://tiki.vn/dep-to-ong-size-39-43-kem-sticker-ngau-nhien-vat-lieu-eva-cao-cap-sieu-ben-sieu-nhe-chong-tron-truot-p274795145.html?spid=274803712</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t xml:space="preserve">VAC </t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>85000</v>
+        <v>83000</v>
       </c>
       <c r="G19" t="n">
-        <v>68000</v>
+        <v>100000</v>
       </c>
       <c r="H19" t="n">
-        <v>-17000</v>
+        <v>17000</v>
       </c>
       <c r="I19" t="n">
-        <v>-20</v>
+        <v>20.48</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,26 +2019,26 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2048,53 +2048,53 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá giảm 17,000đ (20.0%)</t>
+          <t>Giá tăng 17,000đ (+20.5%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>278850221</t>
+          <t>73862702</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Quần Jean Thời Trang Basic Nam Ống Đứng Ninomaxx 2508004</t>
+          <t>ÁO LÓT NỮ REN MÚT DÀY 2CM DÂY TRƠN NÂNG NGỰC 024B</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-jean-thoi-trang-basic-nam-ong-dung-ninomaxx-2508004-p278850221.html?spid=278850229</t>
+          <t>https://tiki.vn/ao-lot-nu-ren-mut-day-2cm-day-tron-nang-nguc-024b-p73862702.html?spid=73862720</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ninomaxx</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>140130</v>
       </c>
       <c r="G20" t="n">
-        <v>769000</v>
+        <v>173000</v>
       </c>
       <c r="H20" t="n">
-        <v>769000</v>
+        <v>32870</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>23.46</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -2103,82 +2103,82 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 32,870đ (+23.5%)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>55139307</t>
+          <t>37126497</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Giày Tây Nam Da Bò BIGGBEN Cao Cấp GT179</t>
+          <t>( 10 cái ) quần lót nữ Su đúc không đường may, hàng đẹp loại xịn W19_503</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/giay-tay-nam-da-bo-biggben-cao-cap-gt179-p55139307.html?spid=55139313</t>
+          <t>https://tiki.vn/set-10-quan-lot-su-duc-khong-duong-may-hang-dep-loai-xin-w19_503-p37126497.html?spid=51720423</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BIGGBEN</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>280000</v>
       </c>
       <c r="G21" t="n">
-        <v>670000</v>
+        <v>210000</v>
       </c>
       <c r="H21" t="n">
-        <v>670000</v>
+        <v>-70000</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>-25</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2187,58 +2187,58 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 70,000đ (25.0%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>172474530</t>
+          <t>74421501</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Quần short thun nam cao cấp, quần short nam vải cotton LN058</t>
+          <t>ÁO LÓT NỮ MỎNG CÓ GỌNG CÀI TRƯỚC VIỀN REN</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-short-thun-nam-cao-cap-quan-short-nam-vai-cotton-ln058-p172474530.html?spid=276662143</t>
+          <t>https://tiki.vn/ao-lot-nu-mong-co-gong-cai-truoc-vien-ren-p74421501.html?spid=74421553</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2247,22 +2247,22 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>85000</v>
+        <v>129600</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>160000</v>
       </c>
       <c r="H22" t="n">
-        <v>-85000</v>
+        <v>30400</v>
       </c>
       <c r="I22" t="n">
-        <v>-100</v>
+        <v>23.46</v>
       </c>
       <c r="J22" t="n">
-        <v>4</v>
+        <v>153</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -2271,76 +2271,76 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="P22" t="n">
-        <v>-4.6</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="S22" t="n">
         <v>0</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá tăng 30,400đ (+23.5%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>278704460</t>
+          <t>277586478</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Áo Thun Basic Tay Ngắn Nam Ninomaxx 2505012</t>
+          <t>Dép nam quai ngang da thật BHD2512 Dép nam trung niên</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-basic-tay-ngan-nam-ninomaxx-2505012-p278704460.html?spid=278704476</t>
+          <t>https://tiki.vn/dep-nam-quai-ngang-da-that-bhd2512-dep-nam-trung-nien-p277586478.html?spid=277586488</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ninomaxx</t>
+          <t>MARRANT</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>269000</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>299000</v>
       </c>
       <c r="H23" t="n">
-        <v>-269000</v>
+        <v>299000</v>
       </c>
       <c r="I23" t="n">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -2374,39 +2374,39 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13307720</t>
+          <t>140429170</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Combo 10 Quần lót nam, sịp chéo nam xuất Nhật thời trang cao cấp</t>
+          <t>Bao tay chơi game găng tay 2 ngón cảm ứng điện thoại gamemobile BT01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-10-quan-lot-nam-sip-cheo-nam-xuat-nhat-thoi-trang-cao-cap-p13307720.html?spid=278703711</t>
+          <t>https://tiki.vn/bao-tay-choi-game-gang-tay-2-ngon-cam-ung-dien-thoai-gamemobile-bt01-p140429170.html?spid=198934954</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2415,22 +2415,22 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>420000</v>
+        <v>9999</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>19999</v>
       </c>
       <c r="H24" t="n">
-        <v>-420000</v>
+        <v>10000</v>
       </c>
       <c r="I24" t="n">
-        <v>-100</v>
+        <v>100.01</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2439,16 +2439,16 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2458,54 +2458,54 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>❌ Đã xóa</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Không còn xuất hiện trong danh sách</t>
+          <t>Giá tăng 10,000đ (+100.0%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>279345710</t>
+          <t>87670339</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Áo thun nữ Ruzimay RA2000 lệch vai co giãn mềm mại thanh lịch</t>
+          <t>Áo Khoác Dù 2 Mặt Cao Cấp Chống Thấm</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-nu-ruzimay-ra2000-lech-vai-co-gian-mem-mai-thanh-lich-p279345710.html?spid=279345726</t>
+          <t>https://tiki.vn/ao-khoac-du-2-mat-cao-cap-chong-tham-p87670339.html?spid=113225543</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ruzimay Style</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>212000</v>
+        <v>317035</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>-212000</v>
+        <v>-317035</v>
       </c>
       <c r="I25" t="n">
         <v>-100</v>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -2559,17 +2559,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>272224450</t>
+          <t>7995659</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dép quai ngang nam, nữ siêu nhẹ DUWA - Hàng chính hãng - TK9056</t>
+          <t>Giày Converse Chuck Taylor All Star Classic Low Top - 121176</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk9056-p272224450.html?spid=272224470</t>
+          <t>https://tiki.vn/giay-converse-chuck-taylor-all-star-classic-low-top-121176-p7995659.html?spid=20340964</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2579,23 +2579,23 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>159000</v>
+        <v>1450000</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>-159000</v>
+        <v>-1450000</v>
       </c>
       <c r="I26" t="n">
         <v>-100</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -2607,16 +2607,16 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>-4.5</v>
+        <v>-4.8</v>
       </c>
       <c r="Q26" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2643,43 +2643,43 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>217139643</t>
+          <t>46773376</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dép quai ngang nam nữ siêu nhẹ DUWA - Hàng chính hãng - TK9048</t>
+          <t>Áo Ngực Tạo 7 Kiểu Mặc Multiway Cực Phong Cách Và Nâng Ngực Siêu Hít AL07</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk9048-p217139643.html?spid=217139655</t>
+          <t>https://tiki.vn/ao-nguc-tao-7-kieu-mac-multiway-cuc-phong-cach-va-nang-nguc-sieu-hit-al07-p46773376.html?spid=52950082</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>159000</v>
+        <v>100000</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>-159000</v>
+        <v>-100000</v>
       </c>
       <c r="I27" t="n">
         <v>-100</v>
       </c>
       <c r="J27" t="n">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -2691,16 +2691,16 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>-4.7</v>
+        <v>-5</v>
       </c>
       <c r="Q27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2727,17 +2727,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>202048399</t>
+          <t>7997276</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dép quai ngang nam, nữ siêu nhẹ DUWA - Hàng chính hãng - TK9045</t>
+          <t>Giày Sneaker Unisex Converse Chuck Taylor All Star 1970s All Hi 2018 - White (Size</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk9045-p202048399.html?spid=202048466</t>
+          <t>https://tiki.vn/giay-sneaker-unisex-converse-chuck-taylor-all-star-1970s-all-white-hi-2018-p7997276.html?spid=26499478</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2747,23 +2747,23 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>Converse</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>159000</v>
+        <v>2000000</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>-159000</v>
+        <v>-2000000</v>
       </c>
       <c r="I28" t="n">
         <v>-100</v>
       </c>
       <c r="J28" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -2784,7 +2784,7 @@
         <v>-5</v>
       </c>
       <c r="Q28" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2811,17 +2811,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>194131743</t>
+          <t>9810961</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dép đúc quai ngang nam, nữ siêu nhẹ DUWA - Hàng chính hãng - TK193</t>
+          <t>Giày Slip On Unisex Vans - VN000EYEBWW</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-duc-quai-ngang-nam-nu-sieu-nhe-duwa-hang-chinh-hang-tk193-p194131743.html?spid=194131775</t>
+          <t>https://tiki.vn/giay-slip-on-unisex-vans-vn000eyebww-p9810961.html?spid=23839235</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2831,23 +2831,23 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>179000</v>
+        <v>1450000</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>-179000</v>
+        <v>-1450000</v>
       </c>
       <c r="I29" t="n">
         <v>-100</v>
       </c>
       <c r="J29" t="n">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -2859,16 +2859,16 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>-4.8</v>
+        <v>-5</v>
       </c>
       <c r="Q29" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2895,43 +2895,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>273466355</t>
+          <t>278994189</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dép xỏ ngón nam, nữ đúc liền khối siêu nhẹ DUWA - Hàng chính hãng - TK288</t>
+          <t>Áo thun tay ngắn nam patch ngực Form Fitted - ROUTINE 10F25TSS003</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-xo-ngon-nam-nu-duc-lien-khoi-sieu-nhe-duwa-hang-chinh-hang-tk288-p273466355.html?spid=273466357</t>
+          <t>https://tiki.vn/ao-thun-tay-ngan-nam-patch-nguc-form-fitted-routine-10f25tss003-p278994189.html?spid=278994205</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>Routine</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>129000</v>
+        <v>349000</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>-129000</v>
+        <v>-349000</v>
       </c>
       <c r="I30" t="n">
         <v>-100</v>
       </c>
       <c r="J30" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -2943,16 +2943,16 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>-4.6</v>
+        <v>-0</v>
       </c>
       <c r="Q30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -2979,17 +2979,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>270791815</t>
+          <t>9810794</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dép đúc siêu nhẹ nam, nữ DUWA - Hàng chính hãng - TK2272</t>
+          <t>Giày Slip On Unisex Vans - VN000EYEBLK</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-duc-sieu-nhe-nam-nu-duwa-hang-chinh-hang-tk2272-p270791815.html?spid=270791831</t>
+          <t>https://tiki.vn/giay-slip-on-unisex-vans-vn000eyeblk-p9810794.html?spid=20459574</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2999,23 +2999,23 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>DUWA</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>159000</v>
+        <v>1450000</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>-159000</v>
+        <v>-1450000</v>
       </c>
       <c r="I31" t="n">
         <v>-100</v>
       </c>
       <c r="J31" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3057,6 +3057,174 @@
       <c r="V31" t="inlineStr">
         <is>
           <t>Không còn xuất hiện trong danh sách</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>72050932</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Khẩu Trang Pitta Nhật Bản Small Chic - Gói 3 cái (mẫu mới 2020)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/khau-trang-pitta-nhat-ban-small-chic-goi-3-cai-mau-moi-2020-p72050932.html?spid=72050933</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Phụ kiện thời trang</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PITTA MASK</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>180000</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-180000</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-100</v>
+      </c>
+      <c r="J32" t="n">
+        <v>49</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>5</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>-5</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>7</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>❌ Đã xóa</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Không còn xuất hiện trong danh sách</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>275276395</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Dép tổ ong TRẮNG nhựa EVA siêu bền, siêu nhẹ, chống trơn trượt, đế dày (FORM LỚN ĐẶT LÙI 1-2 SIZE) Dép Nam Nữ Nhiều Màu Sắc</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://tiki.vn/dep-to-ong-trangvat-lieu-eva-sieu-ben-sieu-nhe-chong-tron-truot-form-size-lon-chau-au-p275276395.html?spid=275276411</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Giày - Dép nam</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VAC </t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G33" t="n">
+        <v>85000</v>
+      </c>
+      <c r="H33" t="n">
+        <v>13000</v>
+      </c>
+      <c r="I33" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="J33" t="n">
+        <v>45</v>
+      </c>
+      <c r="K33" t="n">
+        <v>30</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-15</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-1275000</v>
+      </c>
+      <c r="N33" t="n">
+        <v>5</v>
+      </c>
+      <c r="O33" t="n">
+        <v>5</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>3</v>
+      </c>
+      <c r="R33" t="n">
+        <v>3</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>🔄 Đã cập nhật</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Giá tăng 13,000đ (+18.1%) | Bán thêm -15 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bot tu dong cap nhat ngay 2026-07-31
</commit_message>
<xml_diff>
--- a/tiki_changes_report.xlsx
+++ b/tiki_changes_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,37 +543,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>275276504</t>
+          <t>186434946</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Đồ Bơi Nữ Hai Mảnh Đa Năng Gồm Áo Bơi Nữ Và Váy Bơi Nữ</t>
+          <t>Túi than hoạt tính khử mùi giày - 100% từ gáo dừa Bến Tre (Hộp 2 túi) - Hapaku</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tiki.vn/do-boi-nu-hai-manh-da-nang-gom-ao-boi-nu-va-vay-boi-nu-p275276504.html?spid=275276510</t>
+          <t>https://tiki.vn/tui-than-hoat-tinh-khu-mui-giay-100-tu-gao-dua-ben-tre-hop-2-tui-hapaku-p186434946.html?spid=29882855</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Hapaku</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>219000</v>
+        <v>129000</v>
       </c>
       <c r="H2" t="n">
-        <v>219000</v>
+        <v>129000</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -582,35 +582,35 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="L2" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="M2" t="n">
-        <v>3066000</v>
+        <v>22188000</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="P2" t="n">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -627,37 +627,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>27924842</t>
+          <t>278049759</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cài áo hoa vải</t>
+          <t>Áo sơ mi nam ngắn tay Novelty Casual Hoa văn SMI25001 - 250079N</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://tiki.vn/cai-ao-hoa-vai-p27924842.html?spid=27924852</t>
+          <t>https://tiki.vn/ao-so-mi-nam-ngan-tay-novelty-casual-hoa-van-smi25001-p278049759.html?spid=278049917</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Novelty</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>395000</v>
       </c>
       <c r="G3" t="n">
-        <v>35000</v>
+        <v>395000</v>
       </c>
       <c r="H3" t="n">
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -666,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>1470000</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -694,34 +694,34 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Rating 0.0→5.0 (+5.00) | Review thêm +4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>278092142</t>
+          <t>174585329</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Quần kiểu nữ ống rộng, chất liệu vải Đũi xước, mềm mịn, mặc mát, Quần Short nữ đẹp Nesa Shop</t>
+          <t>Áo lót nâng ngực boya mút mỏng, Áo ngực boya nâng ngực cài sau 522BT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-kieu-nu-ong-rong-chat-lieu-vai-dui-xuoc-mem-min-mac-mat-quan-short-nu-dep-nesa-shop-p278092142.html?spid=278092148</t>
+          <t>https://tiki.vn/ao-lot-nang-nguc-boya-mut-mong-ao-nguc-boya-nang-nguc-cai-sau-522bt-p174585329.html?spid=203717976</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -735,50 +735,50 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>55000</v>
+        <v>86100</v>
       </c>
       <c r="G4" t="n">
-        <v>55000</v>
+        <v>105000</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>18900</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>21.95</v>
       </c>
       <c r="J4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>660000</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="O4" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -788,137 +788,137 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Bán thêm +12 sản phẩm</t>
+          <t>Giá tăng 18,900đ (+22.0%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37733512</t>
+          <t>133160820</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sét 2 kẹp tóc nhựa bền Song An Eco KAH118</t>
+          <t>Quần Lót Su Đúc Nữ (Hàng Loại 1) Không Đường Mai, Thun Lạnh, SIêu Co Dãn, Được Chọn Màu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://tiki.vn/set-2-kep-toc-nhua-ben-song-an-eco-kah118-p37733512.html?spid=37831891</t>
+          <t>https://tiki.vn/quan-lot-su-duc-nu-hang-loai-1-khong-duong-mai-thun-lanh-sieu-co-dan-duoc-chon-mau-p133160820.html?spid=198901960</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Phụ kiện thời trang</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Song An Eco</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>28000</v>
       </c>
       <c r="G5" t="n">
-        <v>22000</v>
+        <v>21840</v>
       </c>
       <c r="H5" t="n">
-        <v>22000</v>
+        <v>-6160</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>-22</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="L5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>176000</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O5" t="n">
         <v>5</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá giảm 6,160đ (22.0%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>276882727</t>
+          <t>158732070</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Áo vest blazer nam phong cách Hàn Quốc vải Linen thoáng mát, mềm mịn</t>
+          <t>❈✣♚Combo 10 quần lót nữ su đúc cao cấp không đường may, chất mát lạnh, mềm mịn, thoáng</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-vest-blazer-nam-phong-cach-han-quoc-vai-linen-thoang-mat-mem-min-p276882727.html?spid=276882729</t>
+          <t>https://tiki.vn/combo-10-quan-lot-nu-su-duc-cao-cap-khong-duong-may-chat-mat-lanh-mem-min-thoang-p158732070.html?spid=242324041</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Haint Boutique</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>252800</v>
       </c>
       <c r="G6" t="n">
-        <v>420000</v>
+        <v>320000</v>
       </c>
       <c r="H6" t="n">
-        <v>420000</v>
+        <v>67200</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>26.58</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -927,58 +927,58 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>🔄 Đã cập nhật</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Giá tăng 67,200đ (+26.6%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>133160820</t>
+          <t>103049077</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Quần Lót Su Đúc Nữ (Hàng Loại 1) Không Đường Mai, Thun Lạnh, SIêu Co Dãn, Được Chọn Màu</t>
+          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://tiki.vn/quan-lot-su-duc-nu-hang-loai-1-khong-duong-mai-thun-lanh-sieu-co-dan-duoc-chon-mau-p133160820.html?spid=198901960</t>
+          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Thời trang nam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -987,22 +987,22 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>21280</v>
+        <v>185000</v>
       </c>
       <c r="G7" t="n">
-        <v>28000</v>
+        <v>144300</v>
       </c>
       <c r="H7" t="n">
-        <v>6720</v>
+        <v>-40700</v>
       </c>
       <c r="I7" t="n">
-        <v>31.58</v>
+        <v>-22</v>
       </c>
       <c r="J7" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -1011,26 +1011,26 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1040,29 +1040,29 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Giá tăng 6,720đ (+31.6%)</t>
+          <t>Giá giảm 40,700đ (22.0%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>101280655</t>
+          <t>244298352</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bộ 5 Quần Lót Nam Đùi Xuất Nhật Chất Mát từ 40kg đến 90kg (Màu Ngẫu Nghiên)</t>
+          <t>Quần Gen Ôm Bụng Dạng Đùi Có Thanh Chống Cuộn Voronin 8292 – Siêu Gọn, Siêu Định Hình</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://tiki.vn/bo-5-quan-lot-nam-dui-xuat-nhat-chat-mat-tu-40kg-den-90kg-mau-ngau-nghien-p101280655.html?spid=101280672</t>
+          <t>https://tiki.vn/quan-gen-chong-cuon-dui-8292-p244298352.html?spid=244298362</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1071,22 +1071,22 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>177000</v>
+        <v>102480</v>
       </c>
       <c r="G8" t="n">
-        <v>177000</v>
+        <v>122000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>19520</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -1095,26 +1095,26 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1124,53 +1124,53 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Review thêm +1</t>
+          <t>Giá tăng 19,520đ (+19.0%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>31638135</t>
+          <t>214706031</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combo 4 quần lót nam Boxer sợi cạp 1cm sợi tre tự nhiên mềm mịn thấm hút mồ hôi, co giãn 4 chiều MRM Manlywear - Màu ngẫu nhiên</t>
+          <t>Áo lót áo ngực Thái lan có gọng mút kép nâng ngực tạo khe, áo lót nữ thông hơi hàng CAO CẤP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-4-quan-sip-dui-nam-quan-lot-nam-boxer-soi-tre-mem-min-sieu-thoang-mat-co-gian-4-chieu-cao-cap-cap-1cm-mrm-fashion-3-mau-p31638135.html?spid=31638146</t>
+          <t>https://tiki.vn/ao-lot-ao-nguc-thai-lan-co-gong-mut-kep-nang-nguc-tao-khe-ao-lot-nu-thong-hoi-hang-cao-cap-p214706031.html?spid=215408041</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Thời trang nữ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MRM Manlywear</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>340000</v>
+        <v>98400</v>
       </c>
       <c r="G9" t="n">
-        <v>279000</v>
+        <v>120000</v>
       </c>
       <c r="H9" t="n">
-        <v>-61000</v>
+        <v>21600</v>
       </c>
       <c r="I9" t="n">
-        <v>-17.94</v>
+        <v>21.95</v>
       </c>
       <c r="J9" t="n">
-        <v>5871</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>5871</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -1179,26 +1179,26 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>1372</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>1372</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1208,24 +1208,24 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Giá giảm 61,000đ (17.9%)</t>
+          <t>Giá tăng 21,600đ (+22.0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>73163978</t>
+          <t>112851354</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hộp miếng dán ngực Silicon màu xanh 5 đôi</t>
+          <t>Áo ngực học sinh</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://tiki.vn/hop-mieng-dan-nguc-silicon-mau-xanh-5-doi-p73163978.html?spid=117659470</t>
+          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138792</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1235,26 +1235,26 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LQ luxury</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>55000</v>
+        <v>42000</v>
       </c>
       <c r="G10" t="n">
-        <v>44550</v>
+        <v>34860</v>
       </c>
       <c r="H10" t="n">
-        <v>-10450</v>
+        <v>-7140</v>
       </c>
       <c r="I10" t="n">
-        <v>-19</v>
+        <v>-17</v>
       </c>
       <c r="J10" t="n">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="K10" t="n">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1263,26 +1263,26 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O10" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1292,24 +1292,24 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Giá giảm 10,450đ (19.0%)</t>
+          <t>Giá giảm 7,140đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>73862702</t>
+          <t>113145806</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ÁO LÓT NỮ REN MÚT DÀY 2CM DÂY TRƠN NÂNG NGỰC 024B</t>
+          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-ren-mut-day-2cm-day-tron-nang-nguc-024b-p73862702.html?spid=73862720</t>
+          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1323,22 +1323,22 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>173000</v>
+        <v>124000</v>
       </c>
       <c r="G11" t="n">
-        <v>145320</v>
+        <v>102920</v>
       </c>
       <c r="H11" t="n">
-        <v>-27680</v>
+        <v>-21080</v>
       </c>
       <c r="I11" t="n">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="J11" t="n">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1347,26 +1347,26 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Giá giảm 27,680đ (16.0%)</t>
+          <t>Giá giảm 21,080đ (17.0%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>113145806</t>
+          <t>144236336</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Áo lót nâng ngực nhẹ quả trơn mẫu siêu bền</t>
+          <t>COMBO 5 ÁO LÓT VẢI KHÔNG GỌNG KHÔNG MÚT (SIZE 32-42)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nang-nguc-nhe-qua-tron-mau-sieu-ben-p113145806.html?spid=142118731</t>
+          <t>https://tiki.vn/combo-5-ao-lot-vai-khong-gong-khong-mut-size-32-42-p144236336.html?spid=146366320</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1407,22 +1407,22 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>95480</v>
+        <v>210000</v>
       </c>
       <c r="G12" t="n">
-        <v>124000</v>
+        <v>163800</v>
       </c>
       <c r="H12" t="n">
-        <v>28520</v>
+        <v>-46200</v>
       </c>
       <c r="I12" t="n">
-        <v>29.87</v>
+        <v>-22</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1431,26 +1431,26 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1460,24 +1460,24 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Giá tăng 28,520đ (+29.9%)</t>
+          <t>Giá giảm 46,200đ (22.0%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>112851354</t>
+          <t>108220832</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Áo ngực học sinh</t>
+          <t>Miếng Dán Ngực Cài Trước Hình Bàn Tay Siêu Nâng Ngực, Siêu Dính P29 Size A-B</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-nguc-hoc-sinh-p112851354.html?spid=142138792</t>
+          <t>https://tiki.vn/bra-dan-nguc-ban-tay-p29-kem-day-trong-p108220832.html?spid=242370964</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1491,22 +1491,22 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>32340</v>
+        <v>63200</v>
       </c>
       <c r="G13" t="n">
-        <v>42000</v>
+        <v>80000</v>
       </c>
       <c r="H13" t="n">
-        <v>9660</v>
+        <v>16800</v>
       </c>
       <c r="I13" t="n">
-        <v>29.87</v>
+        <v>26.58</v>
       </c>
       <c r="J13" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1515,26 +1515,26 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="O13" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1544,24 +1544,24 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Giá tăng 9,660đ (+29.9%)</t>
+          <t>Giá tăng 16,800đ (+26.6%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>74820156</t>
+          <t>244297862</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ÁO LÓT NỮ MỎNG REN 3 MÓC BIG SIZE 395</t>
+          <t>Áo Lót Nữ Bra Ống Su Gân Viền Ren Cài Sau 4003 – Seamless, Co Giãn 4 Chiều</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-mong-ren-3-moc-big-size-395-p74820156.html?spid=74820178</t>
+          <t>https://tiki.vn/ao-bra-ong-su-gan-cai-sau-4003-p244297862.html?spid=244297867</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1575,22 +1575,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>131000</v>
+        <v>38640</v>
       </c>
       <c r="G14" t="n">
-        <v>110040</v>
+        <v>46000</v>
       </c>
       <c r="H14" t="n">
-        <v>-20960</v>
+        <v>7360</v>
       </c>
       <c r="I14" t="n">
-        <v>-16</v>
+        <v>19.05</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1599,26 +1599,26 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1628,24 +1628,24 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Giá giảm 20,960đ (16.0%)</t>
+          <t>Giá tăng 7,360đ (+19.0%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>144236336</t>
+          <t>102939605</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COMBO 5 ÁO LÓT VẢI KHÔNG GỌNG KHÔNG MÚT (SIZE 32-42)</t>
+          <t>áo lót ko gọng cúp B dành cho vòng ngực khủng</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://tiki.vn/combo-5-ao-lot-vai-khong-gong-khong-mut-size-32-42-p144236336.html?spid=146366320</t>
+          <t>https://tiki.vn/ao-lot-ko-gong-cup-b-danh-cho-vong-nguc-khung-p102939605.html?spid=201243133</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1659,22 +1659,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>159600</v>
+        <v>111000</v>
       </c>
       <c r="G15" t="n">
-        <v>210000</v>
+        <v>86580</v>
       </c>
       <c r="H15" t="n">
-        <v>50400</v>
+        <v>-24420</v>
       </c>
       <c r="I15" t="n">
-        <v>31.58</v>
+        <v>-22</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="K15" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1683,26 +1683,26 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="R15" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1712,29 +1712,29 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Giá tăng 50,400đ (+31.6%)</t>
+          <t>Giá giảm 24,420đ (22.0%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>74421501</t>
+          <t>276479781</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ÁO LÓT NỮ MỎNG CÓ GỌNG CÀI TRƯỚC VIỀN REN</t>
+          <t>Mũ Nón Chống Nắng Ninja Fullface Kèm Khẩu Trang Lưới Vải Co Giãn Thoáng Khí Có Thể Gấp Gọn Đi Phượt Dã Ngoại Câu Cá Unisex</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-nu-mong-co-gong-cai-truoc-vien-ren-p74421501.html?spid=74421553</t>
+          <t>https://tiki.vn/mu-non-chong-nang-ninja-fullface-kem-khau-trang-luoi-vai-co-gian-thoang-khi-co-the-gap-gon-di-phuot-da-ngoai-cau-ca-unisex-p276479781.html?spid=276479783</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1743,22 +1743,22 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>160000</v>
+        <v>74000</v>
       </c>
       <c r="G16" t="n">
-        <v>134400</v>
+        <v>148000</v>
       </c>
       <c r="H16" t="n">
-        <v>-25600</v>
+        <v>74000</v>
       </c>
       <c r="I16" t="n">
-        <v>-16</v>
+        <v>100</v>
       </c>
       <c r="J16" t="n">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="K16" t="n">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -1767,26 +1767,26 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1796,53 +1796,53 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Giá giảm 25,600đ (16.0%)</t>
+          <t>Giá tăng 74,000đ (+100.0%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>103049077</t>
+          <t>278993558</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> (Có size lớn) Hộp 4 quần lót boxer nam William WS60 - Quần sịp đùi lưới thông hơi thoáng mát</t>
+          <t>Gọng Kính Cận Giả Cận Nam Nữ Cao Cấp Titanium BLUE LIGHT Mắt Khoan Không Viền Chữ Nhật Bạc Đen Vàng Dày Dặn Cứng Nhẹ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://tiki.vn/co-size-lon-hop-4-quan-lot-boxer-nam-william-ws60-quan-sip-dui-luoi-thong-hoi-thoang-mat-p103049077.html?spid=145612013</t>
+          <t>https://tiki.vn/gong-kinh-can-gia-can-nam-nu-cao-cap-titanium-blue-light-mat-khoan-khong-vien-chu-nhat-bac-den-vang-day-dan-cung-nhe-p278993558.html?spid=278993563</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Thời trang nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>Blue Light</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>140600</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>185000</v>
+        <v>985000</v>
       </c>
       <c r="H17" t="n">
-        <v>44400</v>
+        <v>985000</v>
       </c>
       <c r="I17" t="n">
-        <v>31.58</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -1851,82 +1851,82 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Giá tăng 44,400đ (+31.6%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>127341900</t>
+          <t>77625091</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Áo lót lovely có gọng đệm mỏng thêu hoa nổi xuất nhật</t>
+          <t>Gọng Kính cận, Kính giả cận Mắt vuông form nhỏ cao cấp - GCH2276</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-lovely-co-gong-dem-mong-theu-hoa-noi-xuat-nhat-p127341900.html?spid=142061094</t>
+          <t>https://tiki.vn/gong-kinh-can-kinh-gia-can-mat-vuong-form-nho-cao-cap-gch2276-tang-tuavit-kinh-xinh-mini-tien-loi-p77625091.html?spid=77625097</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>LiLiLa</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>117000</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>94770</v>
+        <v>189000</v>
       </c>
       <c r="H18" t="n">
-        <v>-22230</v>
+        <v>189000</v>
       </c>
       <c r="I18" t="n">
-        <v>-19</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -1935,82 +1935,82 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Giá giảm 22,230đ (19.0%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>277880869</t>
+          <t>44666139</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Áo Thun Unisex - Oversize Chất 100% Cotton 2 chiều Dày 250gsm | Nam Nữ Mặc Siêu Đẹp</t>
+          <t>Mũ lưỡi trai nam nữ vải lưới thoáng mát thời trang không logo, không thêu, che nắng tốt, bảo vệ da</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-thun-unisex-form-rong-chat-100-cotton-2-chieu-day-230gsm-mau-hot-gen-z-nam-nu-mac-sieu-dep-p277880869.html?spid=277880880</t>
+          <t>https://tiki.vn/mu-luoi-trai-nam-nu-vai-luoi-thoang-mat-thoi-trang-khong-logo-khong-theu-che-nang-tot-bao-ve-da-p44666139.html?spid=159968964</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">	SURE FASHION S</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>168000</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>109000</v>
+        <v>35000</v>
       </c>
       <c r="H19" t="n">
-        <v>-59000</v>
+        <v>35000</v>
       </c>
       <c r="I19" t="n">
-        <v>-35.12</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -2019,82 +2019,82 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>🆕 Sản phẩm mới</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Giá giảm 59,000đ (35.1%)</t>
+          <t>Xuất hiện lần đầu trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>102939605</t>
+          <t>188665546</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>áo lót ko gọng cúp B dành cho vòng ngực khủng</t>
+          <t>Lót Giày Nam Chất Liệu Cao Su Non Mềm Êm LGN2022</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://tiki.vn/ao-lot-ko-gong-cup-b-danh-cho-vong-nguc-khung-p102939605.html?spid=201243133</t>
+          <t>https://tiki.vn/lot-giay-nam-chat-lieu-cao-su-non-mem-em-lgn2022-p188665546.html?spid=188665564</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Thời trang nữ</t>
+          <t>Giày - Dép nam</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OEM</t>
+          <t>HA NAM</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>84360</v>
+        <v>22000</v>
       </c>
       <c r="G20" t="n">
-        <v>111000</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>26640</v>
+        <v>-22000</v>
       </c>
       <c r="I20" t="n">
-        <v>31.58</v>
+        <v>-100</v>
       </c>
       <c r="J20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K20" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -2103,82 +2103,82 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Giá tăng 26,640đ (+31.6%)</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>183725406</t>
+          <t>194096379</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Lót giày thể thao, giày tây giày lười cao su non cao 1.5cm TH152</t>
+          <t>Khẩu trang y tế 5 lớp N95+ KHÁNH AN KAN95+ kháng khuẩn màng lọc ngăn 95% bụi mịn nhỏ hơn 2.5 micromet và 99% tia UV, có đệm xốp không bám hơi kính</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://tiki.vn/lot-giay-the-thao-giay-tay-giay-luoi-cao-su-non-cao-1-5cm-th152-p183725406.html?spid=183725414</t>
+          <t>https://tiki.vn/khau-trang-y-te-5-lop-n95-khanh-an-kan95-khang-khuan-mang-loc-ngan-95-bui-min-nho-hon-2-5-micromet-va-99-tia-uv-co-dem-xop-khong-bam-hoi-kinh-p194096379.html?spid=276797873</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Trường Hải</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>99000</v>
+        <v>48000</v>
       </c>
       <c r="G21" t="n">
-        <v>99000</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>-48000</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J21" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="K21" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2187,53 +2187,53 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O21" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>0.2</v>
+        <v>-5</v>
       </c>
       <c r="Q21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Rating 4.5→4.7 (+0.20) | Review thêm +1</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>207936345</t>
+          <t>174305113</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Thắt lưng nữ da thật cao cấp nhãn hiệu Macsim ts008</t>
+          <t>Thùng 300/200 khẩu trang KF94 4D Bảo Long Mask kháng khuẩn chống bụi mịn sản xuất tại Việt Nam theo công nghệ 4D và chuẩn KF94 Hàn Quốc</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://tiki.vn/that-lung-nu-da-that-cao-cap-nhan-hieu-macsim-ts008-p207936345.html?spid=207936349</t>
+          <t>https://tiki.vn/thung-300-200-khau-trang-kf94-4d-bao-long-mask-khang-khuan-chong-bui-min-san-xuat-tai-viet-nam-theo-cong-nghe-4d-va-chuan-kf94-han-quoc-p174305113.html?spid=174305133</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2243,23 +2243,23 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Macsim</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>290000</v>
       </c>
       <c r="G22" t="n">
-        <v>600000</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>600000</v>
+        <v>-290000</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -2271,16 +2271,16 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -2290,60 +2290,60 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>🆕 Sản phẩm mới</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Xuất hiện lần đầu trong danh sách</t>
+          <t>Không còn xuất hiện trong danh sách</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>276750949</t>
+          <t>249587087</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DÉP NAM QUAI NGANG DA BÒ CAO CẤP VATIS</t>
+          <t>[VỎ ĐỎ MÃ MỚI] Vớ Quần tất Nhật SABRINA Natural da trần tự nhiên mặc hàng ngày chống nắng co giãn thoải mái có size lớn</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://tiki.vn/dep-nam-quai-ngang-da-bo-cao-cap-vatis-p276750949.html?spid=276750959</t>
+          <t>https://tiki.vn/vo-do-ma-moi-vo-quan-tat-nhat-sabrina-natural-da-tran-tu-nhien-mac-hang-ngay-chong-nang-co-gian-thoai-mai-co-size-lon-p249587087.html?spid=249587139</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Giày - Dép nam</t>
+          <t>Phụ kiện thời trang</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Vatis</t>
+          <t>OEM</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>149000</v>
+        <v>172000</v>
       </c>
       <c r="G23" t="n">
-        <v>149000</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>-172000</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -2355,876 +2355,36 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>-0.5</v>
+        <v>-0</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>🔄 Đã cập nhật</t>
+          <t>❌ Đã xóa</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Rating 5.0→4.5 (-0.50) | Review thêm +1</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>76369834</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Áo thun nam Novelty cổ tròn 190227 in logo</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-thun-nam-novelty-co-tron-190227-in-logo-p76369834.html?spid=76369844</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Novelty</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>299000</v>
-      </c>
-      <c r="G24" t="n">
-        <v>229000</v>
-      </c>
-      <c r="H24" t="n">
-        <v>-70000</v>
-      </c>
-      <c r="I24" t="n">
-        <v>-23.41</v>
-      </c>
-      <c r="J24" t="n">
-        <v>2</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Giá giảm 70,000đ (23.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>276811753</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Áo khoác nam áo gió vải gió cao cấp 2 lớp chống nắng tia UV và chống nước</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-khoac-nam-ao-gio-vai-gio-cao-cap-2-lop-chong-nang-tia-uv-va-chong-nuoc-p276811753.html?spid=276811773</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Uniman</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>99000</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>-99000</v>
-      </c>
-      <c r="I25" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J25" t="n">
-        <v>5</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>5</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="n">
-        <v>-5</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>1</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
           <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>76403471</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Áo thun nam Novelty cổ tim 190236</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-thun-nam-novelty-co-tim-190236-p76403471.html?spid=76403473</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Novelty</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>229000</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>-229000</v>
-      </c>
-      <c r="I26" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>90642579</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Sơ mi nữ 2 túi trước,sơ mi đũi nữ, áo form rộng SM28</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/so-mi-nu-2-tui-truoc-so-mi-dui-nu-ao-form-rong-sm28-p90642579.html?spid=90642603</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Thời trang nữ</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Haint Boutique</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>249000</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>-249000</v>
-      </c>
-      <c r="I27" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>76309819</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Áo thun nam cổ tròn NOVELTY trơn màu xanh da trời 190154N</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-thun-nam-co-tron-novelty-tron-mau-xanh-da-troi-190154n-p76309819.html?spid=76309825</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Novelty</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>299000</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>-299000</v>
-      </c>
-      <c r="I28" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>186192707</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Áo thun Novelty cổ tim Xanh lý NATMMNMCSR190238N</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/ao-thun-novelty-co-tim-xanh-ly-natmmnmcsr190238n-p186192707.html?spid=186192717</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Thời trang nam</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Novelty</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>299000</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>-299000</v>
-      </c>
-      <c r="I29" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J29" t="n">
-        <v>2</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>277351358</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Nút Nới Rộng Cổ Áo Kim Loại, Mở Rộng Cổ Áo Sơ Mi, Nút Điều Chỉnh Nút Áo Cho Nam Nữ Lò Xo Legaxi</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/nut-noi-rong-co-ao-kim-loai-mo-rong-co-ao-so-mi-nut-dieu-chinh-nut-ao-cho-nam-nu-lo-xo-legaxi-p277351358.html?spid=277351360</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Legaxi</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>8000</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>-8000</v>
-      </c>
-      <c r="I30" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>52726625</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Combo 5 Đôi Tất Nam Vớ Nam Cổ Ngắn Sợi Cotton Cùng Màu</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/combo-5-doi-tat-nam-vo-nam-co-ngan-soi-cotton-cung-mau-p52726625.html?spid=67278816</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>JM Jamano</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>175000</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>-175000</v>
-      </c>
-      <c r="I31" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J31" t="n">
-        <v>1592</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="n">
-        <v>-4.7</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>396</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>44012385</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Khăn choàng cổ nam nữ siêu nhẹ - UNQ001</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/khan-choang-co-nam-nu-sieu-nhe-unq001-p44012385.html?spid=44012389</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Phụ kiện thời trang</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>OEM</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>259000</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>-259000</v>
-      </c>
-      <c r="I32" t="n">
-        <v>-100</v>
-      </c>
-      <c r="J32" t="n">
-        <v>4</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>1</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>❌ Đã xóa</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>Không còn xuất hiện trong danh sách</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>278118538</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Keo Dán Giày Nhiệt Trong Suốt Siêu Dính Dùng Không Tổn Thương Da - Giày Da , Giày Thể Thao</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>https://tiki.vn/keo-dan-giay-nhiet-trong-suot-sieu-dinh-dung-khong-ton-thuong-da-p278118538.html?spid=278118541</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Giày - Dép nam</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>LuckyJQR</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>110000</v>
-      </c>
-      <c r="G33" t="n">
-        <v>110000</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>54</v>
-      </c>
-      <c r="K33" t="n">
-        <v>12</v>
-      </c>
-      <c r="L33" t="n">
-        <v>-42</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-4620000</v>
-      </c>
-      <c r="N33" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O33" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>5</v>
-      </c>
-      <c r="R33" t="n">
-        <v>5</v>
-      </c>
-      <c r="S33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>🔄 Đã cập nhật</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Bán thêm -42 sản phẩm</t>
         </is>
       </c>
     </row>

</xml_diff>